<commit_message>
EGAT retirement pages update 2026-04-07T01:04:38Z
</commit_message>
<xml_diff>
--- a/EGAT Retirement.xlsx
+++ b/EGAT Retirement.xlsx
@@ -683,7 +683,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I8"/>
+  <dimension ref="A1:I9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1030,6 +1030,47 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>08:04:38</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>EGAT1</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>ตราสารหนี้ (EGAT-1)</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>15.72046317947174</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0.3777940752835995</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0.08882055224737062</v>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>https://app.powerbi.com/view?r=eyJrIjoiMzZjYWU3YmQtNWQ1Ny00NjdjLWI1MmEtYjExY2ZiYWIxMzNiIiwidCI6IjVmZWJjNjlmLThlOWMtNDcwOC1iNzBlLWQ4YzYyYmUxODA1YiIsImMiOjEwfQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1041,7 +1082,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I8"/>
+  <dimension ref="A1:I9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1388,6 +1429,47 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>08:04:38</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>EGAT2</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>ตราสารทุน (EGAT-2)</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>39.54954593602872</v>
+      </c>
+      <c r="G9" t="n">
+        <v>1.149881853748846</v>
+      </c>
+      <c r="H9" t="n">
+        <v>16.52871682662138</v>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>https://app.powerbi.com/view?r=eyJrIjoiMzZjYWU3YmQtNWQ1Ny00NjdjLWI1MmEtYjExY2ZiYWIxMzNiIiwidCI6IjVmZWJjNjlmLThlOWMtNDcwOC1iNzBlLWQ4YzYyYmUxODA1YiIsImMiOjEwfQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1399,7 +1481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I8"/>
+  <dimension ref="A1:I9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1746,6 +1828,47 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>08:04:38</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>EGAT3</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>อสังหาริมทรัพย์และโครงสร้างพื้นฐาน (EGAT-3)</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>8.521260245791103</v>
+      </c>
+      <c r="G9" t="n">
+        <v>1.267968056836599</v>
+      </c>
+      <c r="H9" t="n">
+        <v>-1.506933806304867</v>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>https://app.powerbi.com/view?r=eyJrIjoiMzZjYWU3YmQtNWQ1Ny00NjdjLWI1MmEtYjExY2ZiYWIxMzNiIiwidCI6IjVmZWJjNjlmLThlOWMtNDcwOC1iNzBlLWQ4YzYyYmUxODA1YiIsImMiOjEwfQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1757,7 +1880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I8"/>
+  <dimension ref="A1:I9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -2104,6 +2227,47 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>08:04:38</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>EGAT4</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>ตราสารทุนต่างประเทศ (EGAT-4)</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>7.032974117595034</v>
+      </c>
+      <c r="G9" t="n">
+        <v>3.726579412127418</v>
+      </c>
+      <c r="H9" t="n">
+        <v>-2.522818607075272</v>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>https://app.powerbi.com/view?r=eyJrIjoiMzZjYWU3YmQtNWQ1Ny00NjdjLWI1MmEtYjExY2ZiYWIxMzNiIiwidCI6IjVmZWJjNjlmLThlOWMtNDcwOC1iNzBlLWQ4YzYyYmUxODA1YiIsImMiOjEwfQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2115,7 +2279,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I8"/>
+  <dimension ref="A1:I9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -2462,6 +2626,47 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>08:04:38</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>EGAT5</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>ตราสารทุนต่างประเทศแบบอิงดัชนี (EGAT-5)</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>15.08920231624129</v>
+      </c>
+      <c r="G9" t="n">
+        <v>3.873935053088506</v>
+      </c>
+      <c r="H9" t="n">
+        <v>-0.7534985903937974</v>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>https://app.powerbi.com/view?r=eyJrIjoiMzZjYWU3YmQtNWQ1Ny00NjdjLWI1MmEtYjExY2ZiYWIxMzNiIiwidCI6IjVmZWJjNjlmLThlOWMtNDcwOC1iNzBlLWQ4YzYyYmUxODA1YiIsImMiOjEwfQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2473,7 +2678,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I8"/>
+  <dimension ref="A1:I9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -2815,6 +3020,47 @@
         <v>15.80141524296459</v>
       </c>
       <c r="I8" t="inlineStr">
+        <is>
+          <t>https://app.powerbi.com/view?r=eyJrIjoiMzZjYWU3YmQtNWQ1Ny00NjdjLWI1MmEtYjExY2ZiYWIxMzNiIiwidCI6IjVmZWJjNjlmLThlOWMtNDcwOC1iNzBlLWQ4YzYyYmUxODA1YiIsImMiOjEwfQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>08:04:38</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>EGAT6</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>การลงทุนตามหลักศาสนาอิสลาม (EGAT-6)</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>11.41929318757163</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0.6707387202723236</v>
+      </c>
+      <c r="H9" t="n">
+        <v>15.75796772875646</v>
+      </c>
+      <c r="I9" t="inlineStr">
         <is>
           <t>https://app.powerbi.com/view?r=eyJrIjoiMzZjYWU3YmQtNWQ1Ny00NjdjLWI1MmEtYjExY2ZiYWIxMzNiIiwidCI6IjVmZWJjNjlmLThlOWMtNDcwOC1iNzBlLWQ4YzYyYmUxODA1YiIsImMiOjEwfQ%3D%3D</t>
         </is>
@@ -3084,26 +3330,66 @@
           <t>2/4/69</t>
         </is>
       </c>
-      <c r="B4" s="33" t="n"/>
-      <c r="C4" s="33" t="n"/>
-      <c r="D4" s="33" t="n"/>
-      <c r="E4" s="33" t="n"/>
-      <c r="F4" s="12" t="n"/>
-      <c r="G4" s="33" t="n"/>
-      <c r="H4" s="33" t="n"/>
-      <c r="I4" s="12" t="n"/>
-      <c r="J4" s="33" t="n"/>
-      <c r="K4" s="33" t="n"/>
-      <c r="L4" s="12" t="n"/>
-      <c r="M4" s="33" t="n"/>
-      <c r="N4" s="33" t="n"/>
-      <c r="O4" s="12" t="n"/>
-      <c r="P4" s="33" t="n"/>
-      <c r="Q4" s="33" t="n"/>
-      <c r="R4" s="12" t="n"/>
-      <c r="S4" s="33" t="n"/>
-      <c r="T4" s="33" t="n"/>
-      <c r="U4" s="12" t="n"/>
+      <c r="B4" s="35" t="n">
+        <v>4.598709017308546</v>
+      </c>
+      <c r="C4" s="35" t="n">
+        <v>0.3582391979321464</v>
+      </c>
+      <c r="D4" s="35" t="n">
+        <v>0.08882055224737062</v>
+      </c>
+      <c r="E4" s="36" t="n">
+        <v>-0.05878939264665209</v>
+      </c>
+      <c r="F4" s="19" t="n">
+        <v>15.72046317947174</v>
+      </c>
+      <c r="G4" s="35" t="n">
+        <v>16.52871682662138</v>
+      </c>
+      <c r="H4" s="36" t="n">
+        <v>-0.4670407562319383</v>
+      </c>
+      <c r="I4" s="19" t="n">
+        <v>39.54954593602872</v>
+      </c>
+      <c r="J4" s="36" t="n">
+        <v>-1.506933806304867</v>
+      </c>
+      <c r="K4" s="35" t="n">
+        <v>0.3881442431810216</v>
+      </c>
+      <c r="L4" s="19" t="n">
+        <v>8.521260245791103</v>
+      </c>
+      <c r="M4" s="36" t="n">
+        <v>-2.522818607075272</v>
+      </c>
+      <c r="N4" s="35" t="n">
+        <v>1.205717881181168</v>
+      </c>
+      <c r="O4" s="19" t="n">
+        <v>7.032974117595034</v>
+      </c>
+      <c r="P4" s="36" t="n">
+        <v>-0.7534985903937974</v>
+      </c>
+      <c r="Q4" s="35" t="n">
+        <v>1.124850726317406</v>
+      </c>
+      <c r="R4" s="19" t="n">
+        <v>15.08920231624129</v>
+      </c>
+      <c r="S4" s="35" t="n">
+        <v>15.75796772875646</v>
+      </c>
+      <c r="T4" s="36" t="n">
+        <v>-0.0434475142081272</v>
+      </c>
+      <c r="U4" s="19" t="n">
+        <v>11.41929318757163</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="10" t="inlineStr">
@@ -3908,14 +4194,14 @@
       </c>
       <c r="B1" s="4" t="inlineStr">
         <is>
-          <t>1 เม.ย. 69 (พุธ)</t>
+          <t>2 เม.ย. 69 (พฤหัส)</t>
         </is>
       </c>
       <c r="C1" s="20" t="n"/>
       <c r="D1" s="20" t="n"/>
       <c r="E1" s="21" t="inlineStr">
         <is>
-          <t>31 มี.ค. 69 (อังคาร)</t>
+          <t>1 เม.ย. 69 (พุธ)</t>
         </is>
       </c>
       <c r="F1" s="20" t="n"/>
@@ -3978,27 +4264,27 @@
       <c r="G3" s="20" t="n"/>
       <c r="H3" s="22" t="inlineStr">
         <is>
+          <t>2/4/69</t>
+        </is>
+      </c>
+      <c r="I3" s="22" t="inlineStr">
+        <is>
           <t>1/4/69</t>
         </is>
       </c>
-      <c r="I3" s="22" t="inlineStr">
+      <c r="J3" s="22" t="inlineStr">
         <is>
           <t>31/3/69</t>
         </is>
       </c>
-      <c r="J3" s="22" t="inlineStr">
+      <c r="K3" s="22" t="inlineStr">
         <is>
           <t>30/3/69</t>
         </is>
       </c>
-      <c r="K3" s="22" t="inlineStr">
+      <c r="L3" s="22" t="inlineStr">
         <is>
           <t>27/3/69</t>
-        </is>
-      </c>
-      <c r="L3" s="22" t="inlineStr">
-        <is>
-          <t>26/3/69</t>
         </is>
       </c>
     </row>
@@ -4009,37 +4295,37 @@
         </is>
       </c>
       <c r="B4" s="39" t="n">
+        <v>0.08882055224737062</v>
+      </c>
+      <c r="C4" s="37" t="n">
+        <v>-0.05878939264665209</v>
+      </c>
+      <c r="D4" s="26" t="n">
+        <v>15.72046317947174</v>
+      </c>
+      <c r="E4" s="39" t="n">
         <v>0.1476099448940227</v>
       </c>
-      <c r="C4" s="39" t="n">
+      <c r="F4" s="39" t="n">
         <v>0.4354958520295216</v>
       </c>
-      <c r="D4" s="26" t="n">
+      <c r="G4" s="26" t="n">
         <v>15.7296969428166</v>
       </c>
-      <c r="E4" s="37" t="n">
+      <c r="H4" s="39" t="n">
+        <v>0.08882055224737062</v>
+      </c>
+      <c r="I4" s="39" t="n">
+        <v>0.1476099448940227</v>
+      </c>
+      <c r="J4" s="37" t="n">
         <v>-0.2878859071354989</v>
       </c>
-      <c r="F4" s="39" t="n">
-        <v>0.1369467368146138</v>
-      </c>
-      <c r="G4" s="26" t="n">
-        <v>15.66129573208329</v>
-      </c>
-      <c r="H4" s="39" t="n">
-        <v>0.1476099448940227</v>
-      </c>
-      <c r="I4" s="37" t="n">
-        <v>-0.2878859071354989</v>
-      </c>
-      <c r="J4" s="37" t="n">
+      <c r="K4" s="37" t="n">
         <v>-0.4248326439501127</v>
       </c>
-      <c r="K4" s="37" t="n">
+      <c r="L4" s="37" t="n">
         <v>-0.448119100109845</v>
-      </c>
-      <c r="L4" s="37" t="n">
-        <v>-0.3463715599109629</v>
       </c>
     </row>
     <row r="5">
@@ -4049,37 +4335,37 @@
         </is>
       </c>
       <c r="B5" s="39" t="n">
+        <v>16.52871682662138</v>
+      </c>
+      <c r="C5" s="37" t="n">
+        <v>-0.4670407562319383</v>
+      </c>
+      <c r="D5" s="26" t="n">
+        <v>39.54954593602872</v>
+      </c>
+      <c r="E5" s="39" t="n">
         <v>16.99575758285332</v>
       </c>
-      <c r="C5" s="39" t="n">
+      <c r="F5" s="39" t="n">
         <v>1.791750725871939</v>
       </c>
-      <c r="D5" s="26" t="n">
+      <c r="G5" s="26" t="n">
         <v>39.70805836408605</v>
       </c>
-      <c r="E5" s="39" t="n">
+      <c r="H5" s="39" t="n">
+        <v>16.52871682662138</v>
+      </c>
+      <c r="I5" s="39" t="n">
+        <v>16.99575758285332</v>
+      </c>
+      <c r="J5" s="39" t="n">
         <v>15.20400685698138</v>
       </c>
-      <c r="F5" s="39" t="n">
-        <v>0.1314086401793801</v>
-      </c>
-      <c r="G5" s="26" t="n">
-        <v>39.09994278907102</v>
-      </c>
-      <c r="H5" s="39" t="n">
-        <v>16.99575758285332</v>
-      </c>
-      <c r="I5" s="39" t="n">
-        <v>15.20400685698138</v>
-      </c>
-      <c r="J5" s="39" t="n">
+      <c r="K5" s="39" t="n">
         <v>15.072598216802</v>
       </c>
-      <c r="K5" s="39" t="n">
+      <c r="L5" s="39" t="n">
         <v>14.64452490166723</v>
-      </c>
-      <c r="L5" s="39" t="n">
-        <v>14.48925474747622</v>
       </c>
     </row>
     <row r="6">
@@ -4089,37 +4375,37 @@
         </is>
       </c>
       <c r="B6" s="37" t="n">
+        <v>-1.506933806304867</v>
+      </c>
+      <c r="C6" s="39" t="n">
+        <v>0.3881442431810216</v>
+      </c>
+      <c r="D6" s="26" t="n">
+        <v>8.521260245791103</v>
+      </c>
+      <c r="E6" s="37" t="n">
         <v>-1.895078049485888</v>
       </c>
-      <c r="C6" s="39" t="n">
+      <c r="F6" s="39" t="n">
         <v>0.845079491331024</v>
       </c>
-      <c r="D6" s="26" t="n">
+      <c r="G6" s="26" t="n">
         <v>8.487679423943739</v>
       </c>
-      <c r="E6" s="37" t="n">
+      <c r="H6" s="37" t="n">
+        <v>-1.506933806304867</v>
+      </c>
+      <c r="I6" s="37" t="n">
+        <v>-1.895078049485888</v>
+      </c>
+      <c r="J6" s="37" t="n">
         <v>-2.740157540816912</v>
       </c>
-      <c r="F6" s="39" t="n">
-        <v>0.114688021455323</v>
-      </c>
-      <c r="G6" s="26" t="n">
-        <v>8.414566233824845</v>
-      </c>
-      <c r="H6" s="37" t="n">
-        <v>-1.895078049485888</v>
-      </c>
-      <c r="I6" s="37" t="n">
-        <v>-2.740157540816912</v>
-      </c>
-      <c r="J6" s="37" t="n">
+      <c r="K6" s="37" t="n">
         <v>-2.854845562272235</v>
       </c>
-      <c r="K6" s="37" t="n">
+      <c r="L6" s="37" t="n">
         <v>-2.343942461344861</v>
-      </c>
-      <c r="L6" s="37" t="n">
-        <v>-2.894183814516349</v>
       </c>
     </row>
     <row r="7">
@@ -4129,37 +4415,37 @@
         </is>
       </c>
       <c r="B7" s="37" t="n">
+        <v>-2.522818607075272</v>
+      </c>
+      <c r="C7" s="39" t="n">
+        <v>1.205717881181168</v>
+      </c>
+      <c r="D7" s="26" t="n">
+        <v>7.032974117595034</v>
+      </c>
+      <c r="E7" s="37" t="n">
         <v>-3.72853648825644</v>
       </c>
-      <c r="C7" s="39" t="n">
+      <c r="F7" s="39" t="n">
         <v>2.296339734039988</v>
       </c>
-      <c r="D7" s="26" t="n">
+      <c r="G7" s="26" t="n">
         <v>6.94598162837556</v>
       </c>
-      <c r="E7" s="37" t="n">
+      <c r="H7" s="37" t="n">
+        <v>-2.522818607075272</v>
+      </c>
+      <c r="I7" s="37" t="n">
+        <v>-3.72853648825644</v>
+      </c>
+      <c r="J7" s="37" t="n">
         <v>-6.024876222296427</v>
       </c>
-      <c r="F7" s="37" t="n">
-        <v>-0.7234614159503003</v>
-      </c>
-      <c r="G7" s="26" t="n">
-        <v>6.7803008230432</v>
-      </c>
-      <c r="H7" s="37" t="n">
-        <v>-3.72853648825644</v>
-      </c>
-      <c r="I7" s="37" t="n">
-        <v>-6.024876222296427</v>
-      </c>
-      <c r="J7" s="37" t="n">
+      <c r="K7" s="37" t="n">
         <v>-5.301414806346127</v>
       </c>
-      <c r="K7" s="37" t="n">
+      <c r="L7" s="37" t="n">
         <v>-4.09373133511417</v>
-      </c>
-      <c r="L7" s="37" t="n">
-        <v>-1.706959647633877</v>
       </c>
     </row>
     <row r="8">
@@ -4169,37 +4455,37 @@
         </is>
       </c>
       <c r="B8" s="37" t="n">
+        <v>-0.7534985903937974</v>
+      </c>
+      <c r="C8" s="39" t="n">
+        <v>1.124850726317406</v>
+      </c>
+      <c r="D8" s="26" t="n">
+        <v>15.08920231624129</v>
+      </c>
+      <c r="E8" s="37" t="n">
         <v>-1.878349316711203</v>
       </c>
-      <c r="C8" s="39" t="n">
+      <c r="F8" s="39" t="n">
         <v>2.576506120427369</v>
       </c>
-      <c r="D8" s="26" t="n">
+      <c r="G8" s="26" t="n">
         <v>14.91818268387235</v>
       </c>
-      <c r="E8" s="37" t="n">
+      <c r="H8" s="37" t="n">
+        <v>-0.7534985903937974</v>
+      </c>
+      <c r="I8" s="37" t="n">
+        <v>-1.878349316711203</v>
+      </c>
+      <c r="J8" s="37" t="n">
         <v>-4.454855437138572</v>
       </c>
-      <c r="F8" s="37" t="n">
-        <v>-0.2470931144950557</v>
-      </c>
-      <c r="G8" s="26" t="n">
-        <v>14.52645681376123</v>
-      </c>
-      <c r="H8" s="37" t="n">
-        <v>-1.878349316711203</v>
-      </c>
-      <c r="I8" s="37" t="n">
-        <v>-4.454855437138572</v>
-      </c>
-      <c r="J8" s="37" t="n">
+      <c r="K8" s="37" t="n">
         <v>-4.207762322643516</v>
       </c>
-      <c r="K8" s="37" t="n">
+      <c r="L8" s="37" t="n">
         <v>-2.800671018760326</v>
-      </c>
-      <c r="L8" s="37" t="n">
-        <v>-0.7454883778248322</v>
       </c>
     </row>
     <row r="9">
@@ -4209,37 +4495,37 @@
         </is>
       </c>
       <c r="B9" s="39" t="n">
+        <v>15.75796772875646</v>
+      </c>
+      <c r="C9" s="37" t="n">
+        <v>-0.0434475142081272</v>
+      </c>
+      <c r="D9" s="26" t="n">
+        <v>11.41929318757163</v>
+      </c>
+      <c r="E9" s="39" t="n">
         <v>15.80141524296459</v>
       </c>
-      <c r="C9" s="39" t="n">
+      <c r="F9" s="39" t="n">
         <v>0.8147078836333801</v>
       </c>
-      <c r="D9" s="26" t="n">
+      <c r="G9" s="26" t="n">
         <v>11.42357919839877</v>
       </c>
-      <c r="E9" s="39" t="n">
+      <c r="H9" s="39" t="n">
+        <v>15.75796772875646</v>
+      </c>
+      <c r="I9" s="39" t="n">
+        <v>15.80141524296459</v>
+      </c>
+      <c r="J9" s="39" t="n">
         <v>14.98670735933121</v>
       </c>
-      <c r="F9" s="37" t="n">
-        <v>-0.7990668775968714</v>
-      </c>
-      <c r="G9" s="26" t="n">
-        <v>11.34320988673951</v>
-      </c>
-      <c r="H9" s="39" t="n">
-        <v>15.80141524296459</v>
-      </c>
-      <c r="I9" s="39" t="n">
-        <v>14.98670735933121</v>
-      </c>
-      <c r="J9" s="39" t="n">
+      <c r="K9" s="39" t="n">
         <v>15.78577423692808</v>
       </c>
-      <c r="K9" s="39" t="n">
+      <c r="L9" s="39" t="n">
         <v>15.56294612307485</v>
-      </c>
-      <c r="L9" s="39" t="n">
-        <v>15.51468161781753</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
EGAT retirement pages update 2026-04-07T04:15:08Z
</commit_message>
<xml_diff>
--- a/EGAT Retirement.xlsx
+++ b/EGAT Retirement.xlsx
@@ -3358,7 +3358,7 @@
         <v>-1.506933806304867</v>
       </c>
       <c r="K4" s="35" t="n">
-        <v>0.3881442431810216</v>
+        <v>0.3881442431810211</v>
       </c>
       <c r="L4" s="19" t="n">
         <v>8.521260245791103</v>
@@ -3385,7 +3385,7 @@
         <v>15.75796772875646</v>
       </c>
       <c r="T4" s="36" t="n">
-        <v>-0.0434475142081272</v>
+        <v>-0.04344751420812898</v>
       </c>
       <c r="U4" s="19" t="n">
         <v>11.41929318757163</v>
@@ -4378,7 +4378,7 @@
         <v>-1.506933806304867</v>
       </c>
       <c r="C6" s="39" t="n">
-        <v>0.3881442431810216</v>
+        <v>0.3881442431810211</v>
       </c>
       <c r="D6" s="26" t="n">
         <v>8.521260245791103</v>
@@ -4498,7 +4498,7 @@
         <v>15.75796772875646</v>
       </c>
       <c r="C9" s="37" t="n">
-        <v>-0.0434475142081272</v>
+        <v>-0.04344751420812898</v>
       </c>
       <c r="D9" s="26" t="n">
         <v>11.41929318757163</v>

</xml_diff>

<commit_message>
EGAT retirement pages update 2026-04-08T04:15:06Z
</commit_message>
<xml_diff>
--- a/EGAT Retirement.xlsx
+++ b/EGAT Retirement.xlsx
@@ -683,7 +683,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I9"/>
+  <dimension ref="A1:I10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1071,6 +1071,47 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-04-03</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>11:15:06</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>2026-04-03</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>EGAT1</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>ตราสารหนี้ (EGAT-1)</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>15.72616280437217</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0.414187136227806</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0.1251088426979186</v>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>https://app.powerbi.com/view?r=eyJrIjoiMzZjYWU3YmQtNWQ1Ny00NjdjLWI1MmEtYjExY2ZiYWIxMzNiIiwidCI6IjVmZWJjNjlmLThlOWMtNDcwOC1iNzBlLWQ4YzYyYmUxODA1YiIsImMiOjEwfQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1082,7 +1123,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I9"/>
+  <dimension ref="A1:I10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1470,6 +1511,47 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-04-03</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>11:15:06</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>2026-04-03</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>EGAT2</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>ตราสารทุน (EGAT-2)</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>39.2365270656978</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0.3493209117046536</v>
+      </c>
+      <c r="H10" t="n">
+        <v>15.6064385440545</v>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>https://app.powerbi.com/view?r=eyJrIjoiMzZjYWU3YmQtNWQ1Ny00NjdjLWI1MmEtYjExY2ZiYWIxMzNiIiwidCI6IjVmZWJjNjlmLThlOWMtNDcwOC1iNzBlLWQ4YzYyYmUxODA1YiIsImMiOjEwfQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1481,7 +1563,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I9"/>
+  <dimension ref="A1:I10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1869,6 +1951,47 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-04-03</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>11:15:06</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>2026-04-03</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>EGAT3</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>อสังหาริมทรัพย์และโครงสร้างพื้นฐาน (EGAT-3)</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>8.504081918942456</v>
+      </c>
+      <c r="G10" t="n">
+        <v>1.063818177076992</v>
+      </c>
+      <c r="H10" t="n">
+        <v>-1.705489657739689</v>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>https://app.powerbi.com/view?r=eyJrIjoiMzZjYWU3YmQtNWQ1Ny00NjdjLWI1MmEtYjExY2ZiYWIxMzNiIiwidCI6IjVmZWJjNjlmLThlOWMtNDcwOC1iNzBlLWQ4YzYyYmUxODA1YiIsImMiOjEwfQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1880,7 +2003,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I9"/>
+  <dimension ref="A1:I10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -2268,6 +2391,47 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-04-03</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>11:15:06</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>2026-04-03</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>EGAT4</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>ตราสารทุนต่างประเทศ (EGAT-4)</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>7.013124523672051</v>
+      </c>
+      <c r="G10" t="n">
+        <v>3.433825529356871</v>
+      </c>
+      <c r="H10" t="n">
+        <v>-2.79793443077293</v>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>https://app.powerbi.com/view?r=eyJrIjoiMzZjYWU3YmQtNWQ1Ny00NjdjLWI1MmEtYjExY2ZiYWIxMzNiIiwidCI6IjVmZWJjNjlmLThlOWMtNDcwOC1iNzBlLWQ4YzYyYmUxODA1YiIsImMiOjEwfQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2279,7 +2443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I9"/>
+  <dimension ref="A1:I10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -2667,6 +2831,47 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-04-03</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>11:15:06</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>2026-04-03</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>EGAT5</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>ตราสารทุนต่างประเทศแบบอิงดัชนี (EGAT-5)</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>15.07699297370509</v>
+      </c>
+      <c r="G10" t="n">
+        <v>3.789886047245372</v>
+      </c>
+      <c r="H10" t="n">
+        <v>-0.8338033345302587</v>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>https://app.powerbi.com/view?r=eyJrIjoiMzZjYWU3YmQtNWQ1Ny00NjdjLWI1MmEtYjExY2ZiYWIxMzNiIiwidCI6IjVmZWJjNjlmLThlOWMtNDcwOC1iNzBlLWQ4YzYyYmUxODA1YiIsImMiOjEwfQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2678,7 +2883,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I9"/>
+  <dimension ref="A1:I10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -3061,6 +3266,47 @@
         <v>15.75796772875646</v>
       </c>
       <c r="I9" t="inlineStr">
+        <is>
+          <t>https://app.powerbi.com/view?r=eyJrIjoiMzZjYWU3YmQtNWQ1Ny00NjdjLWI1MmEtYjExY2ZiYWIxMzNiIiwidCI6IjVmZWJjNjlmLThlOWMtNDcwOC1iNzBlLWQ4YzYyYmUxODA1YiIsImMiOjEwfQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-04-03</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>11:15:06</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>2026-04-03</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>EGAT6</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>การลงทุนตามหลักศาสนาอิสลาม (EGAT-6)</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>11.3176174526855</v>
+      </c>
+      <c r="G10" t="n">
+        <v>-0.2256189765467265</v>
+      </c>
+      <c r="H10" t="n">
+        <v>14.72727552702231</v>
+      </c>
+      <c r="I10" t="inlineStr">
         <is>
           <t>https://app.powerbi.com/view?r=eyJrIjoiMzZjYWU3YmQtNWQ1Ny00NjdjLWI1MmEtYjExY2ZiYWIxMzNiIiwidCI6IjVmZWJjNjlmLThlOWMtNDcwOC1iNzBlLWQ4YzYyYmUxODA1YiIsImMiOjEwfQ%3D%3D</t>
         </is>
@@ -3397,26 +3643,66 @@
           <t>3/4/69</t>
         </is>
       </c>
-      <c r="B5" s="33" t="n"/>
-      <c r="C5" s="33" t="n"/>
-      <c r="D5" s="33" t="n"/>
-      <c r="E5" s="33" t="n"/>
-      <c r="F5" s="12" t="n"/>
-      <c r="G5" s="33" t="n"/>
-      <c r="H5" s="33" t="n"/>
-      <c r="I5" s="12" t="n"/>
-      <c r="J5" s="33" t="n"/>
-      <c r="K5" s="33" t="n"/>
-      <c r="L5" s="12" t="n"/>
-      <c r="M5" s="33" t="n"/>
-      <c r="N5" s="33" t="n"/>
-      <c r="O5" s="12" t="n"/>
-      <c r="P5" s="33" t="n"/>
-      <c r="Q5" s="33" t="n"/>
-      <c r="R5" s="12" t="n"/>
-      <c r="S5" s="33" t="n"/>
-      <c r="T5" s="33" t="n"/>
-      <c r="U5" s="12" t="n"/>
+      <c r="B5" s="35" t="n">
+        <v>4.186932581788642</v>
+      </c>
+      <c r="C5" s="36" t="n">
+        <v>-0.4117764355199043</v>
+      </c>
+      <c r="D5" s="35" t="n">
+        <v>0.1251088426979186</v>
+      </c>
+      <c r="E5" s="35" t="n">
+        <v>0.03628829045054793</v>
+      </c>
+      <c r="F5" s="19" t="n">
+        <v>15.72616280437217</v>
+      </c>
+      <c r="G5" s="35" t="n">
+        <v>15.6064385440545</v>
+      </c>
+      <c r="H5" s="36" t="n">
+        <v>-0.9222782825668787</v>
+      </c>
+      <c r="I5" s="19" t="n">
+        <v>39.2365270656978</v>
+      </c>
+      <c r="J5" s="36" t="n">
+        <v>-1.705489657739689</v>
+      </c>
+      <c r="K5" s="36" t="n">
+        <v>-0.1985558514348225</v>
+      </c>
+      <c r="L5" s="19" t="n">
+        <v>8.504081918942456</v>
+      </c>
+      <c r="M5" s="36" t="n">
+        <v>-2.79793443077293</v>
+      </c>
+      <c r="N5" s="36" t="n">
+        <v>-0.2751158236976585</v>
+      </c>
+      <c r="O5" s="19" t="n">
+        <v>7.013124523672051</v>
+      </c>
+      <c r="P5" s="36" t="n">
+        <v>-0.8338033345302587</v>
+      </c>
+      <c r="Q5" s="36" t="n">
+        <v>-0.08030474413646127</v>
+      </c>
+      <c r="R5" s="19" t="n">
+        <v>15.07699297370509</v>
+      </c>
+      <c r="S5" s="35" t="n">
+        <v>14.72727552702231</v>
+      </c>
+      <c r="T5" s="36" t="n">
+        <v>-1.03069220173415</v>
+      </c>
+      <c r="U5" s="19" t="n">
+        <v>11.3176174526855</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="13" t="inlineStr">
@@ -4194,14 +4480,14 @@
       </c>
       <c r="B1" s="4" t="inlineStr">
         <is>
-          <t>2 เม.ย. 69 (พฤหัส)</t>
+          <t>3 เม.ย. 69 (ศุกร์)</t>
         </is>
       </c>
       <c r="C1" s="20" t="n"/>
       <c r="D1" s="20" t="n"/>
       <c r="E1" s="21" t="inlineStr">
         <is>
-          <t>1 เม.ย. 69 (พุธ)</t>
+          <t>2 เม.ย. 69 (พฤหัส)</t>
         </is>
       </c>
       <c r="F1" s="20" t="n"/>
@@ -4264,27 +4550,27 @@
       <c r="G3" s="20" t="n"/>
       <c r="H3" s="22" t="inlineStr">
         <is>
+          <t>3/4/69</t>
+        </is>
+      </c>
+      <c r="I3" s="22" t="inlineStr">
+        <is>
           <t>2/4/69</t>
         </is>
       </c>
-      <c r="I3" s="22" t="inlineStr">
+      <c r="J3" s="22" t="inlineStr">
         <is>
           <t>1/4/69</t>
         </is>
       </c>
-      <c r="J3" s="22" t="inlineStr">
+      <c r="K3" s="22" t="inlineStr">
         <is>
           <t>31/3/69</t>
         </is>
       </c>
-      <c r="K3" s="22" t="inlineStr">
+      <c r="L3" s="22" t="inlineStr">
         <is>
           <t>30/3/69</t>
-        </is>
-      </c>
-      <c r="L3" s="22" t="inlineStr">
-        <is>
-          <t>27/3/69</t>
         </is>
       </c>
     </row>
@@ -4295,37 +4581,37 @@
         </is>
       </c>
       <c r="B4" s="39" t="n">
+        <v>0.1251088426979186</v>
+      </c>
+      <c r="C4" s="39" t="n">
+        <v>0.03628829045054793</v>
+      </c>
+      <c r="D4" s="26" t="n">
+        <v>15.72616280437217</v>
+      </c>
+      <c r="E4" s="39" t="n">
         <v>0.08882055224737062</v>
       </c>
-      <c r="C4" s="37" t="n">
+      <c r="F4" s="37" t="n">
         <v>-0.05878939264665209</v>
       </c>
-      <c r="D4" s="26" t="n">
+      <c r="G4" s="26" t="n">
         <v>15.72046317947174</v>
       </c>
-      <c r="E4" s="39" t="n">
+      <c r="H4" s="39" t="n">
+        <v>0.1251088426979186</v>
+      </c>
+      <c r="I4" s="39" t="n">
+        <v>0.08882055224737062</v>
+      </c>
+      <c r="J4" s="39" t="n">
         <v>0.1476099448940227</v>
       </c>
-      <c r="F4" s="39" t="n">
-        <v>0.4354958520295216</v>
-      </c>
-      <c r="G4" s="26" t="n">
-        <v>15.7296969428166</v>
-      </c>
-      <c r="H4" s="39" t="n">
-        <v>0.08882055224737062</v>
-      </c>
-      <c r="I4" s="39" t="n">
-        <v>0.1476099448940227</v>
-      </c>
-      <c r="J4" s="37" t="n">
+      <c r="K4" s="37" t="n">
         <v>-0.2878859071354989</v>
       </c>
-      <c r="K4" s="37" t="n">
+      <c r="L4" s="37" t="n">
         <v>-0.4248326439501127</v>
-      </c>
-      <c r="L4" s="37" t="n">
-        <v>-0.448119100109845</v>
       </c>
     </row>
     <row r="5">
@@ -4335,37 +4621,37 @@
         </is>
       </c>
       <c r="B5" s="39" t="n">
+        <v>15.6064385440545</v>
+      </c>
+      <c r="C5" s="37" t="n">
+        <v>-0.9222782825668787</v>
+      </c>
+      <c r="D5" s="26" t="n">
+        <v>39.2365270656978</v>
+      </c>
+      <c r="E5" s="39" t="n">
         <v>16.52871682662138</v>
       </c>
-      <c r="C5" s="37" t="n">
+      <c r="F5" s="37" t="n">
         <v>-0.4670407562319383</v>
       </c>
-      <c r="D5" s="26" t="n">
+      <c r="G5" s="26" t="n">
         <v>39.54954593602872</v>
       </c>
-      <c r="E5" s="39" t="n">
+      <c r="H5" s="39" t="n">
+        <v>15.6064385440545</v>
+      </c>
+      <c r="I5" s="39" t="n">
+        <v>16.52871682662138</v>
+      </c>
+      <c r="J5" s="39" t="n">
         <v>16.99575758285332</v>
       </c>
-      <c r="F5" s="39" t="n">
-        <v>1.791750725871939</v>
-      </c>
-      <c r="G5" s="26" t="n">
-        <v>39.70805836408605</v>
-      </c>
-      <c r="H5" s="39" t="n">
-        <v>16.52871682662138</v>
-      </c>
-      <c r="I5" s="39" t="n">
-        <v>16.99575758285332</v>
-      </c>
-      <c r="J5" s="39" t="n">
+      <c r="K5" s="39" t="n">
         <v>15.20400685698138</v>
       </c>
-      <c r="K5" s="39" t="n">
+      <c r="L5" s="39" t="n">
         <v>15.072598216802</v>
-      </c>
-      <c r="L5" s="39" t="n">
-        <v>14.64452490166723</v>
       </c>
     </row>
     <row r="6">
@@ -4375,37 +4661,37 @@
         </is>
       </c>
       <c r="B6" s="37" t="n">
+        <v>-1.705489657739689</v>
+      </c>
+      <c r="C6" s="37" t="n">
+        <v>-0.1985558514348225</v>
+      </c>
+      <c r="D6" s="26" t="n">
+        <v>8.504081918942456</v>
+      </c>
+      <c r="E6" s="37" t="n">
         <v>-1.506933806304867</v>
       </c>
-      <c r="C6" s="39" t="n">
+      <c r="F6" s="39" t="n">
         <v>0.3881442431810211</v>
       </c>
-      <c r="D6" s="26" t="n">
+      <c r="G6" s="26" t="n">
         <v>8.521260245791103</v>
       </c>
-      <c r="E6" s="37" t="n">
+      <c r="H6" s="37" t="n">
+        <v>-1.705489657739689</v>
+      </c>
+      <c r="I6" s="37" t="n">
+        <v>-1.506933806304867</v>
+      </c>
+      <c r="J6" s="37" t="n">
         <v>-1.895078049485888</v>
       </c>
-      <c r="F6" s="39" t="n">
-        <v>0.845079491331024</v>
-      </c>
-      <c r="G6" s="26" t="n">
-        <v>8.487679423943739</v>
-      </c>
-      <c r="H6" s="37" t="n">
-        <v>-1.506933806304867</v>
-      </c>
-      <c r="I6" s="37" t="n">
-        <v>-1.895078049485888</v>
-      </c>
-      <c r="J6" s="37" t="n">
+      <c r="K6" s="37" t="n">
         <v>-2.740157540816912</v>
       </c>
-      <c r="K6" s="37" t="n">
+      <c r="L6" s="37" t="n">
         <v>-2.854845562272235</v>
-      </c>
-      <c r="L6" s="37" t="n">
-        <v>-2.343942461344861</v>
       </c>
     </row>
     <row r="7">
@@ -4415,37 +4701,37 @@
         </is>
       </c>
       <c r="B7" s="37" t="n">
+        <v>-2.79793443077293</v>
+      </c>
+      <c r="C7" s="37" t="n">
+        <v>-0.2751158236976585</v>
+      </c>
+      <c r="D7" s="26" t="n">
+        <v>7.013124523672051</v>
+      </c>
+      <c r="E7" s="37" t="n">
         <v>-2.522818607075272</v>
       </c>
-      <c r="C7" s="39" t="n">
+      <c r="F7" s="39" t="n">
         <v>1.205717881181168</v>
       </c>
-      <c r="D7" s="26" t="n">
+      <c r="G7" s="26" t="n">
         <v>7.032974117595034</v>
       </c>
-      <c r="E7" s="37" t="n">
+      <c r="H7" s="37" t="n">
+        <v>-2.79793443077293</v>
+      </c>
+      <c r="I7" s="37" t="n">
+        <v>-2.522818607075272</v>
+      </c>
+      <c r="J7" s="37" t="n">
         <v>-3.72853648825644</v>
       </c>
-      <c r="F7" s="39" t="n">
-        <v>2.296339734039988</v>
-      </c>
-      <c r="G7" s="26" t="n">
-        <v>6.94598162837556</v>
-      </c>
-      <c r="H7" s="37" t="n">
-        <v>-2.522818607075272</v>
-      </c>
-      <c r="I7" s="37" t="n">
-        <v>-3.72853648825644</v>
-      </c>
-      <c r="J7" s="37" t="n">
+      <c r="K7" s="37" t="n">
         <v>-6.024876222296427</v>
       </c>
-      <c r="K7" s="37" t="n">
+      <c r="L7" s="37" t="n">
         <v>-5.301414806346127</v>
-      </c>
-      <c r="L7" s="37" t="n">
-        <v>-4.09373133511417</v>
       </c>
     </row>
     <row r="8">
@@ -4455,37 +4741,37 @@
         </is>
       </c>
       <c r="B8" s="37" t="n">
+        <v>-0.8338033345302587</v>
+      </c>
+      <c r="C8" s="37" t="n">
+        <v>-0.08030474413646127</v>
+      </c>
+      <c r="D8" s="26" t="n">
+        <v>15.07699297370509</v>
+      </c>
+      <c r="E8" s="37" t="n">
         <v>-0.7534985903937974</v>
       </c>
-      <c r="C8" s="39" t="n">
+      <c r="F8" s="39" t="n">
         <v>1.124850726317406</v>
       </c>
-      <c r="D8" s="26" t="n">
+      <c r="G8" s="26" t="n">
         <v>15.08920231624129</v>
       </c>
-      <c r="E8" s="37" t="n">
+      <c r="H8" s="37" t="n">
+        <v>-0.8338033345302587</v>
+      </c>
+      <c r="I8" s="37" t="n">
+        <v>-0.7534985903937974</v>
+      </c>
+      <c r="J8" s="37" t="n">
         <v>-1.878349316711203</v>
       </c>
-      <c r="F8" s="39" t="n">
-        <v>2.576506120427369</v>
-      </c>
-      <c r="G8" s="26" t="n">
-        <v>14.91818268387235</v>
-      </c>
-      <c r="H8" s="37" t="n">
-        <v>-0.7534985903937974</v>
-      </c>
-      <c r="I8" s="37" t="n">
-        <v>-1.878349316711203</v>
-      </c>
-      <c r="J8" s="37" t="n">
+      <c r="K8" s="37" t="n">
         <v>-4.454855437138572</v>
       </c>
-      <c r="K8" s="37" t="n">
+      <c r="L8" s="37" t="n">
         <v>-4.207762322643516</v>
-      </c>
-      <c r="L8" s="37" t="n">
-        <v>-2.800671018760326</v>
       </c>
     </row>
     <row r="9">
@@ -4495,37 +4781,37 @@
         </is>
       </c>
       <c r="B9" s="39" t="n">
+        <v>14.72727552702231</v>
+      </c>
+      <c r="C9" s="37" t="n">
+        <v>-1.03069220173415</v>
+      </c>
+      <c r="D9" s="26" t="n">
+        <v>11.3176174526855</v>
+      </c>
+      <c r="E9" s="39" t="n">
         <v>15.75796772875646</v>
       </c>
-      <c r="C9" s="37" t="n">
+      <c r="F9" s="37" t="n">
         <v>-0.04344751420812898</v>
       </c>
-      <c r="D9" s="26" t="n">
+      <c r="G9" s="26" t="n">
         <v>11.41929318757163</v>
       </c>
-      <c r="E9" s="39" t="n">
+      <c r="H9" s="39" t="n">
+        <v>14.72727552702231</v>
+      </c>
+      <c r="I9" s="39" t="n">
+        <v>15.75796772875646</v>
+      </c>
+      <c r="J9" s="39" t="n">
         <v>15.80141524296459</v>
       </c>
-      <c r="F9" s="39" t="n">
-        <v>0.8147078836333801</v>
-      </c>
-      <c r="G9" s="26" t="n">
-        <v>11.42357919839877</v>
-      </c>
-      <c r="H9" s="39" t="n">
-        <v>15.75796772875646</v>
-      </c>
-      <c r="I9" s="39" t="n">
-        <v>15.80141524296459</v>
-      </c>
-      <c r="J9" s="39" t="n">
+      <c r="K9" s="39" t="n">
         <v>14.98670735933121</v>
       </c>
-      <c r="K9" s="39" t="n">
+      <c r="L9" s="39" t="n">
         <v>15.78577423692808</v>
-      </c>
-      <c r="L9" s="39" t="n">
-        <v>15.56294612307485</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
EGAT retirement pages update 2026-04-09T04:15:10Z
</commit_message>
<xml_diff>
--- a/EGAT Retirement.xlsx
+++ b/EGAT Retirement.xlsx
@@ -683,7 +683,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I10"/>
+  <dimension ref="A1:I11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1112,6 +1112,47 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>11:15:09</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>EGAT1</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>ตราสารหนี้ (EGAT-1)</t>
+        </is>
+      </c>
+      <c r="F11" t="n">
+        <v>15.73147231918833</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0.4480892788536917</v>
+      </c>
+      <c r="H11" t="n">
+        <v>0.1589133858329816</v>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>https://app.powerbi.com/view?r=eyJrIjoiMzZjYWU3YmQtNWQ1Ny00NjdjLWI1MmEtYjExY2ZiYWIxMzNiIiwidCI6IjVmZWJjNjlmLThlOWMtNDcwOC1iNzBlLWQ4YzYyYmUxODA1YiIsImMiOjEwfQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1123,7 +1164,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I10"/>
+  <dimension ref="A1:I11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1552,6 +1593,47 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>11:15:09</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>EGAT2</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>ตราสารทุน (EGAT-2)</t>
+        </is>
+      </c>
+      <c r="F11" t="n">
+        <v>39.47520867717733</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0.9597607089369076</v>
+      </c>
+      <c r="H11" t="n">
+        <v>16.30968964991566</v>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>https://app.powerbi.com/view?r=eyJrIjoiMzZjYWU3YmQtNWQ1Ny00NjdjLWI1MmEtYjExY2ZiYWIxMzNiIiwidCI6IjVmZWJjNjlmLThlOWMtNDcwOC1iNzBlLWQ4YzYyYmUxODA1YiIsImMiOjEwfQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1563,7 +1645,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I10"/>
+  <dimension ref="A1:I11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1992,6 +2074,47 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>11:15:09</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>EGAT3</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>อสังหาริมทรัพย์และโครงสร้างพื้นฐาน (EGAT-3)</t>
+        </is>
+      </c>
+      <c r="F11" t="n">
+        <v>8.510515755764585</v>
+      </c>
+      <c r="G11" t="n">
+        <v>1.140278883943457</v>
+      </c>
+      <c r="H11" t="n">
+        <v>-1.631124094698189</v>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>https://app.powerbi.com/view?r=eyJrIjoiMzZjYWU3YmQtNWQ1Ny00NjdjLWI1MmEtYjExY2ZiYWIxMzNiIiwidCI6IjVmZWJjNjlmLThlOWMtNDcwOC1iNzBlLWQ4YzYyYmUxODA1YiIsImMiOjEwfQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2003,7 +2126,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I10"/>
+  <dimension ref="A1:I11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -2432,6 +2555,47 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>11:15:09</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>EGAT4</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>ตราสารทุนต่างประเทศ (EGAT-4)</t>
+        </is>
+      </c>
+      <c r="F11" t="n">
+        <v>7.026671469699702</v>
+      </c>
+      <c r="G11" t="n">
+        <v>3.633624127991464</v>
+      </c>
+      <c r="H11" t="n">
+        <v>-2.610173450399955</v>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>https://app.powerbi.com/view?r=eyJrIjoiMzZjYWU3YmQtNWQ1Ny00NjdjLWI1MmEtYjExY2ZiYWIxMzNiIiwidCI6IjVmZWJjNjlmLThlOWMtNDcwOC1iNzBlLWQ4YzYyYmUxODA1YiIsImMiOjEwfQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2443,7 +2607,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I10"/>
+  <dimension ref="A1:I11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -2872,6 +3036,47 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>11:15:09</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>EGAT5</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>ตราสารทุนต่างประเทศแบบอิงดัชนี (EGAT-5)</t>
+        </is>
+      </c>
+      <c r="F11" t="n">
+        <v>15.08672754982331</v>
+      </c>
+      <c r="G11" t="n">
+        <v>3.856898782993823</v>
+      </c>
+      <c r="H11" t="n">
+        <v>-0.7697759192838771</v>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>https://app.powerbi.com/view?r=eyJrIjoiMzZjYWU3YmQtNWQ1Ny00NjdjLWI1MmEtYjExY2ZiYWIxMzNiIiwidCI6IjVmZWJjNjlmLThlOWMtNDcwOC1iNzBlLWQ4YzYyYmUxODA1YiIsImMiOjEwfQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2883,7 +3088,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I10"/>
+  <dimension ref="A1:I11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -3307,6 +3512,47 @@
         <v>14.72727552702231</v>
       </c>
       <c r="I10" t="inlineStr">
+        <is>
+          <t>https://app.powerbi.com/view?r=eyJrIjoiMzZjYWU3YmQtNWQ1Ny00NjdjLWI1MmEtYjExY2ZiYWIxMzNiIiwidCI6IjVmZWJjNjlmLThlOWMtNDcwOC1iNzBlLWQ4YzYyYmUxODA1YiIsImMiOjEwfQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>11:15:09</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>EGAT6</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>การลงทุนตามหลักศาสนาอิสลาม (EGAT-6)</t>
+        </is>
+      </c>
+      <c r="F11" t="n">
+        <v>11.42568187506592</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0.7270604101474509</v>
+      </c>
+      <c r="H11" t="n">
+        <v>15.822730185473</v>
+      </c>
+      <c r="I11" t="inlineStr">
         <is>
           <t>https://app.powerbi.com/view?r=eyJrIjoiMzZjYWU3YmQtNWQ1Ny00NjdjLWI1MmEtYjExY2ZiYWIxMzNiIiwidCI6IjVmZWJjNjlmLThlOWMtNDcwOC1iNzBlLWQ4YzYyYmUxODA1YiIsImMiOjEwfQ%3D%3D</t>
         </is>
@@ -3653,7 +3899,7 @@
         <v>0.1251088426979186</v>
       </c>
       <c r="E5" s="35" t="n">
-        <v>0.03628829045054793</v>
+        <v>0.03628829045054799</v>
       </c>
       <c r="F5" s="19" t="n">
         <v>15.72616280437217</v>
@@ -3662,7 +3908,7 @@
         <v>15.6064385440545</v>
       </c>
       <c r="H5" s="36" t="n">
-        <v>-0.9222782825668787</v>
+        <v>-0.9222782825668805</v>
       </c>
       <c r="I5" s="19" t="n">
         <v>39.2365270656978</v>
@@ -3671,7 +3917,7 @@
         <v>-1.705489657739689</v>
       </c>
       <c r="K5" s="36" t="n">
-        <v>-0.1985558514348225</v>
+        <v>-0.198555851434822</v>
       </c>
       <c r="L5" s="19" t="n">
         <v>8.504081918942456</v>
@@ -3680,7 +3926,7 @@
         <v>-2.79793443077293</v>
       </c>
       <c r="N5" s="36" t="n">
-        <v>-0.2751158236976585</v>
+        <v>-0.2751158236976581</v>
       </c>
       <c r="O5" s="19" t="n">
         <v>7.013124523672051</v>
@@ -3791,26 +4037,66 @@
           <t>7/4/69</t>
         </is>
       </c>
-      <c r="B9" s="33" t="n"/>
-      <c r="C9" s="33" t="n"/>
-      <c r="D9" s="33" t="n"/>
-      <c r="E9" s="33" t="n"/>
-      <c r="F9" s="12" t="n"/>
-      <c r="G9" s="33" t="n"/>
-      <c r="H9" s="33" t="n"/>
-      <c r="I9" s="12" t="n"/>
-      <c r="J9" s="33" t="n"/>
-      <c r="K9" s="33" t="n"/>
-      <c r="L9" s="12" t="n"/>
-      <c r="M9" s="33" t="n"/>
-      <c r="N9" s="33" t="n"/>
-      <c r="O9" s="12" t="n"/>
-      <c r="P9" s="33" t="n"/>
-      <c r="Q9" s="33" t="n"/>
-      <c r="R9" s="12" t="n"/>
-      <c r="S9" s="33" t="n"/>
-      <c r="T9" s="33" t="n"/>
-      <c r="U9" s="12" t="n"/>
+      <c r="B9" s="35" t="n">
+        <v>4.54670995947327</v>
+      </c>
+      <c r="C9" s="35" t="n">
+        <v>0.3597773776846278</v>
+      </c>
+      <c r="D9" s="35" t="n">
+        <v>0.1589133858329816</v>
+      </c>
+      <c r="E9" s="35" t="n">
+        <v>0.03380454313506304</v>
+      </c>
+      <c r="F9" s="19" t="n">
+        <v>15.73147231918833</v>
+      </c>
+      <c r="G9" s="35" t="n">
+        <v>16.30968964991566</v>
+      </c>
+      <c r="H9" s="35" t="n">
+        <v>0.7032511058611615</v>
+      </c>
+      <c r="I9" s="19" t="n">
+        <v>39.47520867717733</v>
+      </c>
+      <c r="J9" s="36" t="n">
+        <v>-1.631124094698189</v>
+      </c>
+      <c r="K9" s="35" t="n">
+        <v>0.07436556304150033</v>
+      </c>
+      <c r="L9" s="19" t="n">
+        <v>8.510515755764585</v>
+      </c>
+      <c r="M9" s="36" t="n">
+        <v>-2.610173450399955</v>
+      </c>
+      <c r="N9" s="35" t="n">
+        <v>0.1877609803729747</v>
+      </c>
+      <c r="O9" s="19" t="n">
+        <v>7.026671469699702</v>
+      </c>
+      <c r="P9" s="36" t="n">
+        <v>-0.7697759192838771</v>
+      </c>
+      <c r="Q9" s="35" t="n">
+        <v>0.06402741524638156</v>
+      </c>
+      <c r="R9" s="19" t="n">
+        <v>15.08672754982331</v>
+      </c>
+      <c r="S9" s="35" t="n">
+        <v>15.822730185473</v>
+      </c>
+      <c r="T9" s="35" t="n">
+        <v>1.095454658450688</v>
+      </c>
+      <c r="U9" s="19" t="n">
+        <v>11.42568187506592</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="10" t="inlineStr">
@@ -4480,14 +4766,14 @@
       </c>
       <c r="B1" s="4" t="inlineStr">
         <is>
-          <t>3 เม.ย. 69 (ศุกร์)</t>
+          <t>7 เม.ย. 69 (อังคาร)</t>
         </is>
       </c>
       <c r="C1" s="20" t="n"/>
       <c r="D1" s="20" t="n"/>
       <c r="E1" s="21" t="inlineStr">
         <is>
-          <t>2 เม.ย. 69 (พฤหัส)</t>
+          <t>3 เม.ย. 69 (ศุกร์)</t>
         </is>
       </c>
       <c r="F1" s="20" t="n"/>
@@ -4550,27 +4836,27 @@
       <c r="G3" s="20" t="n"/>
       <c r="H3" s="22" t="inlineStr">
         <is>
+          <t>7/4/69</t>
+        </is>
+      </c>
+      <c r="I3" s="22" t="inlineStr">
+        <is>
           <t>3/4/69</t>
         </is>
       </c>
-      <c r="I3" s="22" t="inlineStr">
+      <c r="J3" s="22" t="inlineStr">
         <is>
           <t>2/4/69</t>
         </is>
       </c>
-      <c r="J3" s="22" t="inlineStr">
+      <c r="K3" s="22" t="inlineStr">
         <is>
           <t>1/4/69</t>
         </is>
       </c>
-      <c r="K3" s="22" t="inlineStr">
+      <c r="L3" s="22" t="inlineStr">
         <is>
           <t>31/3/69</t>
-        </is>
-      </c>
-      <c r="L3" s="22" t="inlineStr">
-        <is>
-          <t>30/3/69</t>
         </is>
       </c>
     </row>
@@ -4581,37 +4867,37 @@
         </is>
       </c>
       <c r="B4" s="39" t="n">
+        <v>0.1589133858329816</v>
+      </c>
+      <c r="C4" s="39" t="n">
+        <v>0.03380454313506304</v>
+      </c>
+      <c r="D4" s="26" t="n">
+        <v>15.73147231918833</v>
+      </c>
+      <c r="E4" s="39" t="n">
         <v>0.1251088426979186</v>
       </c>
-      <c r="C4" s="39" t="n">
-        <v>0.03628829045054793</v>
-      </c>
-      <c r="D4" s="26" t="n">
+      <c r="F4" s="39" t="n">
+        <v>0.03628829045054799</v>
+      </c>
+      <c r="G4" s="26" t="n">
         <v>15.72616280437217</v>
       </c>
-      <c r="E4" s="39" t="n">
+      <c r="H4" s="39" t="n">
+        <v>0.1589133858329816</v>
+      </c>
+      <c r="I4" s="39" t="n">
+        <v>0.1251088426979186</v>
+      </c>
+      <c r="J4" s="39" t="n">
         <v>0.08882055224737062</v>
       </c>
-      <c r="F4" s="37" t="n">
-        <v>-0.05878939264665209</v>
-      </c>
-      <c r="G4" s="26" t="n">
-        <v>15.72046317947174</v>
-      </c>
-      <c r="H4" s="39" t="n">
-        <v>0.1251088426979186</v>
-      </c>
-      <c r="I4" s="39" t="n">
-        <v>0.08882055224737062</v>
-      </c>
-      <c r="J4" s="39" t="n">
+      <c r="K4" s="39" t="n">
         <v>0.1476099448940227</v>
       </c>
-      <c r="K4" s="37" t="n">
+      <c r="L4" s="37" t="n">
         <v>-0.2878859071354989</v>
-      </c>
-      <c r="L4" s="37" t="n">
-        <v>-0.4248326439501127</v>
       </c>
     </row>
     <row r="5">
@@ -4621,37 +4907,37 @@
         </is>
       </c>
       <c r="B5" s="39" t="n">
+        <v>16.30968964991566</v>
+      </c>
+      <c r="C5" s="39" t="n">
+        <v>0.7032511058611615</v>
+      </c>
+      <c r="D5" s="26" t="n">
+        <v>39.47520867717733</v>
+      </c>
+      <c r="E5" s="39" t="n">
         <v>15.6064385440545</v>
       </c>
-      <c r="C5" s="37" t="n">
-        <v>-0.9222782825668787</v>
-      </c>
-      <c r="D5" s="26" t="n">
+      <c r="F5" s="37" t="n">
+        <v>-0.9222782825668805</v>
+      </c>
+      <c r="G5" s="26" t="n">
         <v>39.2365270656978</v>
       </c>
-      <c r="E5" s="39" t="n">
+      <c r="H5" s="39" t="n">
+        <v>16.30968964991566</v>
+      </c>
+      <c r="I5" s="39" t="n">
+        <v>15.6064385440545</v>
+      </c>
+      <c r="J5" s="39" t="n">
         <v>16.52871682662138</v>
       </c>
-      <c r="F5" s="37" t="n">
-        <v>-0.4670407562319383</v>
-      </c>
-      <c r="G5" s="26" t="n">
-        <v>39.54954593602872</v>
-      </c>
-      <c r="H5" s="39" t="n">
-        <v>15.6064385440545</v>
-      </c>
-      <c r="I5" s="39" t="n">
-        <v>16.52871682662138</v>
-      </c>
-      <c r="J5" s="39" t="n">
+      <c r="K5" s="39" t="n">
         <v>16.99575758285332</v>
       </c>
-      <c r="K5" s="39" t="n">
+      <c r="L5" s="39" t="n">
         <v>15.20400685698138</v>
-      </c>
-      <c r="L5" s="39" t="n">
-        <v>15.072598216802</v>
       </c>
     </row>
     <row r="6">
@@ -4661,37 +4947,37 @@
         </is>
       </c>
       <c r="B6" s="37" t="n">
+        <v>-1.631124094698189</v>
+      </c>
+      <c r="C6" s="39" t="n">
+        <v>0.07436556304150033</v>
+      </c>
+      <c r="D6" s="26" t="n">
+        <v>8.510515755764585</v>
+      </c>
+      <c r="E6" s="37" t="n">
         <v>-1.705489657739689</v>
       </c>
-      <c r="C6" s="37" t="n">
-        <v>-0.1985558514348225</v>
-      </c>
-      <c r="D6" s="26" t="n">
+      <c r="F6" s="37" t="n">
+        <v>-0.198555851434822</v>
+      </c>
+      <c r="G6" s="26" t="n">
         <v>8.504081918942456</v>
       </c>
-      <c r="E6" s="37" t="n">
+      <c r="H6" s="37" t="n">
+        <v>-1.631124094698189</v>
+      </c>
+      <c r="I6" s="37" t="n">
+        <v>-1.705489657739689</v>
+      </c>
+      <c r="J6" s="37" t="n">
         <v>-1.506933806304867</v>
       </c>
-      <c r="F6" s="39" t="n">
-        <v>0.3881442431810211</v>
-      </c>
-      <c r="G6" s="26" t="n">
-        <v>8.521260245791103</v>
-      </c>
-      <c r="H6" s="37" t="n">
-        <v>-1.705489657739689</v>
-      </c>
-      <c r="I6" s="37" t="n">
-        <v>-1.506933806304867</v>
-      </c>
-      <c r="J6" s="37" t="n">
+      <c r="K6" s="37" t="n">
         <v>-1.895078049485888</v>
       </c>
-      <c r="K6" s="37" t="n">
+      <c r="L6" s="37" t="n">
         <v>-2.740157540816912</v>
-      </c>
-      <c r="L6" s="37" t="n">
-        <v>-2.854845562272235</v>
       </c>
     </row>
     <row r="7">
@@ -4701,37 +4987,37 @@
         </is>
       </c>
       <c r="B7" s="37" t="n">
+        <v>-2.610173450399955</v>
+      </c>
+      <c r="C7" s="39" t="n">
+        <v>0.1877609803729747</v>
+      </c>
+      <c r="D7" s="26" t="n">
+        <v>7.026671469699702</v>
+      </c>
+      <c r="E7" s="37" t="n">
         <v>-2.79793443077293</v>
       </c>
-      <c r="C7" s="37" t="n">
-        <v>-0.2751158236976585</v>
-      </c>
-      <c r="D7" s="26" t="n">
+      <c r="F7" s="37" t="n">
+        <v>-0.2751158236976581</v>
+      </c>
+      <c r="G7" s="26" t="n">
         <v>7.013124523672051</v>
       </c>
-      <c r="E7" s="37" t="n">
+      <c r="H7" s="37" t="n">
+        <v>-2.610173450399955</v>
+      </c>
+      <c r="I7" s="37" t="n">
+        <v>-2.79793443077293</v>
+      </c>
+      <c r="J7" s="37" t="n">
         <v>-2.522818607075272</v>
       </c>
-      <c r="F7" s="39" t="n">
-        <v>1.205717881181168</v>
-      </c>
-      <c r="G7" s="26" t="n">
-        <v>7.032974117595034</v>
-      </c>
-      <c r="H7" s="37" t="n">
-        <v>-2.79793443077293</v>
-      </c>
-      <c r="I7" s="37" t="n">
-        <v>-2.522818607075272</v>
-      </c>
-      <c r="J7" s="37" t="n">
+      <c r="K7" s="37" t="n">
         <v>-3.72853648825644</v>
       </c>
-      <c r="K7" s="37" t="n">
+      <c r="L7" s="37" t="n">
         <v>-6.024876222296427</v>
-      </c>
-      <c r="L7" s="37" t="n">
-        <v>-5.301414806346127</v>
       </c>
     </row>
     <row r="8">
@@ -4741,37 +5027,37 @@
         </is>
       </c>
       <c r="B8" s="37" t="n">
+        <v>-0.7697759192838771</v>
+      </c>
+      <c r="C8" s="39" t="n">
+        <v>0.06402741524638156</v>
+      </c>
+      <c r="D8" s="26" t="n">
+        <v>15.08672754982331</v>
+      </c>
+      <c r="E8" s="37" t="n">
         <v>-0.8338033345302587</v>
       </c>
-      <c r="C8" s="37" t="n">
+      <c r="F8" s="37" t="n">
         <v>-0.08030474413646127</v>
       </c>
-      <c r="D8" s="26" t="n">
+      <c r="G8" s="26" t="n">
         <v>15.07699297370509</v>
       </c>
-      <c r="E8" s="37" t="n">
+      <c r="H8" s="37" t="n">
+        <v>-0.7697759192838771</v>
+      </c>
+      <c r="I8" s="37" t="n">
+        <v>-0.8338033345302587</v>
+      </c>
+      <c r="J8" s="37" t="n">
         <v>-0.7534985903937974</v>
       </c>
-      <c r="F8" s="39" t="n">
-        <v>1.124850726317406</v>
-      </c>
-      <c r="G8" s="26" t="n">
-        <v>15.08920231624129</v>
-      </c>
-      <c r="H8" s="37" t="n">
-        <v>-0.8338033345302587</v>
-      </c>
-      <c r="I8" s="37" t="n">
-        <v>-0.7534985903937974</v>
-      </c>
-      <c r="J8" s="37" t="n">
+      <c r="K8" s="37" t="n">
         <v>-1.878349316711203</v>
       </c>
-      <c r="K8" s="37" t="n">
+      <c r="L8" s="37" t="n">
         <v>-4.454855437138572</v>
-      </c>
-      <c r="L8" s="37" t="n">
-        <v>-4.207762322643516</v>
       </c>
     </row>
     <row r="9">
@@ -4781,37 +5067,37 @@
         </is>
       </c>
       <c r="B9" s="39" t="n">
+        <v>15.822730185473</v>
+      </c>
+      <c r="C9" s="39" t="n">
+        <v>1.095454658450688</v>
+      </c>
+      <c r="D9" s="26" t="n">
+        <v>11.42568187506592</v>
+      </c>
+      <c r="E9" s="39" t="n">
         <v>14.72727552702231</v>
       </c>
-      <c r="C9" s="37" t="n">
+      <c r="F9" s="37" t="n">
         <v>-1.03069220173415</v>
       </c>
-      <c r="D9" s="26" t="n">
+      <c r="G9" s="26" t="n">
         <v>11.3176174526855</v>
       </c>
-      <c r="E9" s="39" t="n">
+      <c r="H9" s="39" t="n">
+        <v>15.822730185473</v>
+      </c>
+      <c r="I9" s="39" t="n">
+        <v>14.72727552702231</v>
+      </c>
+      <c r="J9" s="39" t="n">
         <v>15.75796772875646</v>
       </c>
-      <c r="F9" s="37" t="n">
-        <v>-0.04344751420812898</v>
-      </c>
-      <c r="G9" s="26" t="n">
-        <v>11.41929318757163</v>
-      </c>
-      <c r="H9" s="39" t="n">
-        <v>14.72727552702231</v>
-      </c>
-      <c r="I9" s="39" t="n">
-        <v>15.75796772875646</v>
-      </c>
-      <c r="J9" s="39" t="n">
+      <c r="K9" s="39" t="n">
         <v>15.80141524296459</v>
       </c>
-      <c r="K9" s="39" t="n">
+      <c r="L9" s="39" t="n">
         <v>14.98670735933121</v>
-      </c>
-      <c r="L9" s="39" t="n">
-        <v>15.78577423692808</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
EGAT retirement pages update 2026-04-10T04:15:05Z
</commit_message>
<xml_diff>
--- a/EGAT Retirement.xlsx
+++ b/EGAT Retirement.xlsx
@@ -683,7 +683,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I11"/>
+  <dimension ref="A1:I12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1153,6 +1153,47 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>11:15:04</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>EGAT1</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>ตราสารหนี้ (EGAT-1)</t>
+        </is>
+      </c>
+      <c r="F12" t="n">
+        <v>15.75751902428132</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0.6144018594892664</v>
+      </c>
+      <c r="H12" t="n">
+        <v>0.3247471759871168</v>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>https://app.powerbi.com/view?r=eyJrIjoiMzZjYWU3YmQtNWQ1Ny00NjdjLWI1MmEtYjExY2ZiYWIxMzNiIiwidCI6IjVmZWJjNjlmLThlOWMtNDcwOC1iNzBlLWQ4YzYyYmUxODA1YiIsImMiOjEwfQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1164,7 +1205,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I11"/>
+  <dimension ref="A1:I12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1634,6 +1675,47 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>11:15:04</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>EGAT2</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>ตราสารทุน (EGAT-2)</t>
+        </is>
+      </c>
+      <c r="F12" t="n">
+        <v>40.14404168359091</v>
+      </c>
+      <c r="G12" t="n">
+        <v>2.670333560722571</v>
+      </c>
+      <c r="H12" t="n">
+        <v>18.2803381153805</v>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>https://app.powerbi.com/view?r=eyJrIjoiMzZjYWU3YmQtNWQ1Ny00NjdjLWI1MmEtYjExY2ZiYWIxMzNiIiwidCI6IjVmZWJjNjlmLThlOWMtNDcwOC1iNzBlLWQ4YzYyYmUxODA1YiIsImMiOjEwfQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1645,7 +1727,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I11"/>
+  <dimension ref="A1:I12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -2115,6 +2197,47 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>11:15:04</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>EGAT3</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>อสังหาริมทรัพย์และโครงสร้างพื้นฐาน (EGAT-3)</t>
+        </is>
+      </c>
+      <c r="F12" t="n">
+        <v>8.648509211476886</v>
+      </c>
+      <c r="G12" t="n">
+        <v>2.780214346779264</v>
+      </c>
+      <c r="H12" t="n">
+        <v>-0.0361254471118011</v>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>https://app.powerbi.com/view?r=eyJrIjoiMzZjYWU3YmQtNWQ1Ny00NjdjLWI1MmEtYjExY2ZiYWIxMzNiIiwidCI6IjVmZWJjNjlmLThlOWMtNDcwOC1iNzBlLWQ4YzYyYmUxODA1YiIsImMiOjEwfQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2126,7 +2249,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I11"/>
+  <dimension ref="A1:I12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -2596,6 +2719,47 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>11:15:04</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>EGAT4</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>ตราสารทุนต่างประเทศ (EGAT-4)</t>
+        </is>
+      </c>
+      <c r="F12" t="n">
+        <v>6.981342578519967</v>
+      </c>
+      <c r="G12" t="n">
+        <v>2.965086073961731</v>
+      </c>
+      <c r="H12" t="n">
+        <v>-3.238432914175438</v>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>https://app.powerbi.com/view?r=eyJrIjoiMzZjYWU3YmQtNWQ1Ny00NjdjLWI1MmEtYjExY2ZiYWIxMzNiIiwidCI6IjVmZWJjNjlmLThlOWMtNDcwOC1iNzBlLWQ4YzYyYmUxODA1YiIsImMiOjEwfQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2607,7 +2771,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I11"/>
+  <dimension ref="A1:I12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -3077,6 +3241,47 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>11:15:04</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>EGAT5</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>ตราสารทุนต่างประเทศแบบอิงดัชนี (EGAT-5)</t>
+        </is>
+      </c>
+      <c r="F12" t="n">
+        <v>14.96953906501773</v>
+      </c>
+      <c r="G12" t="n">
+        <v>3.05017429189447</v>
+      </c>
+      <c r="H12" t="n">
+        <v>-1.540562000528767</v>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>https://app.powerbi.com/view?r=eyJrIjoiMzZjYWU3YmQtNWQ1Ny00NjdjLWI1MmEtYjExY2ZiYWIxMzNiIiwidCI6IjVmZWJjNjlmLThlOWMtNDcwOC1iNzBlLWQ4YzYyYmUxODA1YiIsImMiOjEwfQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3088,7 +3293,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I11"/>
+  <dimension ref="A1:I12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -3553,6 +3758,47 @@
         <v>15.822730185473</v>
       </c>
       <c r="I11" t="inlineStr">
+        <is>
+          <t>https://app.powerbi.com/view?r=eyJrIjoiMzZjYWU3YmQtNWQ1Ny00NjdjLWI1MmEtYjExY2ZiYWIxMzNiIiwidCI6IjVmZWJjNjlmLThlOWMtNDcwOC1iNzBlLWQ4YzYyYmUxODA1YiIsImMiOjEwfQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>11:15:04</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>EGAT6</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>การลงทุนตามหลักศาสนาอิสลาม (EGAT-6)</t>
+        </is>
+      </c>
+      <c r="F12" t="n">
+        <v>11.49202139040016</v>
+      </c>
+      <c r="G12" t="n">
+        <v>1.311899410718032</v>
+      </c>
+      <c r="H12" t="n">
+        <v>16.49521729558234</v>
+      </c>
+      <c r="I12" t="inlineStr">
         <is>
           <t>https://app.powerbi.com/view?r=eyJrIjoiMzZjYWU3YmQtNWQ1Ny00NjdjLWI1MmEtYjExY2ZiYWIxMzNiIiwidCI6IjVmZWJjNjlmLThlOWMtNDcwOC1iNzBlLWQ4YzYyYmUxODA1YiIsImMiOjEwfQ%3D%3D</t>
         </is>
@@ -4038,16 +4284,16 @@
         </is>
       </c>
       <c r="B9" s="35" t="n">
-        <v>4.54670995947327</v>
+        <v>4.546709959473271</v>
       </c>
       <c r="C9" s="35" t="n">
-        <v>0.3597773776846278</v>
+        <v>0.3597773776846287</v>
       </c>
       <c r="D9" s="35" t="n">
         <v>0.1589133858329816</v>
       </c>
       <c r="E9" s="35" t="n">
-        <v>0.03380454313506304</v>
+        <v>0.03380454313506298</v>
       </c>
       <c r="F9" s="19" t="n">
         <v>15.73147231918833</v>
@@ -4065,7 +4311,7 @@
         <v>-1.631124094698189</v>
       </c>
       <c r="K9" s="35" t="n">
-        <v>0.07436556304150033</v>
+        <v>0.07436556304149988</v>
       </c>
       <c r="L9" s="19" t="n">
         <v>8.510515755764585</v>
@@ -4092,7 +4338,7 @@
         <v>15.822730185473</v>
       </c>
       <c r="T9" s="35" t="n">
-        <v>1.095454658450688</v>
+        <v>1.09545465845069</v>
       </c>
       <c r="U9" s="19" t="n">
         <v>11.42568187506592</v>
@@ -4104,26 +4350,66 @@
           <t>8/4/69</t>
         </is>
       </c>
-      <c r="B10" s="33" t="n"/>
-      <c r="C10" s="33" t="n"/>
-      <c r="D10" s="33" t="n"/>
-      <c r="E10" s="33" t="n"/>
-      <c r="F10" s="12" t="n"/>
-      <c r="G10" s="33" t="n"/>
-      <c r="H10" s="33" t="n"/>
-      <c r="I10" s="12" t="n"/>
-      <c r="J10" s="33" t="n"/>
-      <c r="K10" s="33" t="n"/>
-      <c r="L10" s="12" t="n"/>
-      <c r="M10" s="33" t="n"/>
-      <c r="N10" s="33" t="n"/>
-      <c r="O10" s="12" t="n"/>
-      <c r="P10" s="33" t="n"/>
-      <c r="Q10" s="33" t="n"/>
-      <c r="R10" s="12" t="n"/>
-      <c r="S10" s="33" t="n"/>
-      <c r="T10" s="33" t="n"/>
-      <c r="U10" s="12" t="n"/>
+      <c r="B10" s="35" t="n">
+        <v>5.047530370855659</v>
+      </c>
+      <c r="C10" s="35" t="n">
+        <v>0.5008204113823886</v>
+      </c>
+      <c r="D10" s="35" t="n">
+        <v>0.3247471759871168</v>
+      </c>
+      <c r="E10" s="35" t="n">
+        <v>0.1658337901541352</v>
+      </c>
+      <c r="F10" s="19" t="n">
+        <v>15.75751902428132</v>
+      </c>
+      <c r="G10" s="35" t="n">
+        <v>18.2803381153805</v>
+      </c>
+      <c r="H10" s="35" t="n">
+        <v>1.970648465464841</v>
+      </c>
+      <c r="I10" s="19" t="n">
+        <v>40.14404168359091</v>
+      </c>
+      <c r="J10" s="36" t="n">
+        <v>-0.0361254471118011</v>
+      </c>
+      <c r="K10" s="35" t="n">
+        <v>1.594998647586388</v>
+      </c>
+      <c r="L10" s="19" t="n">
+        <v>8.648509211476886</v>
+      </c>
+      <c r="M10" s="36" t="n">
+        <v>-3.238432914175438</v>
+      </c>
+      <c r="N10" s="36" t="n">
+        <v>-0.6282594637754824</v>
+      </c>
+      <c r="O10" s="19" t="n">
+        <v>6.981342578519967</v>
+      </c>
+      <c r="P10" s="36" t="n">
+        <v>-1.540562000528767</v>
+      </c>
+      <c r="Q10" s="36" t="n">
+        <v>-0.7707860812448897</v>
+      </c>
+      <c r="R10" s="19" t="n">
+        <v>14.96953906501773</v>
+      </c>
+      <c r="S10" s="35" t="n">
+        <v>16.49521729558234</v>
+      </c>
+      <c r="T10" s="35" t="n">
+        <v>0.6724871101093424</v>
+      </c>
+      <c r="U10" s="19" t="n">
+        <v>11.49202139040016</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="10" t="inlineStr">
@@ -4766,14 +5052,14 @@
       </c>
       <c r="B1" s="4" t="inlineStr">
         <is>
-          <t>7 เม.ย. 69 (อังคาร)</t>
+          <t>8 เม.ย. 69 (พุธ)</t>
         </is>
       </c>
       <c r="C1" s="20" t="n"/>
       <c r="D1" s="20" t="n"/>
       <c r="E1" s="21" t="inlineStr">
         <is>
-          <t>3 เม.ย. 69 (ศุกร์)</t>
+          <t>7 เม.ย. 69 (อังคาร)</t>
         </is>
       </c>
       <c r="F1" s="20" t="n"/>
@@ -4836,27 +5122,27 @@
       <c r="G3" s="20" t="n"/>
       <c r="H3" s="22" t="inlineStr">
         <is>
+          <t>8/4/69</t>
+        </is>
+      </c>
+      <c r="I3" s="22" t="inlineStr">
+        <is>
           <t>7/4/69</t>
         </is>
       </c>
-      <c r="I3" s="22" t="inlineStr">
+      <c r="J3" s="22" t="inlineStr">
         <is>
           <t>3/4/69</t>
         </is>
       </c>
-      <c r="J3" s="22" t="inlineStr">
+      <c r="K3" s="22" t="inlineStr">
         <is>
           <t>2/4/69</t>
         </is>
       </c>
-      <c r="K3" s="22" t="inlineStr">
+      <c r="L3" s="22" t="inlineStr">
         <is>
           <t>1/4/69</t>
-        </is>
-      </c>
-      <c r="L3" s="22" t="inlineStr">
-        <is>
-          <t>31/3/69</t>
         </is>
       </c>
     </row>
@@ -4867,37 +5153,37 @@
         </is>
       </c>
       <c r="B4" s="39" t="n">
+        <v>0.3247471759871168</v>
+      </c>
+      <c r="C4" s="39" t="n">
+        <v>0.1658337901541352</v>
+      </c>
+      <c r="D4" s="26" t="n">
+        <v>15.75751902428132</v>
+      </c>
+      <c r="E4" s="39" t="n">
         <v>0.1589133858329816</v>
       </c>
-      <c r="C4" s="39" t="n">
-        <v>0.03380454313506304</v>
-      </c>
-      <c r="D4" s="26" t="n">
+      <c r="F4" s="39" t="n">
+        <v>0.03380454313506298</v>
+      </c>
+      <c r="G4" s="26" t="n">
         <v>15.73147231918833</v>
       </c>
-      <c r="E4" s="39" t="n">
+      <c r="H4" s="39" t="n">
+        <v>0.3247471759871168</v>
+      </c>
+      <c r="I4" s="39" t="n">
+        <v>0.1589133858329816</v>
+      </c>
+      <c r="J4" s="39" t="n">
         <v>0.1251088426979186</v>
       </c>
-      <c r="F4" s="39" t="n">
-        <v>0.03628829045054799</v>
-      </c>
-      <c r="G4" s="26" t="n">
-        <v>15.72616280437217</v>
-      </c>
-      <c r="H4" s="39" t="n">
-        <v>0.1589133858329816</v>
-      </c>
-      <c r="I4" s="39" t="n">
-        <v>0.1251088426979186</v>
-      </c>
-      <c r="J4" s="39" t="n">
+      <c r="K4" s="39" t="n">
         <v>0.08882055224737062</v>
       </c>
-      <c r="K4" s="39" t="n">
+      <c r="L4" s="39" t="n">
         <v>0.1476099448940227</v>
-      </c>
-      <c r="L4" s="37" t="n">
-        <v>-0.2878859071354989</v>
       </c>
     </row>
     <row r="5">
@@ -4907,37 +5193,37 @@
         </is>
       </c>
       <c r="B5" s="39" t="n">
+        <v>18.2803381153805</v>
+      </c>
+      <c r="C5" s="39" t="n">
+        <v>1.970648465464841</v>
+      </c>
+      <c r="D5" s="26" t="n">
+        <v>40.14404168359091</v>
+      </c>
+      <c r="E5" s="39" t="n">
         <v>16.30968964991566</v>
       </c>
-      <c r="C5" s="39" t="n">
+      <c r="F5" s="39" t="n">
         <v>0.7032511058611615</v>
       </c>
-      <c r="D5" s="26" t="n">
+      <c r="G5" s="26" t="n">
         <v>39.47520867717733</v>
       </c>
-      <c r="E5" s="39" t="n">
+      <c r="H5" s="39" t="n">
+        <v>18.2803381153805</v>
+      </c>
+      <c r="I5" s="39" t="n">
+        <v>16.30968964991566</v>
+      </c>
+      <c r="J5" s="39" t="n">
         <v>15.6064385440545</v>
       </c>
-      <c r="F5" s="37" t="n">
-        <v>-0.9222782825668805</v>
-      </c>
-      <c r="G5" s="26" t="n">
-        <v>39.2365270656978</v>
-      </c>
-      <c r="H5" s="39" t="n">
-        <v>16.30968964991566</v>
-      </c>
-      <c r="I5" s="39" t="n">
-        <v>15.6064385440545</v>
-      </c>
-      <c r="J5" s="39" t="n">
+      <c r="K5" s="39" t="n">
         <v>16.52871682662138</v>
       </c>
-      <c r="K5" s="39" t="n">
+      <c r="L5" s="39" t="n">
         <v>16.99575758285332</v>
-      </c>
-      <c r="L5" s="39" t="n">
-        <v>15.20400685698138</v>
       </c>
     </row>
     <row r="6">
@@ -4947,37 +5233,37 @@
         </is>
       </c>
       <c r="B6" s="37" t="n">
+        <v>-0.0361254471118011</v>
+      </c>
+      <c r="C6" s="39" t="n">
+        <v>1.594998647586388</v>
+      </c>
+      <c r="D6" s="26" t="n">
+        <v>8.648509211476886</v>
+      </c>
+      <c r="E6" s="37" t="n">
         <v>-1.631124094698189</v>
       </c>
-      <c r="C6" s="39" t="n">
-        <v>0.07436556304150033</v>
-      </c>
-      <c r="D6" s="26" t="n">
+      <c r="F6" s="39" t="n">
+        <v>0.07436556304149988</v>
+      </c>
+      <c r="G6" s="26" t="n">
         <v>8.510515755764585</v>
       </c>
-      <c r="E6" s="37" t="n">
+      <c r="H6" s="37" t="n">
+        <v>-0.0361254471118011</v>
+      </c>
+      <c r="I6" s="37" t="n">
+        <v>-1.631124094698189</v>
+      </c>
+      <c r="J6" s="37" t="n">
         <v>-1.705489657739689</v>
       </c>
-      <c r="F6" s="37" t="n">
-        <v>-0.198555851434822</v>
-      </c>
-      <c r="G6" s="26" t="n">
-        <v>8.504081918942456</v>
-      </c>
-      <c r="H6" s="37" t="n">
-        <v>-1.631124094698189</v>
-      </c>
-      <c r="I6" s="37" t="n">
-        <v>-1.705489657739689</v>
-      </c>
-      <c r="J6" s="37" t="n">
+      <c r="K6" s="37" t="n">
         <v>-1.506933806304867</v>
       </c>
-      <c r="K6" s="37" t="n">
+      <c r="L6" s="37" t="n">
         <v>-1.895078049485888</v>
-      </c>
-      <c r="L6" s="37" t="n">
-        <v>-2.740157540816912</v>
       </c>
     </row>
     <row r="7">
@@ -4987,37 +5273,37 @@
         </is>
       </c>
       <c r="B7" s="37" t="n">
+        <v>-3.238432914175438</v>
+      </c>
+      <c r="C7" s="37" t="n">
+        <v>-0.6282594637754824</v>
+      </c>
+      <c r="D7" s="26" t="n">
+        <v>6.981342578519967</v>
+      </c>
+      <c r="E7" s="37" t="n">
         <v>-2.610173450399955</v>
       </c>
-      <c r="C7" s="39" t="n">
+      <c r="F7" s="39" t="n">
         <v>0.1877609803729747</v>
       </c>
-      <c r="D7" s="26" t="n">
+      <c r="G7" s="26" t="n">
         <v>7.026671469699702</v>
       </c>
-      <c r="E7" s="37" t="n">
+      <c r="H7" s="37" t="n">
+        <v>-3.238432914175438</v>
+      </c>
+      <c r="I7" s="37" t="n">
+        <v>-2.610173450399955</v>
+      </c>
+      <c r="J7" s="37" t="n">
         <v>-2.79793443077293</v>
       </c>
-      <c r="F7" s="37" t="n">
-        <v>-0.2751158236976581</v>
-      </c>
-      <c r="G7" s="26" t="n">
-        <v>7.013124523672051</v>
-      </c>
-      <c r="H7" s="37" t="n">
-        <v>-2.610173450399955</v>
-      </c>
-      <c r="I7" s="37" t="n">
-        <v>-2.79793443077293</v>
-      </c>
-      <c r="J7" s="37" t="n">
+      <c r="K7" s="37" t="n">
         <v>-2.522818607075272</v>
       </c>
-      <c r="K7" s="37" t="n">
+      <c r="L7" s="37" t="n">
         <v>-3.72853648825644</v>
-      </c>
-      <c r="L7" s="37" t="n">
-        <v>-6.024876222296427</v>
       </c>
     </row>
     <row r="8">
@@ -5027,37 +5313,37 @@
         </is>
       </c>
       <c r="B8" s="37" t="n">
+        <v>-1.540562000528767</v>
+      </c>
+      <c r="C8" s="37" t="n">
+        <v>-0.7707860812448897</v>
+      </c>
+      <c r="D8" s="26" t="n">
+        <v>14.96953906501773</v>
+      </c>
+      <c r="E8" s="37" t="n">
         <v>-0.7697759192838771</v>
       </c>
-      <c r="C8" s="39" t="n">
+      <c r="F8" s="39" t="n">
         <v>0.06402741524638156</v>
       </c>
-      <c r="D8" s="26" t="n">
+      <c r="G8" s="26" t="n">
         <v>15.08672754982331</v>
       </c>
-      <c r="E8" s="37" t="n">
+      <c r="H8" s="37" t="n">
+        <v>-1.540562000528767</v>
+      </c>
+      <c r="I8" s="37" t="n">
+        <v>-0.7697759192838771</v>
+      </c>
+      <c r="J8" s="37" t="n">
         <v>-0.8338033345302587</v>
       </c>
-      <c r="F8" s="37" t="n">
-        <v>-0.08030474413646127</v>
-      </c>
-      <c r="G8" s="26" t="n">
-        <v>15.07699297370509</v>
-      </c>
-      <c r="H8" s="37" t="n">
-        <v>-0.7697759192838771</v>
-      </c>
-      <c r="I8" s="37" t="n">
-        <v>-0.8338033345302587</v>
-      </c>
-      <c r="J8" s="37" t="n">
+      <c r="K8" s="37" t="n">
         <v>-0.7534985903937974</v>
       </c>
-      <c r="K8" s="37" t="n">
+      <c r="L8" s="37" t="n">
         <v>-1.878349316711203</v>
-      </c>
-      <c r="L8" s="37" t="n">
-        <v>-4.454855437138572</v>
       </c>
     </row>
     <row r="9">
@@ -5067,37 +5353,37 @@
         </is>
       </c>
       <c r="B9" s="39" t="n">
+        <v>16.49521729558234</v>
+      </c>
+      <c r="C9" s="39" t="n">
+        <v>0.6724871101093424</v>
+      </c>
+      <c r="D9" s="26" t="n">
+        <v>11.49202139040016</v>
+      </c>
+      <c r="E9" s="39" t="n">
         <v>15.822730185473</v>
       </c>
-      <c r="C9" s="39" t="n">
-        <v>1.095454658450688</v>
-      </c>
-      <c r="D9" s="26" t="n">
+      <c r="F9" s="39" t="n">
+        <v>1.09545465845069</v>
+      </c>
+      <c r="G9" s="26" t="n">
         <v>11.42568187506592</v>
       </c>
-      <c r="E9" s="39" t="n">
+      <c r="H9" s="39" t="n">
+        <v>16.49521729558234</v>
+      </c>
+      <c r="I9" s="39" t="n">
+        <v>15.822730185473</v>
+      </c>
+      <c r="J9" s="39" t="n">
         <v>14.72727552702231</v>
       </c>
-      <c r="F9" s="37" t="n">
-        <v>-1.03069220173415</v>
-      </c>
-      <c r="G9" s="26" t="n">
-        <v>11.3176174526855</v>
-      </c>
-      <c r="H9" s="39" t="n">
-        <v>15.822730185473</v>
-      </c>
-      <c r="I9" s="39" t="n">
-        <v>14.72727552702231</v>
-      </c>
-      <c r="J9" s="39" t="n">
+      <c r="K9" s="39" t="n">
         <v>15.75796772875646</v>
       </c>
-      <c r="K9" s="39" t="n">
+      <c r="L9" s="39" t="n">
         <v>15.80141524296459</v>
-      </c>
-      <c r="L9" s="39" t="n">
-        <v>14.98670735933121</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
EGAT retirement pages update 2026-04-16T04:15:08Z
</commit_message>
<xml_diff>
--- a/EGAT Retirement.xlsx
+++ b/EGAT Retirement.xlsx
@@ -683,7 +683,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I12"/>
+  <dimension ref="A1:I13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1194,6 +1194,47 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>11:15:07</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>EGAT1</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>ตราสารหนี้ (EGAT-1)</t>
+        </is>
+      </c>
+      <c r="F13" t="n">
+        <v>15.75491057164188</v>
+      </c>
+      <c r="G13" t="n">
+        <v>0.5977464518904352</v>
+      </c>
+      <c r="H13" t="n">
+        <v>0.3081397169595324</v>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>https://app.powerbi.com/view?r=eyJrIjoiMzZjYWU3YmQtNWQ1Ny00NjdjLWI1MmEtYjExY2ZiYWIxMzNiIiwidCI6IjVmZWJjNjlmLThlOWMtNDcwOC1iNzBlLWQ4YzYyYmUxODA1YiIsImMiOjEwfQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1205,7 +1246,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I12"/>
+  <dimension ref="A1:I13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1716,6 +1757,47 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>11:15:07</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>EGAT2</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>ตราสารทุน (EGAT-2)</t>
+        </is>
+      </c>
+      <c r="F13" t="n">
+        <v>40.16706991626674</v>
+      </c>
+      <c r="G13" t="n">
+        <v>2.729229382642484</v>
+      </c>
+      <c r="H13" t="n">
+        <v>18.34818846210358</v>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>https://app.powerbi.com/view?r=eyJrIjoiMzZjYWU3YmQtNWQ1Ny00NjdjLWI1MmEtYjExY2ZiYWIxMzNiIiwidCI6IjVmZWJjNjlmLThlOWMtNDcwOC1iNzBlLWQ4YzYyYmUxODA1YiIsImMiOjEwfQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1727,7 +1809,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I12"/>
+  <dimension ref="A1:I13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -2238,6 +2320,47 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>11:15:07</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>EGAT3</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>อสังหาริมทรัพย์และโครงสร้างพื้นฐาน (EGAT-3)</t>
+        </is>
+      </c>
+      <c r="F13" t="n">
+        <v>8.64882939326854</v>
+      </c>
+      <c r="G13" t="n">
+        <v>2.784019436462515</v>
+      </c>
+      <c r="H13" t="n">
+        <v>-0.03242462288043368</v>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>https://app.powerbi.com/view?r=eyJrIjoiMzZjYWU3YmQtNWQ1Ny00NjdjLWI1MmEtYjExY2ZiYWIxMzNiIiwidCI6IjVmZWJjNjlmLThlOWMtNDcwOC1iNzBlLWQ4YzYyYmUxODA1YiIsImMiOjEwfQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2249,7 +2372,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I12"/>
+  <dimension ref="A1:I13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -2760,6 +2883,47 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>11:15:07</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>EGAT4</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>ตราสารทุนต่างประเทศ (EGAT-4)</t>
+        </is>
+      </c>
+      <c r="F13" t="n">
+        <v>7.208836469285037</v>
+      </c>
+      <c r="G13" t="n">
+        <v>6.320304326106552</v>
+      </c>
+      <c r="H13" t="n">
+        <v>-0.08536240871025447</v>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>https://app.powerbi.com/view?r=eyJrIjoiMzZjYWU3YmQtNWQ1Ny00NjdjLWI1MmEtYjExY2ZiYWIxMzNiIiwidCI6IjVmZWJjNjlmLThlOWMtNDcwOC1iNzBlLWQ4YzYyYmUxODA1YiIsImMiOjEwfQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2771,7 +2935,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I12"/>
+  <dimension ref="A1:I13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -3282,6 +3446,47 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>11:15:07</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>EGAT5</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>ตราสารทุนต่างประเทศแบบอิงดัชนี (EGAT-5)</t>
+        </is>
+      </c>
+      <c r="F13" t="n">
+        <v>15.45892475383101</v>
+      </c>
+      <c r="G13" t="n">
+        <v>6.419101037676511</v>
+      </c>
+      <c r="H13" t="n">
+        <v>1.678283928945601</v>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>https://app.powerbi.com/view?r=eyJrIjoiMzZjYWU3YmQtNWQ1Ny00NjdjLWI1MmEtYjExY2ZiYWIxMzNiIiwidCI6IjVmZWJjNjlmLThlOWMtNDcwOC1iNzBlLWQ4YzYyYmUxODA1YiIsImMiOjEwfQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3293,7 +3498,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I12"/>
+  <dimension ref="A1:I13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -3799,6 +4004,47 @@
         <v>16.49521729558234</v>
       </c>
       <c r="I12" t="inlineStr">
+        <is>
+          <t>https://app.powerbi.com/view?r=eyJrIjoiMzZjYWU3YmQtNWQ1Ny00NjdjLWI1MmEtYjExY2ZiYWIxMzNiIiwidCI6IjVmZWJjNjlmLThlOWMtNDcwOC1iNzBlLWQ4YzYyYmUxODA1YiIsImMiOjEwfQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>11:15:07</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>EGAT6</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>การลงทุนตามหลักศาสนาอิสลาม (EGAT-6)</t>
+        </is>
+      </c>
+      <c r="F13" t="n">
+        <v>11.61532101888666</v>
+      </c>
+      <c r="G13" t="n">
+        <v>2.398890039628521</v>
+      </c>
+      <c r="H13" t="n">
+        <v>17.74511202907099</v>
+      </c>
+      <c r="I13" t="inlineStr">
         <is>
           <t>https://app.powerbi.com/view?r=eyJrIjoiMzZjYWU3YmQtNWQ1Ny00NjdjLWI1MmEtYjExY2ZiYWIxMzNiIiwidCI6IjVmZWJjNjlmLThlOWMtNDcwOC1iNzBlLWQ4YzYyYmUxODA1YiIsImMiOjEwfQ%3D%3D</t>
         </is>
@@ -4351,10 +4597,10 @@
         </is>
       </c>
       <c r="B10" s="35" t="n">
-        <v>5.047530370855659</v>
+        <v>5.047530370855658</v>
       </c>
       <c r="C10" s="35" t="n">
-        <v>0.5008204113823886</v>
+        <v>0.5008204113823878</v>
       </c>
       <c r="D10" s="35" t="n">
         <v>0.3247471759871168</v>
@@ -4369,7 +4615,7 @@
         <v>18.2803381153805</v>
       </c>
       <c r="H10" s="35" t="n">
-        <v>1.970648465464841</v>
+        <v>1.970648465464837</v>
       </c>
       <c r="I10" s="19" t="n">
         <v>40.14404168359091</v>
@@ -4387,7 +4633,7 @@
         <v>-3.238432914175438</v>
       </c>
       <c r="N10" s="36" t="n">
-        <v>-0.6282594637754824</v>
+        <v>-0.6282594637754828</v>
       </c>
       <c r="O10" s="19" t="n">
         <v>6.981342578519967</v>
@@ -4396,7 +4642,7 @@
         <v>-1.540562000528767</v>
       </c>
       <c r="Q10" s="36" t="n">
-        <v>-0.7707860812448897</v>
+        <v>-0.7707860812448899</v>
       </c>
       <c r="R10" s="19" t="n">
         <v>14.96953906501773</v>
@@ -4405,7 +4651,7 @@
         <v>16.49521729558234</v>
       </c>
       <c r="T10" s="35" t="n">
-        <v>0.6724871101093424</v>
+        <v>0.6724871101093388</v>
       </c>
       <c r="U10" s="19" t="n">
         <v>11.49202139040016</v>
@@ -4417,26 +4663,66 @@
           <t>9/4/69</t>
         </is>
       </c>
-      <c r="B11" s="33" t="n"/>
-      <c r="C11" s="33" t="n"/>
-      <c r="D11" s="33" t="n"/>
-      <c r="E11" s="33" t="n"/>
-      <c r="F11" s="12" t="n"/>
-      <c r="G11" s="33" t="n"/>
-      <c r="H11" s="33" t="n"/>
-      <c r="I11" s="12" t="n"/>
-      <c r="J11" s="33" t="n"/>
-      <c r="K11" s="33" t="n"/>
-      <c r="L11" s="12" t="n"/>
-      <c r="M11" s="33" t="n"/>
-      <c r="N11" s="33" t="n"/>
-      <c r="O11" s="12" t="n"/>
-      <c r="P11" s="33" t="n"/>
-      <c r="Q11" s="33" t="n"/>
-      <c r="R11" s="12" t="n"/>
-      <c r="S11" s="33" t="n"/>
-      <c r="T11" s="33" t="n"/>
-      <c r="U11" s="12" t="n"/>
+      <c r="B11" s="35" t="n">
+        <v>6.326989517581501</v>
+      </c>
+      <c r="C11" s="35" t="n">
+        <v>1.279459146725843</v>
+      </c>
+      <c r="D11" s="35" t="n">
+        <v>0.3081397169595324</v>
+      </c>
+      <c r="E11" s="36" t="n">
+        <v>-0.01660745902758443</v>
+      </c>
+      <c r="F11" s="19" t="n">
+        <v>15.75491057164188</v>
+      </c>
+      <c r="G11" s="35" t="n">
+        <v>18.34818846210358</v>
+      </c>
+      <c r="H11" s="35" t="n">
+        <v>0.06785034672307688</v>
+      </c>
+      <c r="I11" s="19" t="n">
+        <v>40.16706991626674</v>
+      </c>
+      <c r="J11" s="36" t="n">
+        <v>-0.03242462288043368</v>
+      </c>
+      <c r="K11" s="35" t="n">
+        <v>0.003700824231367417</v>
+      </c>
+      <c r="L11" s="19" t="n">
+        <v>8.64882939326854</v>
+      </c>
+      <c r="M11" s="36" t="n">
+        <v>-0.08536240871025447</v>
+      </c>
+      <c r="N11" s="35" t="n">
+        <v>3.153070505465184</v>
+      </c>
+      <c r="O11" s="19" t="n">
+        <v>7.208836469285037</v>
+      </c>
+      <c r="P11" s="35" t="n">
+        <v>1.678283928945601</v>
+      </c>
+      <c r="Q11" s="35" t="n">
+        <v>3.218845929474368</v>
+      </c>
+      <c r="R11" s="19" t="n">
+        <v>15.45892475383101</v>
+      </c>
+      <c r="S11" s="35" t="n">
+        <v>17.74511202907099</v>
+      </c>
+      <c r="T11" s="35" t="n">
+        <v>1.249894733488649</v>
+      </c>
+      <c r="U11" s="19" t="n">
+        <v>11.61532101888666</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="10" t="inlineStr">
@@ -5052,14 +5338,14 @@
       </c>
       <c r="B1" s="4" t="inlineStr">
         <is>
-          <t>8 เม.ย. 69 (พุธ)</t>
+          <t>9 เม.ย. 69 (พฤหัส)</t>
         </is>
       </c>
       <c r="C1" s="20" t="n"/>
       <c r="D1" s="20" t="n"/>
       <c r="E1" s="21" t="inlineStr">
         <is>
-          <t>7 เม.ย. 69 (อังคาร)</t>
+          <t>8 เม.ย. 69 (พุธ)</t>
         </is>
       </c>
       <c r="F1" s="20" t="n"/>
@@ -5122,27 +5408,27 @@
       <c r="G3" s="20" t="n"/>
       <c r="H3" s="22" t="inlineStr">
         <is>
+          <t>9/4/69</t>
+        </is>
+      </c>
+      <c r="I3" s="22" t="inlineStr">
+        <is>
           <t>8/4/69</t>
         </is>
       </c>
-      <c r="I3" s="22" t="inlineStr">
+      <c r="J3" s="22" t="inlineStr">
         <is>
           <t>7/4/69</t>
         </is>
       </c>
-      <c r="J3" s="22" t="inlineStr">
+      <c r="K3" s="22" t="inlineStr">
         <is>
           <t>3/4/69</t>
         </is>
       </c>
-      <c r="K3" s="22" t="inlineStr">
+      <c r="L3" s="22" t="inlineStr">
         <is>
           <t>2/4/69</t>
-        </is>
-      </c>
-      <c r="L3" s="22" t="inlineStr">
-        <is>
-          <t>1/4/69</t>
         </is>
       </c>
     </row>
@@ -5153,37 +5439,37 @@
         </is>
       </c>
       <c r="B4" s="39" t="n">
+        <v>0.3081397169595324</v>
+      </c>
+      <c r="C4" s="37" t="n">
+        <v>-0.01660745902758443</v>
+      </c>
+      <c r="D4" s="26" t="n">
+        <v>15.75491057164188</v>
+      </c>
+      <c r="E4" s="39" t="n">
         <v>0.3247471759871168</v>
       </c>
-      <c r="C4" s="39" t="n">
+      <c r="F4" s="39" t="n">
         <v>0.1658337901541352</v>
       </c>
-      <c r="D4" s="26" t="n">
+      <c r="G4" s="26" t="n">
         <v>15.75751902428132</v>
       </c>
-      <c r="E4" s="39" t="n">
+      <c r="H4" s="39" t="n">
+        <v>0.3081397169595324</v>
+      </c>
+      <c r="I4" s="39" t="n">
+        <v>0.3247471759871168</v>
+      </c>
+      <c r="J4" s="39" t="n">
         <v>0.1589133858329816</v>
       </c>
-      <c r="F4" s="39" t="n">
-        <v>0.03380454313506298</v>
-      </c>
-      <c r="G4" s="26" t="n">
-        <v>15.73147231918833</v>
-      </c>
-      <c r="H4" s="39" t="n">
-        <v>0.3247471759871168</v>
-      </c>
-      <c r="I4" s="39" t="n">
-        <v>0.1589133858329816</v>
-      </c>
-      <c r="J4" s="39" t="n">
+      <c r="K4" s="39" t="n">
         <v>0.1251088426979186</v>
       </c>
-      <c r="K4" s="39" t="n">
+      <c r="L4" s="39" t="n">
         <v>0.08882055224737062</v>
-      </c>
-      <c r="L4" s="39" t="n">
-        <v>0.1476099448940227</v>
       </c>
     </row>
     <row r="5">
@@ -5193,37 +5479,37 @@
         </is>
       </c>
       <c r="B5" s="39" t="n">
+        <v>18.34818846210358</v>
+      </c>
+      <c r="C5" s="39" t="n">
+        <v>0.06785034672307688</v>
+      </c>
+      <c r="D5" s="26" t="n">
+        <v>40.16706991626674</v>
+      </c>
+      <c r="E5" s="39" t="n">
         <v>18.2803381153805</v>
       </c>
-      <c r="C5" s="39" t="n">
-        <v>1.970648465464841</v>
-      </c>
-      <c r="D5" s="26" t="n">
+      <c r="F5" s="39" t="n">
+        <v>1.970648465464837</v>
+      </c>
+      <c r="G5" s="26" t="n">
         <v>40.14404168359091</v>
       </c>
-      <c r="E5" s="39" t="n">
+      <c r="H5" s="39" t="n">
+        <v>18.34818846210358</v>
+      </c>
+      <c r="I5" s="39" t="n">
+        <v>18.2803381153805</v>
+      </c>
+      <c r="J5" s="39" t="n">
         <v>16.30968964991566</v>
       </c>
-      <c r="F5" s="39" t="n">
-        <v>0.7032511058611615</v>
-      </c>
-      <c r="G5" s="26" t="n">
-        <v>39.47520867717733</v>
-      </c>
-      <c r="H5" s="39" t="n">
-        <v>18.2803381153805</v>
-      </c>
-      <c r="I5" s="39" t="n">
-        <v>16.30968964991566</v>
-      </c>
-      <c r="J5" s="39" t="n">
+      <c r="K5" s="39" t="n">
         <v>15.6064385440545</v>
       </c>
-      <c r="K5" s="39" t="n">
+      <c r="L5" s="39" t="n">
         <v>16.52871682662138</v>
-      </c>
-      <c r="L5" s="39" t="n">
-        <v>16.99575758285332</v>
       </c>
     </row>
     <row r="6">
@@ -5233,37 +5519,37 @@
         </is>
       </c>
       <c r="B6" s="37" t="n">
+        <v>-0.03242462288043368</v>
+      </c>
+      <c r="C6" s="39" t="n">
+        <v>0.003700824231367417</v>
+      </c>
+      <c r="D6" s="26" t="n">
+        <v>8.64882939326854</v>
+      </c>
+      <c r="E6" s="37" t="n">
         <v>-0.0361254471118011</v>
       </c>
-      <c r="C6" s="39" t="n">
+      <c r="F6" s="39" t="n">
         <v>1.594998647586388</v>
       </c>
-      <c r="D6" s="26" t="n">
+      <c r="G6" s="26" t="n">
         <v>8.648509211476886</v>
       </c>
-      <c r="E6" s="37" t="n">
+      <c r="H6" s="37" t="n">
+        <v>-0.03242462288043368</v>
+      </c>
+      <c r="I6" s="37" t="n">
+        <v>-0.0361254471118011</v>
+      </c>
+      <c r="J6" s="37" t="n">
         <v>-1.631124094698189</v>
       </c>
-      <c r="F6" s="39" t="n">
-        <v>0.07436556304149988</v>
-      </c>
-      <c r="G6" s="26" t="n">
-        <v>8.510515755764585</v>
-      </c>
-      <c r="H6" s="37" t="n">
-        <v>-0.0361254471118011</v>
-      </c>
-      <c r="I6" s="37" t="n">
-        <v>-1.631124094698189</v>
-      </c>
-      <c r="J6" s="37" t="n">
+      <c r="K6" s="37" t="n">
         <v>-1.705489657739689</v>
       </c>
-      <c r="K6" s="37" t="n">
+      <c r="L6" s="37" t="n">
         <v>-1.506933806304867</v>
-      </c>
-      <c r="L6" s="37" t="n">
-        <v>-1.895078049485888</v>
       </c>
     </row>
     <row r="7">
@@ -5273,37 +5559,37 @@
         </is>
       </c>
       <c r="B7" s="37" t="n">
+        <v>-0.08536240871025447</v>
+      </c>
+      <c r="C7" s="39" t="n">
+        <v>3.153070505465184</v>
+      </c>
+      <c r="D7" s="26" t="n">
+        <v>7.208836469285037</v>
+      </c>
+      <c r="E7" s="37" t="n">
         <v>-3.238432914175438</v>
       </c>
-      <c r="C7" s="37" t="n">
-        <v>-0.6282594637754824</v>
-      </c>
-      <c r="D7" s="26" t="n">
+      <c r="F7" s="37" t="n">
+        <v>-0.6282594637754828</v>
+      </c>
+      <c r="G7" s="26" t="n">
         <v>6.981342578519967</v>
       </c>
-      <c r="E7" s="37" t="n">
+      <c r="H7" s="37" t="n">
+        <v>-0.08536240871025447</v>
+      </c>
+      <c r="I7" s="37" t="n">
+        <v>-3.238432914175438</v>
+      </c>
+      <c r="J7" s="37" t="n">
         <v>-2.610173450399955</v>
       </c>
-      <c r="F7" s="39" t="n">
-        <v>0.1877609803729747</v>
-      </c>
-      <c r="G7" s="26" t="n">
-        <v>7.026671469699702</v>
-      </c>
-      <c r="H7" s="37" t="n">
-        <v>-3.238432914175438</v>
-      </c>
-      <c r="I7" s="37" t="n">
-        <v>-2.610173450399955</v>
-      </c>
-      <c r="J7" s="37" t="n">
+      <c r="K7" s="37" t="n">
         <v>-2.79793443077293</v>
       </c>
-      <c r="K7" s="37" t="n">
+      <c r="L7" s="37" t="n">
         <v>-2.522818607075272</v>
-      </c>
-      <c r="L7" s="37" t="n">
-        <v>-3.72853648825644</v>
       </c>
     </row>
     <row r="8">
@@ -5312,38 +5598,38 @@
           <t>ตราสารทุนต่างประเทศแบบอิงดัชนี (E5)</t>
         </is>
       </c>
-      <c r="B8" s="37" t="n">
+      <c r="B8" s="39" t="n">
+        <v>1.678283928945601</v>
+      </c>
+      <c r="C8" s="39" t="n">
+        <v>3.218845929474368</v>
+      </c>
+      <c r="D8" s="26" t="n">
+        <v>15.45892475383101</v>
+      </c>
+      <c r="E8" s="37" t="n">
         <v>-1.540562000528767</v>
       </c>
-      <c r="C8" s="37" t="n">
-        <v>-0.7707860812448897</v>
-      </c>
-      <c r="D8" s="26" t="n">
+      <c r="F8" s="37" t="n">
+        <v>-0.7707860812448899</v>
+      </c>
+      <c r="G8" s="26" t="n">
         <v>14.96953906501773</v>
       </c>
-      <c r="E8" s="37" t="n">
+      <c r="H8" s="39" t="n">
+        <v>1.678283928945601</v>
+      </c>
+      <c r="I8" s="37" t="n">
+        <v>-1.540562000528767</v>
+      </c>
+      <c r="J8" s="37" t="n">
         <v>-0.7697759192838771</v>
       </c>
-      <c r="F8" s="39" t="n">
-        <v>0.06402741524638156</v>
-      </c>
-      <c r="G8" s="26" t="n">
-        <v>15.08672754982331</v>
-      </c>
-      <c r="H8" s="37" t="n">
-        <v>-1.540562000528767</v>
-      </c>
-      <c r="I8" s="37" t="n">
-        <v>-0.7697759192838771</v>
-      </c>
-      <c r="J8" s="37" t="n">
+      <c r="K8" s="37" t="n">
         <v>-0.8338033345302587</v>
       </c>
-      <c r="K8" s="37" t="n">
+      <c r="L8" s="37" t="n">
         <v>-0.7534985903937974</v>
-      </c>
-      <c r="L8" s="37" t="n">
-        <v>-1.878349316711203</v>
       </c>
     </row>
     <row r="9">
@@ -5353,37 +5639,37 @@
         </is>
       </c>
       <c r="B9" s="39" t="n">
+        <v>17.74511202907099</v>
+      </c>
+      <c r="C9" s="39" t="n">
+        <v>1.249894733488649</v>
+      </c>
+      <c r="D9" s="26" t="n">
+        <v>11.61532101888666</v>
+      </c>
+      <c r="E9" s="39" t="n">
         <v>16.49521729558234</v>
       </c>
-      <c r="C9" s="39" t="n">
-        <v>0.6724871101093424</v>
-      </c>
-      <c r="D9" s="26" t="n">
+      <c r="F9" s="39" t="n">
+        <v>0.6724871101093388</v>
+      </c>
+      <c r="G9" s="26" t="n">
         <v>11.49202139040016</v>
       </c>
-      <c r="E9" s="39" t="n">
+      <c r="H9" s="39" t="n">
+        <v>17.74511202907099</v>
+      </c>
+      <c r="I9" s="39" t="n">
+        <v>16.49521729558234</v>
+      </c>
+      <c r="J9" s="39" t="n">
         <v>15.822730185473</v>
       </c>
-      <c r="F9" s="39" t="n">
-        <v>1.09545465845069</v>
-      </c>
-      <c r="G9" s="26" t="n">
-        <v>11.42568187506592</v>
-      </c>
-      <c r="H9" s="39" t="n">
-        <v>16.49521729558234</v>
-      </c>
-      <c r="I9" s="39" t="n">
-        <v>15.822730185473</v>
-      </c>
-      <c r="J9" s="39" t="n">
+      <c r="K9" s="39" t="n">
         <v>14.72727552702231</v>
       </c>
-      <c r="K9" s="39" t="n">
+      <c r="L9" s="39" t="n">
         <v>15.75796772875646</v>
-      </c>
-      <c r="L9" s="39" t="n">
-        <v>15.80141524296459</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
EGAT retirement pages update 2026-04-17T04:15:09Z
</commit_message>
<xml_diff>
--- a/EGAT Retirement.xlsx
+++ b/EGAT Retirement.xlsx
@@ -683,7 +683,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I13"/>
+  <dimension ref="A1:I14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1235,6 +1235,47 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>11:15:09</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>EGAT1</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>ตราสารหนี้ (EGAT-1)</t>
+        </is>
+      </c>
+      <c r="F14" t="n">
+        <v>15.75456181105879</v>
+      </c>
+      <c r="G14" t="n">
+        <v>0.595519557072377</v>
+      </c>
+      <c r="H14" t="n">
+        <v>0.3059192330578275</v>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>https://app.powerbi.com/view?r=eyJrIjoiMzZjYWU3YmQtNWQ1Ny00NjdjLWI1MmEtYjExY2ZiYWIxMzNiIiwidCI6IjVmZWJjNjlmLThlOWMtNDcwOC1iNzBlLWQ4YzYyYmUxODA1YiIsImMiOjEwfQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1246,7 +1287,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I13"/>
+  <dimension ref="A1:I14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1798,6 +1839,47 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>11:15:09</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>EGAT2</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>ตราสารทุน (EGAT-2)</t>
+        </is>
+      </c>
+      <c r="F14" t="n">
+        <v>40.61124847791206</v>
+      </c>
+      <c r="G14" t="n">
+        <v>3.8652375963667</v>
+      </c>
+      <c r="H14" t="n">
+        <v>19.65691544253829</v>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>https://app.powerbi.com/view?r=eyJrIjoiMzZjYWU3YmQtNWQ1Ny00NjdjLWI1MmEtYjExY2ZiYWIxMzNiIiwidCI6IjVmZWJjNjlmLThlOWMtNDcwOC1iNzBlLWQ4YzYyYmUxODA1YiIsImMiOjEwfQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1809,7 +1891,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I13"/>
+  <dimension ref="A1:I14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -2361,6 +2443,47 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>11:15:09</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>EGAT3</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>อสังหาริมทรัพย์และโครงสร้างพื้นฐาน (EGAT-3)</t>
+        </is>
+      </c>
+      <c r="F14" t="n">
+        <v>8.665765484051152</v>
+      </c>
+      <c r="G14" t="n">
+        <v>2.985290545536823</v>
+      </c>
+      <c r="H14" t="n">
+        <v>0.1633313407210846</v>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>https://app.powerbi.com/view?r=eyJrIjoiMzZjYWU3YmQtNWQ1Ny00NjdjLWI1MmEtYjExY2ZiYWIxMzNiIiwidCI6IjVmZWJjNjlmLThlOWMtNDcwOC1iNzBlLWQ4YzYyYmUxODA1YiIsImMiOjEwfQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2372,7 +2495,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I13"/>
+  <dimension ref="A1:I14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -2924,6 +3047,47 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>11:15:09</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>EGAT4</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>ตราสารทุนต่างประเทศ (EGAT-4)</t>
+        </is>
+      </c>
+      <c r="F14" t="n">
+        <v>7.24476210014947</v>
+      </c>
+      <c r="G14" t="n">
+        <v>6.850157378383193</v>
+      </c>
+      <c r="H14" t="n">
+        <v>0.4125676530066569</v>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>https://app.powerbi.com/view?r=eyJrIjoiMzZjYWU3YmQtNWQ1Ny00NjdjLWI1MmEtYjExY2ZiYWIxMzNiIiwidCI6IjVmZWJjNjlmLThlOWMtNDcwOC1iNzBlLWQ4YzYyYmUxODA1YiIsImMiOjEwfQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2935,7 +3099,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I13"/>
+  <dimension ref="A1:I14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -3487,6 +3651,47 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>11:15:09</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>EGAT5</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>ตราสารทุนต่างประเทศแบบอิงดัชนี (EGAT-5)</t>
+        </is>
+      </c>
+      <c r="F14" t="n">
+        <v>15.54267216853362</v>
+      </c>
+      <c r="G14" t="n">
+        <v>6.995617498478457</v>
+      </c>
+      <c r="H14" t="n">
+        <v>2.229117414847503</v>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>https://app.powerbi.com/view?r=eyJrIjoiMzZjYWU3YmQtNWQ1Ny00NjdjLWI1MmEtYjExY2ZiYWIxMzNiIiwidCI6IjVmZWJjNjlmLThlOWMtNDcwOC1iNzBlLWQ4YzYyYmUxODA1YiIsImMiOjEwfQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3498,7 +3703,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I13"/>
+  <dimension ref="A1:I14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -4045,6 +4250,47 @@
         <v>17.74511202907099</v>
       </c>
       <c r="I13" t="inlineStr">
+        <is>
+          <t>https://app.powerbi.com/view?r=eyJrIjoiMzZjYWU3YmQtNWQ1Ny00NjdjLWI1MmEtYjExY2ZiYWIxMzNiIiwidCI6IjVmZWJjNjlmLThlOWMtNDcwOC1iNzBlLWQ4YzYyYmUxODA1YiIsImMiOjEwfQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>11:15:09</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>EGAT6</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>การลงทุนตามหลักศาสนาอิสลาม (EGAT-6)</t>
+        </is>
+      </c>
+      <c r="F14" t="n">
+        <v>11.78660841528292</v>
+      </c>
+      <c r="G14" t="n">
+        <v>3.908933476244303</v>
+      </c>
+      <c r="H14" t="n">
+        <v>19.48146125653116</v>
+      </c>
+      <c r="I14" t="inlineStr">
         <is>
           <t>https://app.powerbi.com/view?r=eyJrIjoiMzZjYWU3YmQtNWQ1Ny00NjdjLWI1MmEtYjExY2ZiYWIxMzNiIiwidCI6IjVmZWJjNjlmLThlOWMtNDcwOC1iNzBlLWQ4YzYyYmUxODA1YiIsImMiOjEwfQ%3D%3D</t>
         </is>
@@ -4664,16 +4910,16 @@
         </is>
       </c>
       <c r="B11" s="35" t="n">
-        <v>6.326989517581501</v>
+        <v>6.326989517581502</v>
       </c>
       <c r="C11" s="35" t="n">
-        <v>1.279459146725843</v>
+        <v>1.279459146725844</v>
       </c>
       <c r="D11" s="35" t="n">
         <v>0.3081397169595324</v>
       </c>
       <c r="E11" s="36" t="n">
-        <v>-0.01660745902758443</v>
+        <v>-0.01660745902758437</v>
       </c>
       <c r="F11" s="19" t="n">
         <v>15.75491057164188</v>
@@ -4682,7 +4928,7 @@
         <v>18.34818846210358</v>
       </c>
       <c r="H11" s="35" t="n">
-        <v>0.06785034672307688</v>
+        <v>0.06785034672308043</v>
       </c>
       <c r="I11" s="19" t="n">
         <v>40.16706991626674</v>
@@ -4691,7 +4937,7 @@
         <v>-0.03242462288043368</v>
       </c>
       <c r="K11" s="35" t="n">
-        <v>0.003700824231367417</v>
+        <v>0.003700824231367424</v>
       </c>
       <c r="L11" s="19" t="n">
         <v>8.64882939326854</v>
@@ -4718,7 +4964,7 @@
         <v>17.74511202907099</v>
       </c>
       <c r="T11" s="35" t="n">
-        <v>1.249894733488649</v>
+        <v>1.249894733488652</v>
       </c>
       <c r="U11" s="19" t="n">
         <v>11.61532101888666</v>
@@ -4730,26 +4976,66 @@
           <t>10/4/69</t>
         </is>
       </c>
-      <c r="B12" s="33" t="n"/>
-      <c r="C12" s="33" t="n"/>
-      <c r="D12" s="33" t="n"/>
-      <c r="E12" s="33" t="n"/>
-      <c r="F12" s="12" t="n"/>
-      <c r="G12" s="33" t="n"/>
-      <c r="H12" s="33" t="n"/>
-      <c r="I12" s="12" t="n"/>
-      <c r="J12" s="33" t="n"/>
-      <c r="K12" s="33" t="n"/>
-      <c r="L12" s="12" t="n"/>
-      <c r="M12" s="33" t="n"/>
-      <c r="N12" s="33" t="n"/>
-      <c r="O12" s="12" t="n"/>
-      <c r="P12" s="33" t="n"/>
-      <c r="Q12" s="33" t="n"/>
-      <c r="R12" s="12" t="n"/>
-      <c r="S12" s="33" t="n"/>
-      <c r="T12" s="33" t="n"/>
-      <c r="U12" s="12" t="n"/>
+      <c r="B12" s="35" t="n">
+        <v>7.041552056783754</v>
+      </c>
+      <c r="C12" s="35" t="n">
+        <v>0.7145625392022517</v>
+      </c>
+      <c r="D12" s="35" t="n">
+        <v>0.3059192330578275</v>
+      </c>
+      <c r="E12" s="36" t="n">
+        <v>-0.002220483901704873</v>
+      </c>
+      <c r="F12" s="19" t="n">
+        <v>15.75456181105879</v>
+      </c>
+      <c r="G12" s="35" t="n">
+        <v>19.65691544253829</v>
+      </c>
+      <c r="H12" s="35" t="n">
+        <v>1.308726980434713</v>
+      </c>
+      <c r="I12" s="19" t="n">
+        <v>40.61124847791206</v>
+      </c>
+      <c r="J12" s="35" t="n">
+        <v>0.1633313407210846</v>
+      </c>
+      <c r="K12" s="35" t="n">
+        <v>0.1957559636015183</v>
+      </c>
+      <c r="L12" s="19" t="n">
+        <v>8.665765484051152</v>
+      </c>
+      <c r="M12" s="35" t="n">
+        <v>0.4125676530066569</v>
+      </c>
+      <c r="N12" s="35" t="n">
+        <v>0.4979300617169113</v>
+      </c>
+      <c r="O12" s="19" t="n">
+        <v>7.24476210014947</v>
+      </c>
+      <c r="P12" s="35" t="n">
+        <v>2.229117414847503</v>
+      </c>
+      <c r="Q12" s="35" t="n">
+        <v>0.5508334859019024</v>
+      </c>
+      <c r="R12" s="19" t="n">
+        <v>15.54267216853362</v>
+      </c>
+      <c r="S12" s="35" t="n">
+        <v>19.48146125653116</v>
+      </c>
+      <c r="T12" s="35" t="n">
+        <v>1.73634922746017</v>
+      </c>
+      <c r="U12" s="19" t="n">
+        <v>11.78660841528292</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="13" t="inlineStr">
@@ -5338,14 +5624,14 @@
       </c>
       <c r="B1" s="4" t="inlineStr">
         <is>
-          <t>9 เม.ย. 69 (พฤหัส)</t>
+          <t>10 เม.ย. 69 (ศุกร์)</t>
         </is>
       </c>
       <c r="C1" s="20" t="n"/>
       <c r="D1" s="20" t="n"/>
       <c r="E1" s="21" t="inlineStr">
         <is>
-          <t>8 เม.ย. 69 (พุธ)</t>
+          <t>9 เม.ย. 69 (พฤหัส)</t>
         </is>
       </c>
       <c r="F1" s="20" t="n"/>
@@ -5408,27 +5694,27 @@
       <c r="G3" s="20" t="n"/>
       <c r="H3" s="22" t="inlineStr">
         <is>
+          <t>10/4/69</t>
+        </is>
+      </c>
+      <c r="I3" s="22" t="inlineStr">
+        <is>
           <t>9/4/69</t>
         </is>
       </c>
-      <c r="I3" s="22" t="inlineStr">
+      <c r="J3" s="22" t="inlineStr">
         <is>
           <t>8/4/69</t>
         </is>
       </c>
-      <c r="J3" s="22" t="inlineStr">
+      <c r="K3" s="22" t="inlineStr">
         <is>
           <t>7/4/69</t>
         </is>
       </c>
-      <c r="K3" s="22" t="inlineStr">
+      <c r="L3" s="22" t="inlineStr">
         <is>
           <t>3/4/69</t>
-        </is>
-      </c>
-      <c r="L3" s="22" t="inlineStr">
-        <is>
-          <t>2/4/69</t>
         </is>
       </c>
     </row>
@@ -5439,37 +5725,37 @@
         </is>
       </c>
       <c r="B4" s="39" t="n">
+        <v>0.3059192330578275</v>
+      </c>
+      <c r="C4" s="37" t="n">
+        <v>-0.002220483901704873</v>
+      </c>
+      <c r="D4" s="26" t="n">
+        <v>15.75456181105879</v>
+      </c>
+      <c r="E4" s="39" t="n">
         <v>0.3081397169595324</v>
       </c>
-      <c r="C4" s="37" t="n">
-        <v>-0.01660745902758443</v>
-      </c>
-      <c r="D4" s="26" t="n">
+      <c r="F4" s="37" t="n">
+        <v>-0.01660745902758437</v>
+      </c>
+      <c r="G4" s="26" t="n">
         <v>15.75491057164188</v>
       </c>
-      <c r="E4" s="39" t="n">
+      <c r="H4" s="39" t="n">
+        <v>0.3059192330578275</v>
+      </c>
+      <c r="I4" s="39" t="n">
+        <v>0.3081397169595324</v>
+      </c>
+      <c r="J4" s="39" t="n">
         <v>0.3247471759871168</v>
       </c>
-      <c r="F4" s="39" t="n">
-        <v>0.1658337901541352</v>
-      </c>
-      <c r="G4" s="26" t="n">
-        <v>15.75751902428132</v>
-      </c>
-      <c r="H4" s="39" t="n">
-        <v>0.3081397169595324</v>
-      </c>
-      <c r="I4" s="39" t="n">
-        <v>0.3247471759871168</v>
-      </c>
-      <c r="J4" s="39" t="n">
+      <c r="K4" s="39" t="n">
         <v>0.1589133858329816</v>
       </c>
-      <c r="K4" s="39" t="n">
+      <c r="L4" s="39" t="n">
         <v>0.1251088426979186</v>
-      </c>
-      <c r="L4" s="39" t="n">
-        <v>0.08882055224737062</v>
       </c>
     </row>
     <row r="5">
@@ -5479,37 +5765,37 @@
         </is>
       </c>
       <c r="B5" s="39" t="n">
+        <v>19.65691544253829</v>
+      </c>
+      <c r="C5" s="39" t="n">
+        <v>1.308726980434713</v>
+      </c>
+      <c r="D5" s="26" t="n">
+        <v>40.61124847791206</v>
+      </c>
+      <c r="E5" s="39" t="n">
         <v>18.34818846210358</v>
       </c>
-      <c r="C5" s="39" t="n">
-        <v>0.06785034672307688</v>
-      </c>
-      <c r="D5" s="26" t="n">
+      <c r="F5" s="39" t="n">
+        <v>0.06785034672308043</v>
+      </c>
+      <c r="G5" s="26" t="n">
         <v>40.16706991626674</v>
       </c>
-      <c r="E5" s="39" t="n">
+      <c r="H5" s="39" t="n">
+        <v>19.65691544253829</v>
+      </c>
+      <c r="I5" s="39" t="n">
+        <v>18.34818846210358</v>
+      </c>
+      <c r="J5" s="39" t="n">
         <v>18.2803381153805</v>
       </c>
-      <c r="F5" s="39" t="n">
-        <v>1.970648465464837</v>
-      </c>
-      <c r="G5" s="26" t="n">
-        <v>40.14404168359091</v>
-      </c>
-      <c r="H5" s="39" t="n">
-        <v>18.34818846210358</v>
-      </c>
-      <c r="I5" s="39" t="n">
-        <v>18.2803381153805</v>
-      </c>
-      <c r="J5" s="39" t="n">
+      <c r="K5" s="39" t="n">
         <v>16.30968964991566</v>
       </c>
-      <c r="K5" s="39" t="n">
+      <c r="L5" s="39" t="n">
         <v>15.6064385440545</v>
-      </c>
-      <c r="L5" s="39" t="n">
-        <v>16.52871682662138</v>
       </c>
     </row>
     <row r="6">
@@ -5518,38 +5804,38 @@
           <t>อสังหาริมทรัพย์และโครงสร้างพื้นฐาน (E3)</t>
         </is>
       </c>
-      <c r="B6" s="37" t="n">
+      <c r="B6" s="39" t="n">
+        <v>0.1633313407210846</v>
+      </c>
+      <c r="C6" s="39" t="n">
+        <v>0.1957559636015183</v>
+      </c>
+      <c r="D6" s="26" t="n">
+        <v>8.665765484051152</v>
+      </c>
+      <c r="E6" s="37" t="n">
         <v>-0.03242462288043368</v>
       </c>
-      <c r="C6" s="39" t="n">
-        <v>0.003700824231367417</v>
-      </c>
-      <c r="D6" s="26" t="n">
+      <c r="F6" s="39" t="n">
+        <v>0.003700824231367424</v>
+      </c>
+      <c r="G6" s="26" t="n">
         <v>8.64882939326854</v>
       </c>
-      <c r="E6" s="37" t="n">
+      <c r="H6" s="39" t="n">
+        <v>0.1633313407210846</v>
+      </c>
+      <c r="I6" s="37" t="n">
+        <v>-0.03242462288043368</v>
+      </c>
+      <c r="J6" s="37" t="n">
         <v>-0.0361254471118011</v>
       </c>
-      <c r="F6" s="39" t="n">
-        <v>1.594998647586388</v>
-      </c>
-      <c r="G6" s="26" t="n">
-        <v>8.648509211476886</v>
-      </c>
-      <c r="H6" s="37" t="n">
-        <v>-0.03242462288043368</v>
-      </c>
-      <c r="I6" s="37" t="n">
-        <v>-0.0361254471118011</v>
-      </c>
-      <c r="J6" s="37" t="n">
+      <c r="K6" s="37" t="n">
         <v>-1.631124094698189</v>
       </c>
-      <c r="K6" s="37" t="n">
+      <c r="L6" s="37" t="n">
         <v>-1.705489657739689</v>
-      </c>
-      <c r="L6" s="37" t="n">
-        <v>-1.506933806304867</v>
       </c>
     </row>
     <row r="7">
@@ -5558,38 +5844,38 @@
           <t>ตราสารทุนต่างประเทศ (E4)</t>
         </is>
       </c>
-      <c r="B7" s="37" t="n">
+      <c r="B7" s="39" t="n">
+        <v>0.4125676530066569</v>
+      </c>
+      <c r="C7" s="39" t="n">
+        <v>0.4979300617169113</v>
+      </c>
+      <c r="D7" s="26" t="n">
+        <v>7.24476210014947</v>
+      </c>
+      <c r="E7" s="37" t="n">
         <v>-0.08536240871025447</v>
       </c>
-      <c r="C7" s="39" t="n">
+      <c r="F7" s="39" t="n">
         <v>3.153070505465184</v>
       </c>
-      <c r="D7" s="26" t="n">
+      <c r="G7" s="26" t="n">
         <v>7.208836469285037</v>
       </c>
-      <c r="E7" s="37" t="n">
+      <c r="H7" s="39" t="n">
+        <v>0.4125676530066569</v>
+      </c>
+      <c r="I7" s="37" t="n">
+        <v>-0.08536240871025447</v>
+      </c>
+      <c r="J7" s="37" t="n">
         <v>-3.238432914175438</v>
       </c>
-      <c r="F7" s="37" t="n">
-        <v>-0.6282594637754828</v>
-      </c>
-      <c r="G7" s="26" t="n">
-        <v>6.981342578519967</v>
-      </c>
-      <c r="H7" s="37" t="n">
-        <v>-0.08536240871025447</v>
-      </c>
-      <c r="I7" s="37" t="n">
-        <v>-3.238432914175438</v>
-      </c>
-      <c r="J7" s="37" t="n">
+      <c r="K7" s="37" t="n">
         <v>-2.610173450399955</v>
       </c>
-      <c r="K7" s="37" t="n">
+      <c r="L7" s="37" t="n">
         <v>-2.79793443077293</v>
-      </c>
-      <c r="L7" s="37" t="n">
-        <v>-2.522818607075272</v>
       </c>
     </row>
     <row r="8">
@@ -5599,37 +5885,37 @@
         </is>
       </c>
       <c r="B8" s="39" t="n">
+        <v>2.229117414847503</v>
+      </c>
+      <c r="C8" s="39" t="n">
+        <v>0.5508334859019024</v>
+      </c>
+      <c r="D8" s="26" t="n">
+        <v>15.54267216853362</v>
+      </c>
+      <c r="E8" s="39" t="n">
         <v>1.678283928945601</v>
       </c>
-      <c r="C8" s="39" t="n">
+      <c r="F8" s="39" t="n">
         <v>3.218845929474368</v>
       </c>
-      <c r="D8" s="26" t="n">
+      <c r="G8" s="26" t="n">
         <v>15.45892475383101</v>
       </c>
-      <c r="E8" s="37" t="n">
+      <c r="H8" s="39" t="n">
+        <v>2.229117414847503</v>
+      </c>
+      <c r="I8" s="39" t="n">
+        <v>1.678283928945601</v>
+      </c>
+      <c r="J8" s="37" t="n">
         <v>-1.540562000528767</v>
       </c>
-      <c r="F8" s="37" t="n">
-        <v>-0.7707860812448899</v>
-      </c>
-      <c r="G8" s="26" t="n">
-        <v>14.96953906501773</v>
-      </c>
-      <c r="H8" s="39" t="n">
-        <v>1.678283928945601</v>
-      </c>
-      <c r="I8" s="37" t="n">
-        <v>-1.540562000528767</v>
-      </c>
-      <c r="J8" s="37" t="n">
+      <c r="K8" s="37" t="n">
         <v>-0.7697759192838771</v>
       </c>
-      <c r="K8" s="37" t="n">
+      <c r="L8" s="37" t="n">
         <v>-0.8338033345302587</v>
-      </c>
-      <c r="L8" s="37" t="n">
-        <v>-0.7534985903937974</v>
       </c>
     </row>
     <row r="9">
@@ -5639,37 +5925,37 @@
         </is>
       </c>
       <c r="B9" s="39" t="n">
+        <v>19.48146125653116</v>
+      </c>
+      <c r="C9" s="39" t="n">
+        <v>1.73634922746017</v>
+      </c>
+      <c r="D9" s="26" t="n">
+        <v>11.78660841528292</v>
+      </c>
+      <c r="E9" s="39" t="n">
         <v>17.74511202907099</v>
       </c>
-      <c r="C9" s="39" t="n">
-        <v>1.249894733488649</v>
-      </c>
-      <c r="D9" s="26" t="n">
+      <c r="F9" s="39" t="n">
+        <v>1.249894733488652</v>
+      </c>
+      <c r="G9" s="26" t="n">
         <v>11.61532101888666</v>
       </c>
-      <c r="E9" s="39" t="n">
+      <c r="H9" s="39" t="n">
+        <v>19.48146125653116</v>
+      </c>
+      <c r="I9" s="39" t="n">
+        <v>17.74511202907099</v>
+      </c>
+      <c r="J9" s="39" t="n">
         <v>16.49521729558234</v>
       </c>
-      <c r="F9" s="39" t="n">
-        <v>0.6724871101093388</v>
-      </c>
-      <c r="G9" s="26" t="n">
-        <v>11.49202139040016</v>
-      </c>
-      <c r="H9" s="39" t="n">
-        <v>17.74511202907099</v>
-      </c>
-      <c r="I9" s="39" t="n">
-        <v>16.49521729558234</v>
-      </c>
-      <c r="J9" s="39" t="n">
+      <c r="K9" s="39" t="n">
         <v>15.822730185473</v>
       </c>
-      <c r="K9" s="39" t="n">
+      <c r="L9" s="39" t="n">
         <v>14.72727552702231</v>
-      </c>
-      <c r="L9" s="39" t="n">
-        <v>15.75796772875646</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
EGAT retirement pages update 2026-04-20T04:15:08Z
</commit_message>
<xml_diff>
--- a/EGAT Retirement.xlsx
+++ b/EGAT Retirement.xlsx
@@ -683,7 +683,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I14"/>
+  <dimension ref="A1:I15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1276,6 +1276,47 @@
         </is>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>11:15:08</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>EGAT1</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>ตราสารหนี้ (EGAT-1)</t>
+        </is>
+      </c>
+      <c r="F15" t="n">
+        <v>15.76692605409251</v>
+      </c>
+      <c r="G15" t="n">
+        <v>0.6744673226036557</v>
+      </c>
+      <c r="H15" t="n">
+        <v>0.3846397190981454</v>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>https://app.powerbi.com/view?r=eyJrIjoiMzZjYWU3YmQtNWQ1Ny00NjdjLWI1MmEtYjExY2ZiYWIxMzNiIiwidCI6IjVmZWJjNjlmLThlOWMtNDcwOC1iNzBlLWQ4YzYyYmUxODA1YiIsImMiOjEwfQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1287,7 +1328,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I14"/>
+  <dimension ref="A1:I15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1880,6 +1921,47 @@
         </is>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>11:15:08</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>EGAT2</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>ตราสารทุน (EGAT-2)</t>
+        </is>
+      </c>
+      <c r="F15" t="n">
+        <v>40.28668355491568</v>
+      </c>
+      <c r="G15" t="n">
+        <v>3.035147064655996</v>
+      </c>
+      <c r="H15" t="n">
+        <v>18.70061788946713</v>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>https://app.powerbi.com/view?r=eyJrIjoiMzZjYWU3YmQtNWQ1Ny00NjdjLWI1MmEtYjExY2ZiYWIxMzNiIiwidCI6IjVmZWJjNjlmLThlOWMtNDcwOC1iNzBlLWQ4YzYyYmUxODA1YiIsImMiOjEwfQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1891,7 +1973,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I14"/>
+  <dimension ref="A1:I15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -2484,6 +2566,47 @@
         </is>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>11:15:08</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>EGAT3</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>อสังหาริมทรัพย์และโครงสร้างพื้นฐาน (EGAT-3)</t>
+        </is>
+      </c>
+      <c r="F15" t="n">
+        <v>8.712144740764185</v>
+      </c>
+      <c r="G15" t="n">
+        <v>3.536468769395795</v>
+      </c>
+      <c r="H15" t="n">
+        <v>0.6994064129156596</v>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>https://app.powerbi.com/view?r=eyJrIjoiMzZjYWU3YmQtNWQ1Ny00NjdjLWI1MmEtYjExY2ZiYWIxMzNiIiwidCI6IjVmZWJjNjlmLThlOWMtNDcwOC1iNzBlLWQ4YzYyYmUxODA1YiIsImMiOjEwfQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2495,7 +2618,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I14"/>
+  <dimension ref="A1:I15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -3088,6 +3211,47 @@
         </is>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>11:15:08</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>EGAT4</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>ตราสารทุนต่างประเทศ (EGAT-4)</t>
+        </is>
+      </c>
+      <c r="F15" t="n">
+        <v>7.414424832044875</v>
+      </c>
+      <c r="G15" t="n">
+        <v>9.352446529312864</v>
+      </c>
+      <c r="H15" t="n">
+        <v>2.76409697986888</v>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>https://app.powerbi.com/view?r=eyJrIjoiMzZjYWU3YmQtNWQ1Ny00NjdjLWI1MmEtYjExY2ZiYWIxMzNiIiwidCI6IjVmZWJjNjlmLThlOWMtNDcwOC1iNzBlLWQ4YzYyYmUxODA1YiIsImMiOjEwfQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3099,7 +3263,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I14"/>
+  <dimension ref="A1:I15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -3692,6 +3856,47 @@
         </is>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>11:15:08</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>EGAT5</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>ตราสารทุนต่างประเทศแบบอิงดัชนี (EGAT-5)</t>
+        </is>
+      </c>
+      <c r="F15" t="n">
+        <v>15.86490824291597</v>
+      </c>
+      <c r="G15" t="n">
+        <v>9.213887779481089</v>
+      </c>
+      <c r="H15" t="n">
+        <v>4.348566961626465</v>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>https://app.powerbi.com/view?r=eyJrIjoiMzZjYWU3YmQtNWQ1Ny00NjdjLWI1MmEtYjExY2ZiYWIxMzNiIiwidCI6IjVmZWJjNjlmLThlOWMtNDcwOC1iNzBlLWQ4YzYyYmUxODA1YiIsImMiOjEwfQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3703,7 +3908,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I14"/>
+  <dimension ref="A1:I15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -4291,6 +4496,47 @@
         <v>19.48146125653116</v>
       </c>
       <c r="I14" t="inlineStr">
+        <is>
+          <t>https://app.powerbi.com/view?r=eyJrIjoiMzZjYWU3YmQtNWQ1Ny00NjdjLWI1MmEtYjExY2ZiYWIxMzNiIiwidCI6IjVmZWJjNjlmLThlOWMtNDcwOC1iNzBlLWQ4YzYyYmUxODA1YiIsImMiOjEwfQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>11:15:08</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>EGAT6</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>การลงทุนตามหลักศาสนาอิสลาม (EGAT-6)</t>
+        </is>
+      </c>
+      <c r="F15" t="n">
+        <v>11.60974402225383</v>
+      </c>
+      <c r="G15" t="n">
+        <v>2.349724091995387</v>
+      </c>
+      <c r="H15" t="n">
+        <v>17.68857772474563</v>
+      </c>
+      <c r="I15" t="inlineStr">
         <is>
           <t>https://app.powerbi.com/view?r=eyJrIjoiMzZjYWU3YmQtNWQ1Ny00NjdjLWI1MmEtYjExY2ZiYWIxMzNiIiwidCI6IjVmZWJjNjlmLThlOWMtNDcwOC1iNzBlLWQ4YzYyYmUxODA1YiIsImMiOjEwfQ%3D%3D</t>
         </is>
@@ -4977,16 +5223,16 @@
         </is>
       </c>
       <c r="B12" s="35" t="n">
-        <v>7.041552056783754</v>
+        <v>7.041552056783753</v>
       </c>
       <c r="C12" s="35" t="n">
-        <v>0.7145625392022517</v>
+        <v>0.7145625392022508</v>
       </c>
       <c r="D12" s="35" t="n">
         <v>0.3059192330578275</v>
       </c>
       <c r="E12" s="36" t="n">
-        <v>-0.002220483901704873</v>
+        <v>-0.002220483901704928</v>
       </c>
       <c r="F12" s="19" t="n">
         <v>15.75456181105879</v>
@@ -4995,7 +5241,7 @@
         <v>19.65691544253829</v>
       </c>
       <c r="H12" s="35" t="n">
-        <v>1.308726980434713</v>
+        <v>1.308726980434709</v>
       </c>
       <c r="I12" s="19" t="n">
         <v>40.61124847791206</v>
@@ -5022,7 +5268,7 @@
         <v>2.229117414847503</v>
       </c>
       <c r="Q12" s="35" t="n">
-        <v>0.5508334859019024</v>
+        <v>0.550833485901902</v>
       </c>
       <c r="R12" s="19" t="n">
         <v>15.54267216853362</v>
@@ -5031,7 +5277,7 @@
         <v>19.48146125653116</v>
       </c>
       <c r="T12" s="35" t="n">
-        <v>1.73634922746017</v>
+        <v>1.736349227460167</v>
       </c>
       <c r="U12" s="19" t="n">
         <v>11.78660841528292</v>
@@ -5178,26 +5424,66 @@
           <t>16/4/69</t>
         </is>
       </c>
-      <c r="B18" s="33" t="n"/>
-      <c r="C18" s="33" t="n"/>
-      <c r="D18" s="33" t="n"/>
-      <c r="E18" s="33" t="n"/>
-      <c r="F18" s="12" t="n"/>
-      <c r="G18" s="33" t="n"/>
-      <c r="H18" s="33" t="n"/>
-      <c r="I18" s="12" t="n"/>
-      <c r="J18" s="33" t="n"/>
-      <c r="K18" s="33" t="n"/>
-      <c r="L18" s="12" t="n"/>
-      <c r="M18" s="33" t="n"/>
-      <c r="N18" s="33" t="n"/>
-      <c r="O18" s="12" t="n"/>
-      <c r="P18" s="33" t="n"/>
-      <c r="Q18" s="33" t="n"/>
-      <c r="R18" s="12" t="n"/>
-      <c r="S18" s="33" t="n"/>
-      <c r="T18" s="33" t="n"/>
-      <c r="U18" s="12" t="n"/>
+      <c r="B18" s="35" t="n">
+        <v>7.430984281286986</v>
+      </c>
+      <c r="C18" s="35" t="n">
+        <v>0.3894322245032331</v>
+      </c>
+      <c r="D18" s="35" t="n">
+        <v>0.3846397190981454</v>
+      </c>
+      <c r="E18" s="35" t="n">
+        <v>0.07872048604031795</v>
+      </c>
+      <c r="F18" s="19" t="n">
+        <v>15.76692605409251</v>
+      </c>
+      <c r="G18" s="35" t="n">
+        <v>18.70061788946713</v>
+      </c>
+      <c r="H18" s="36" t="n">
+        <v>-0.9562975530711562</v>
+      </c>
+      <c r="I18" s="19" t="n">
+        <v>40.28668355491568</v>
+      </c>
+      <c r="J18" s="35" t="n">
+        <v>0.6994064129156596</v>
+      </c>
+      <c r="K18" s="35" t="n">
+        <v>0.5360750721945751</v>
+      </c>
+      <c r="L18" s="19" t="n">
+        <v>8.712144740764185</v>
+      </c>
+      <c r="M18" s="35" t="n">
+        <v>2.76409697986888</v>
+      </c>
+      <c r="N18" s="35" t="n">
+        <v>2.351529326862223</v>
+      </c>
+      <c r="O18" s="19" t="n">
+        <v>7.414424832044875</v>
+      </c>
+      <c r="P18" s="35" t="n">
+        <v>4.348566961626465</v>
+      </c>
+      <c r="Q18" s="35" t="n">
+        <v>2.119449546778962</v>
+      </c>
+      <c r="R18" s="19" t="n">
+        <v>15.86490824291597</v>
+      </c>
+      <c r="S18" s="35" t="n">
+        <v>17.68857772474563</v>
+      </c>
+      <c r="T18" s="36" t="n">
+        <v>-1.792883531785524</v>
+      </c>
+      <c r="U18" s="19" t="n">
+        <v>11.60974402225383</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="10" t="inlineStr">
@@ -5624,14 +5910,14 @@
       </c>
       <c r="B1" s="4" t="inlineStr">
         <is>
-          <t>10 เม.ย. 69 (ศุกร์)</t>
+          <t>16 เม.ย. 69 (พฤหัส)</t>
         </is>
       </c>
       <c r="C1" s="20" t="n"/>
       <c r="D1" s="20" t="n"/>
       <c r="E1" s="21" t="inlineStr">
         <is>
-          <t>9 เม.ย. 69 (พฤหัส)</t>
+          <t>10 เม.ย. 69 (ศุกร์)</t>
         </is>
       </c>
       <c r="F1" s="20" t="n"/>
@@ -5694,27 +5980,27 @@
       <c r="G3" s="20" t="n"/>
       <c r="H3" s="22" t="inlineStr">
         <is>
+          <t>16/4/69</t>
+        </is>
+      </c>
+      <c r="I3" s="22" t="inlineStr">
+        <is>
           <t>10/4/69</t>
         </is>
       </c>
-      <c r="I3" s="22" t="inlineStr">
+      <c r="J3" s="22" t="inlineStr">
         <is>
           <t>9/4/69</t>
         </is>
       </c>
-      <c r="J3" s="22" t="inlineStr">
+      <c r="K3" s="22" t="inlineStr">
         <is>
           <t>8/4/69</t>
         </is>
       </c>
-      <c r="K3" s="22" t="inlineStr">
+      <c r="L3" s="22" t="inlineStr">
         <is>
           <t>7/4/69</t>
-        </is>
-      </c>
-      <c r="L3" s="22" t="inlineStr">
-        <is>
-          <t>3/4/69</t>
         </is>
       </c>
     </row>
@@ -5725,37 +6011,37 @@
         </is>
       </c>
       <c r="B4" s="39" t="n">
+        <v>0.3846397190981454</v>
+      </c>
+      <c r="C4" s="39" t="n">
+        <v>0.07872048604031795</v>
+      </c>
+      <c r="D4" s="26" t="n">
+        <v>15.76692605409251</v>
+      </c>
+      <c r="E4" s="39" t="n">
         <v>0.3059192330578275</v>
       </c>
-      <c r="C4" s="37" t="n">
-        <v>-0.002220483901704873</v>
-      </c>
-      <c r="D4" s="26" t="n">
+      <c r="F4" s="37" t="n">
+        <v>-0.002220483901704928</v>
+      </c>
+      <c r="G4" s="26" t="n">
         <v>15.75456181105879</v>
       </c>
-      <c r="E4" s="39" t="n">
+      <c r="H4" s="39" t="n">
+        <v>0.3846397190981454</v>
+      </c>
+      <c r="I4" s="39" t="n">
+        <v>0.3059192330578275</v>
+      </c>
+      <c r="J4" s="39" t="n">
         <v>0.3081397169595324</v>
       </c>
-      <c r="F4" s="37" t="n">
-        <v>-0.01660745902758437</v>
-      </c>
-      <c r="G4" s="26" t="n">
-        <v>15.75491057164188</v>
-      </c>
-      <c r="H4" s="39" t="n">
-        <v>0.3059192330578275</v>
-      </c>
-      <c r="I4" s="39" t="n">
-        <v>0.3081397169595324</v>
-      </c>
-      <c r="J4" s="39" t="n">
+      <c r="K4" s="39" t="n">
         <v>0.3247471759871168</v>
       </c>
-      <c r="K4" s="39" t="n">
+      <c r="L4" s="39" t="n">
         <v>0.1589133858329816</v>
-      </c>
-      <c r="L4" s="39" t="n">
-        <v>0.1251088426979186</v>
       </c>
     </row>
     <row r="5">
@@ -5765,37 +6051,37 @@
         </is>
       </c>
       <c r="B5" s="39" t="n">
+        <v>18.70061788946713</v>
+      </c>
+      <c r="C5" s="37" t="n">
+        <v>-0.9562975530711562</v>
+      </c>
+      <c r="D5" s="26" t="n">
+        <v>40.28668355491568</v>
+      </c>
+      <c r="E5" s="39" t="n">
         <v>19.65691544253829</v>
       </c>
-      <c r="C5" s="39" t="n">
-        <v>1.308726980434713</v>
-      </c>
-      <c r="D5" s="26" t="n">
+      <c r="F5" s="39" t="n">
+        <v>1.308726980434709</v>
+      </c>
+      <c r="G5" s="26" t="n">
         <v>40.61124847791206</v>
       </c>
-      <c r="E5" s="39" t="n">
+      <c r="H5" s="39" t="n">
+        <v>18.70061788946713</v>
+      </c>
+      <c r="I5" s="39" t="n">
+        <v>19.65691544253829</v>
+      </c>
+      <c r="J5" s="39" t="n">
         <v>18.34818846210358</v>
       </c>
-      <c r="F5" s="39" t="n">
-        <v>0.06785034672308043</v>
-      </c>
-      <c r="G5" s="26" t="n">
-        <v>40.16706991626674</v>
-      </c>
-      <c r="H5" s="39" t="n">
-        <v>19.65691544253829</v>
-      </c>
-      <c r="I5" s="39" t="n">
-        <v>18.34818846210358</v>
-      </c>
-      <c r="J5" s="39" t="n">
+      <c r="K5" s="39" t="n">
         <v>18.2803381153805</v>
       </c>
-      <c r="K5" s="39" t="n">
+      <c r="L5" s="39" t="n">
         <v>16.30968964991566</v>
-      </c>
-      <c r="L5" s="39" t="n">
-        <v>15.6064385440545</v>
       </c>
     </row>
     <row r="6">
@@ -5805,37 +6091,37 @@
         </is>
       </c>
       <c r="B6" s="39" t="n">
+        <v>0.6994064129156596</v>
+      </c>
+      <c r="C6" s="39" t="n">
+        <v>0.5360750721945751</v>
+      </c>
+      <c r="D6" s="26" t="n">
+        <v>8.712144740764185</v>
+      </c>
+      <c r="E6" s="39" t="n">
         <v>0.1633313407210846</v>
       </c>
-      <c r="C6" s="39" t="n">
+      <c r="F6" s="39" t="n">
         <v>0.1957559636015183</v>
       </c>
-      <c r="D6" s="26" t="n">
+      <c r="G6" s="26" t="n">
         <v>8.665765484051152</v>
       </c>
-      <c r="E6" s="37" t="n">
+      <c r="H6" s="39" t="n">
+        <v>0.6994064129156596</v>
+      </c>
+      <c r="I6" s="39" t="n">
+        <v>0.1633313407210846</v>
+      </c>
+      <c r="J6" s="37" t="n">
         <v>-0.03242462288043368</v>
       </c>
-      <c r="F6" s="39" t="n">
-        <v>0.003700824231367424</v>
-      </c>
-      <c r="G6" s="26" t="n">
-        <v>8.64882939326854</v>
-      </c>
-      <c r="H6" s="39" t="n">
-        <v>0.1633313407210846</v>
-      </c>
-      <c r="I6" s="37" t="n">
-        <v>-0.03242462288043368</v>
-      </c>
-      <c r="J6" s="37" t="n">
+      <c r="K6" s="37" t="n">
         <v>-0.0361254471118011</v>
       </c>
-      <c r="K6" s="37" t="n">
+      <c r="L6" s="37" t="n">
         <v>-1.631124094698189</v>
-      </c>
-      <c r="L6" s="37" t="n">
-        <v>-1.705489657739689</v>
       </c>
     </row>
     <row r="7">
@@ -5845,37 +6131,37 @@
         </is>
       </c>
       <c r="B7" s="39" t="n">
+        <v>2.76409697986888</v>
+      </c>
+      <c r="C7" s="39" t="n">
+        <v>2.351529326862223</v>
+      </c>
+      <c r="D7" s="26" t="n">
+        <v>7.414424832044875</v>
+      </c>
+      <c r="E7" s="39" t="n">
         <v>0.4125676530066569</v>
       </c>
-      <c r="C7" s="39" t="n">
+      <c r="F7" s="39" t="n">
         <v>0.4979300617169113</v>
       </c>
-      <c r="D7" s="26" t="n">
+      <c r="G7" s="26" t="n">
         <v>7.24476210014947</v>
       </c>
-      <c r="E7" s="37" t="n">
+      <c r="H7" s="39" t="n">
+        <v>2.76409697986888</v>
+      </c>
+      <c r="I7" s="39" t="n">
+        <v>0.4125676530066569</v>
+      </c>
+      <c r="J7" s="37" t="n">
         <v>-0.08536240871025447</v>
       </c>
-      <c r="F7" s="39" t="n">
-        <v>3.153070505465184</v>
-      </c>
-      <c r="G7" s="26" t="n">
-        <v>7.208836469285037</v>
-      </c>
-      <c r="H7" s="39" t="n">
-        <v>0.4125676530066569</v>
-      </c>
-      <c r="I7" s="37" t="n">
-        <v>-0.08536240871025447</v>
-      </c>
-      <c r="J7" s="37" t="n">
+      <c r="K7" s="37" t="n">
         <v>-3.238432914175438</v>
       </c>
-      <c r="K7" s="37" t="n">
+      <c r="L7" s="37" t="n">
         <v>-2.610173450399955</v>
-      </c>
-      <c r="L7" s="37" t="n">
-        <v>-2.79793443077293</v>
       </c>
     </row>
     <row r="8">
@@ -5885,37 +6171,37 @@
         </is>
       </c>
       <c r="B8" s="39" t="n">
+        <v>4.348566961626465</v>
+      </c>
+      <c r="C8" s="39" t="n">
+        <v>2.119449546778962</v>
+      </c>
+      <c r="D8" s="26" t="n">
+        <v>15.86490824291597</v>
+      </c>
+      <c r="E8" s="39" t="n">
         <v>2.229117414847503</v>
       </c>
-      <c r="C8" s="39" t="n">
-        <v>0.5508334859019024</v>
-      </c>
-      <c r="D8" s="26" t="n">
+      <c r="F8" s="39" t="n">
+        <v>0.550833485901902</v>
+      </c>
+      <c r="G8" s="26" t="n">
         <v>15.54267216853362</v>
       </c>
-      <c r="E8" s="39" t="n">
+      <c r="H8" s="39" t="n">
+        <v>4.348566961626465</v>
+      </c>
+      <c r="I8" s="39" t="n">
+        <v>2.229117414847503</v>
+      </c>
+      <c r="J8" s="39" t="n">
         <v>1.678283928945601</v>
       </c>
-      <c r="F8" s="39" t="n">
-        <v>3.218845929474368</v>
-      </c>
-      <c r="G8" s="26" t="n">
-        <v>15.45892475383101</v>
-      </c>
-      <c r="H8" s="39" t="n">
-        <v>2.229117414847503</v>
-      </c>
-      <c r="I8" s="39" t="n">
-        <v>1.678283928945601</v>
-      </c>
-      <c r="J8" s="37" t="n">
+      <c r="K8" s="37" t="n">
         <v>-1.540562000528767</v>
       </c>
-      <c r="K8" s="37" t="n">
+      <c r="L8" s="37" t="n">
         <v>-0.7697759192838771</v>
-      </c>
-      <c r="L8" s="37" t="n">
-        <v>-0.8338033345302587</v>
       </c>
     </row>
     <row r="9">
@@ -5925,37 +6211,37 @@
         </is>
       </c>
       <c r="B9" s="39" t="n">
+        <v>17.68857772474563</v>
+      </c>
+      <c r="C9" s="37" t="n">
+        <v>-1.792883531785524</v>
+      </c>
+      <c r="D9" s="26" t="n">
+        <v>11.60974402225383</v>
+      </c>
+      <c r="E9" s="39" t="n">
         <v>19.48146125653116</v>
       </c>
-      <c r="C9" s="39" t="n">
-        <v>1.73634922746017</v>
-      </c>
-      <c r="D9" s="26" t="n">
+      <c r="F9" s="39" t="n">
+        <v>1.736349227460167</v>
+      </c>
+      <c r="G9" s="26" t="n">
         <v>11.78660841528292</v>
       </c>
-      <c r="E9" s="39" t="n">
+      <c r="H9" s="39" t="n">
+        <v>17.68857772474563</v>
+      </c>
+      <c r="I9" s="39" t="n">
+        <v>19.48146125653116</v>
+      </c>
+      <c r="J9" s="39" t="n">
         <v>17.74511202907099</v>
       </c>
-      <c r="F9" s="39" t="n">
-        <v>1.249894733488652</v>
-      </c>
-      <c r="G9" s="26" t="n">
-        <v>11.61532101888666</v>
-      </c>
-      <c r="H9" s="39" t="n">
-        <v>19.48146125653116</v>
-      </c>
-      <c r="I9" s="39" t="n">
-        <v>17.74511202907099</v>
-      </c>
-      <c r="J9" s="39" t="n">
+      <c r="K9" s="39" t="n">
         <v>16.49521729558234</v>
       </c>
-      <c r="K9" s="39" t="n">
+      <c r="L9" s="39" t="n">
         <v>15.822730185473</v>
-      </c>
-      <c r="L9" s="39" t="n">
-        <v>14.72727552702231</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
EGAT retirement pages update 2026-04-21T04:15:07Z
</commit_message>
<xml_diff>
--- a/EGAT Retirement.xlsx
+++ b/EGAT Retirement.xlsx
@@ -683,7 +683,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I15"/>
+  <dimension ref="A1:I16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1317,6 +1317,47 @@
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>11:15:07</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>EGAT1</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>ตราสารหนี้ (EGAT-1)</t>
+        </is>
+      </c>
+      <c r="F16" t="n">
+        <v>15.76730382101877</v>
+      </c>
+      <c r="G16" t="n">
+        <v>0.6768794277878243</v>
+      </c>
+      <c r="H16" t="n">
+        <v>0.3870448801714277</v>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>https://app.powerbi.com/view?r=eyJrIjoiMzZjYWU3YmQtNWQ1Ny00NjdjLWI1MmEtYjExY2ZiYWIxMzNiIiwidCI6IjVmZWJjNjlmLThlOWMtNDcwOC1iNzBlLWQ4YzYyYmUxODA1YiIsImMiOjEwfQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1328,7 +1369,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I15"/>
+  <dimension ref="A1:I16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1962,6 +2003,47 @@
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>11:15:07</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>EGAT2</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>ตราสารทุน (EGAT-2)</t>
+        </is>
+      </c>
+      <c r="F16" t="n">
+        <v>40.0224030990135</v>
+      </c>
+      <c r="G16" t="n">
+        <v>2.359236981288704</v>
+      </c>
+      <c r="H16" t="n">
+        <v>17.92194239067766</v>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>https://app.powerbi.com/view?r=eyJrIjoiMzZjYWU3YmQtNWQ1Ny00NjdjLWI1MmEtYjExY2ZiYWIxMzNiIiwidCI6IjVmZWJjNjlmLThlOWMtNDcwOC1iNzBlLWQ4YzYyYmUxODA1YiIsImMiOjEwfQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1973,7 +2055,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I15"/>
+  <dimension ref="A1:I16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -2607,6 +2689,47 @@
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>11:15:07</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>EGAT3</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>อสังหาริมทรัพย์และโครงสร้างพื้นฐาน (EGAT-3)</t>
+        </is>
+      </c>
+      <c r="F16" t="n">
+        <v>8.772780739390125</v>
+      </c>
+      <c r="G16" t="n">
+        <v>4.25707630804939</v>
+      </c>
+      <c r="H16" t="n">
+        <v>1.400268169759111</v>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>https://app.powerbi.com/view?r=eyJrIjoiMzZjYWU3YmQtNWQ1Ny00NjdjLWI1MmEtYjExY2ZiYWIxMzNiIiwidCI6IjVmZWJjNjlmLThlOWMtNDcwOC1iNzBlLWQ4YzYyYmUxODA1YiIsImMiOjEwfQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2618,7 +2741,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I15"/>
+  <dimension ref="A1:I16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -3252,6 +3375,47 @@
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>11:15:07</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>EGAT4</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>ตราสารทุนต่างประเทศ (EGAT-4)</t>
+        </is>
+      </c>
+      <c r="F16" t="n">
+        <v>7.462318551064556</v>
+      </c>
+      <c r="G16" t="n">
+        <v>10.05881222413443</v>
+      </c>
+      <c r="H16" t="n">
+        <v>3.427905015900667</v>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>https://app.powerbi.com/view?r=eyJrIjoiMzZjYWU3YmQtNWQ1Ny00NjdjLWI1MmEtYjExY2ZiYWIxMzNiIiwidCI6IjVmZWJjNjlmLThlOWMtNDcwOC1iNzBlLWQ4YzYyYmUxODA1YiIsImMiOjEwfQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3263,7 +3427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I15"/>
+  <dimension ref="A1:I16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -3897,6 +4061,47 @@
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>11:15:07</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>EGAT5</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>ตราสารทุนต่างประเทศแบบอิงดัชนี (EGAT-5)</t>
+        </is>
+      </c>
+      <c r="F16" t="n">
+        <v>15.89489459642429</v>
+      </c>
+      <c r="G16" t="n">
+        <v>9.420313571350093</v>
+      </c>
+      <c r="H16" t="n">
+        <v>4.545796782882716</v>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>https://app.powerbi.com/view?r=eyJrIjoiMzZjYWU3YmQtNWQ1Ny00NjdjLWI1MmEtYjExY2ZiYWIxMzNiIiwidCI6IjVmZWJjNjlmLThlOWMtNDcwOC1iNzBlLWQ4YzYyYmUxODA1YiIsImMiOjEwfQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3908,7 +4113,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I15"/>
+  <dimension ref="A1:I16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -4537,6 +4742,47 @@
         <v>17.68857772474563</v>
       </c>
       <c r="I15" t="inlineStr">
+        <is>
+          <t>https://app.powerbi.com/view?r=eyJrIjoiMzZjYWU3YmQtNWQ1Ny00NjdjLWI1MmEtYjExY2ZiYWIxMzNiIiwidCI6IjVmZWJjNjlmLThlOWMtNDcwOC1iNzBlLWQ4YzYyYmUxODA1YiIsImMiOjEwfQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>11:15:07</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>EGAT6</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>การลงทุนตามหลักศาสนาอิสลาม (EGAT-6)</t>
+        </is>
+      </c>
+      <c r="F16" t="n">
+        <v>11.57984704129328</v>
+      </c>
+      <c r="G16" t="n">
+        <v>2.086156889597901</v>
+      </c>
+      <c r="H16" t="n">
+        <v>17.38551047702965</v>
+      </c>
+      <c r="I16" t="inlineStr">
         <is>
           <t>https://app.powerbi.com/view?r=eyJrIjoiMzZjYWU3YmQtNWQ1Ny00NjdjLWI1MmEtYjExY2ZiYWIxMzNiIiwidCI6IjVmZWJjNjlmLThlOWMtNDcwOC1iNzBlLWQ4YzYyYmUxODA1YiIsImMiOjEwfQ%3D%3D</t>
         </is>
@@ -5425,10 +5671,10 @@
         </is>
       </c>
       <c r="B18" s="35" t="n">
-        <v>7.430984281286986</v>
+        <v>7.430984281286985</v>
       </c>
       <c r="C18" s="35" t="n">
-        <v>0.3894322245032331</v>
+        <v>0.3894322245032322</v>
       </c>
       <c r="D18" s="35" t="n">
         <v>0.3846397190981454</v>
@@ -5443,7 +5689,7 @@
         <v>18.70061788946713</v>
       </c>
       <c r="H18" s="36" t="n">
-        <v>-0.9562975530711562</v>
+        <v>-0.9562975530711597</v>
       </c>
       <c r="I18" s="19" t="n">
         <v>40.28668355491568</v>
@@ -5479,7 +5725,7 @@
         <v>17.68857772474563</v>
       </c>
       <c r="T18" s="36" t="n">
-        <v>-1.792883531785524</v>
+        <v>-1.792883531785527</v>
       </c>
       <c r="U18" s="19" t="n">
         <v>11.60974402225383</v>
@@ -5491,26 +5737,66 @@
           <t>17/4/69</t>
         </is>
       </c>
-      <c r="B19" s="33" t="n"/>
-      <c r="C19" s="33" t="n"/>
-      <c r="D19" s="33" t="n"/>
-      <c r="E19" s="33" t="n"/>
-      <c r="F19" s="12" t="n"/>
-      <c r="G19" s="33" t="n"/>
-      <c r="H19" s="33" t="n"/>
-      <c r="I19" s="12" t="n"/>
-      <c r="J19" s="33" t="n"/>
-      <c r="K19" s="33" t="n"/>
-      <c r="L19" s="12" t="n"/>
-      <c r="M19" s="33" t="n"/>
-      <c r="N19" s="33" t="n"/>
-      <c r="O19" s="12" t="n"/>
-      <c r="P19" s="33" t="n"/>
-      <c r="Q19" s="33" t="n"/>
-      <c r="R19" s="12" t="n"/>
-      <c r="S19" s="33" t="n"/>
-      <c r="T19" s="33" t="n"/>
-      <c r="U19" s="12" t="n"/>
+      <c r="B19" s="35" t="n">
+        <v>7.511411286070206</v>
+      </c>
+      <c r="C19" s="35" t="n">
+        <v>0.08042700478322029</v>
+      </c>
+      <c r="D19" s="35" t="n">
+        <v>0.3870448801714277</v>
+      </c>
+      <c r="E19" s="35" t="n">
+        <v>0.002405161073282258</v>
+      </c>
+      <c r="F19" s="19" t="n">
+        <v>15.76730382101877</v>
+      </c>
+      <c r="G19" s="35" t="n">
+        <v>17.92194239067766</v>
+      </c>
+      <c r="H19" s="36" t="n">
+        <v>-0.7786754987894717</v>
+      </c>
+      <c r="I19" s="19" t="n">
+        <v>40.0224030990135</v>
+      </c>
+      <c r="J19" s="35" t="n">
+        <v>1.400268169759111</v>
+      </c>
+      <c r="K19" s="35" t="n">
+        <v>0.7008617568434516</v>
+      </c>
+      <c r="L19" s="19" t="n">
+        <v>8.772780739390125</v>
+      </c>
+      <c r="M19" s="35" t="n">
+        <v>3.427905015900667</v>
+      </c>
+      <c r="N19" s="35" t="n">
+        <v>0.6638080360317873</v>
+      </c>
+      <c r="O19" s="19" t="n">
+        <v>7.462318551064556</v>
+      </c>
+      <c r="P19" s="35" t="n">
+        <v>4.545796782882716</v>
+      </c>
+      <c r="Q19" s="35" t="n">
+        <v>0.1972298212562515</v>
+      </c>
+      <c r="R19" s="19" t="n">
+        <v>15.89489459642429</v>
+      </c>
+      <c r="S19" s="35" t="n">
+        <v>17.38551047702965</v>
+      </c>
+      <c r="T19" s="36" t="n">
+        <v>-0.3030672477159762</v>
+      </c>
+      <c r="U19" s="19" t="n">
+        <v>11.57984704129328</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="13" t="inlineStr">
@@ -5910,14 +6196,14 @@
       </c>
       <c r="B1" s="4" t="inlineStr">
         <is>
-          <t>16 เม.ย. 69 (พฤหัส)</t>
+          <t>17 เม.ย. 69 (ศุกร์)</t>
         </is>
       </c>
       <c r="C1" s="20" t="n"/>
       <c r="D1" s="20" t="n"/>
       <c r="E1" s="21" t="inlineStr">
         <is>
-          <t>10 เม.ย. 69 (ศุกร์)</t>
+          <t>16 เม.ย. 69 (พฤหัส)</t>
         </is>
       </c>
       <c r="F1" s="20" t="n"/>
@@ -5980,27 +6266,27 @@
       <c r="G3" s="20" t="n"/>
       <c r="H3" s="22" t="inlineStr">
         <is>
+          <t>17/4/69</t>
+        </is>
+      </c>
+      <c r="I3" s="22" t="inlineStr">
+        <is>
           <t>16/4/69</t>
         </is>
       </c>
-      <c r="I3" s="22" t="inlineStr">
+      <c r="J3" s="22" t="inlineStr">
         <is>
           <t>10/4/69</t>
         </is>
       </c>
-      <c r="J3" s="22" t="inlineStr">
+      <c r="K3" s="22" t="inlineStr">
         <is>
           <t>9/4/69</t>
         </is>
       </c>
-      <c r="K3" s="22" t="inlineStr">
+      <c r="L3" s="22" t="inlineStr">
         <is>
           <t>8/4/69</t>
-        </is>
-      </c>
-      <c r="L3" s="22" t="inlineStr">
-        <is>
-          <t>7/4/69</t>
         </is>
       </c>
     </row>
@@ -6011,37 +6297,37 @@
         </is>
       </c>
       <c r="B4" s="39" t="n">
+        <v>0.3870448801714277</v>
+      </c>
+      <c r="C4" s="39" t="n">
+        <v>0.002405161073282258</v>
+      </c>
+      <c r="D4" s="26" t="n">
+        <v>15.76730382101877</v>
+      </c>
+      <c r="E4" s="39" t="n">
         <v>0.3846397190981454</v>
       </c>
-      <c r="C4" s="39" t="n">
+      <c r="F4" s="39" t="n">
         <v>0.07872048604031795</v>
       </c>
-      <c r="D4" s="26" t="n">
+      <c r="G4" s="26" t="n">
         <v>15.76692605409251</v>
       </c>
-      <c r="E4" s="39" t="n">
+      <c r="H4" s="39" t="n">
+        <v>0.3870448801714277</v>
+      </c>
+      <c r="I4" s="39" t="n">
+        <v>0.3846397190981454</v>
+      </c>
+      <c r="J4" s="39" t="n">
         <v>0.3059192330578275</v>
       </c>
-      <c r="F4" s="37" t="n">
-        <v>-0.002220483901704928</v>
-      </c>
-      <c r="G4" s="26" t="n">
-        <v>15.75456181105879</v>
-      </c>
-      <c r="H4" s="39" t="n">
-        <v>0.3846397190981454</v>
-      </c>
-      <c r="I4" s="39" t="n">
-        <v>0.3059192330578275</v>
-      </c>
-      <c r="J4" s="39" t="n">
+      <c r="K4" s="39" t="n">
         <v>0.3081397169595324</v>
       </c>
-      <c r="K4" s="39" t="n">
+      <c r="L4" s="39" t="n">
         <v>0.3247471759871168</v>
-      </c>
-      <c r="L4" s="39" t="n">
-        <v>0.1589133858329816</v>
       </c>
     </row>
     <row r="5">
@@ -6051,37 +6337,37 @@
         </is>
       </c>
       <c r="B5" s="39" t="n">
+        <v>17.92194239067766</v>
+      </c>
+      <c r="C5" s="37" t="n">
+        <v>-0.7786754987894717</v>
+      </c>
+      <c r="D5" s="26" t="n">
+        <v>40.0224030990135</v>
+      </c>
+      <c r="E5" s="39" t="n">
         <v>18.70061788946713</v>
       </c>
-      <c r="C5" s="37" t="n">
-        <v>-0.9562975530711562</v>
-      </c>
-      <c r="D5" s="26" t="n">
+      <c r="F5" s="37" t="n">
+        <v>-0.9562975530711597</v>
+      </c>
+      <c r="G5" s="26" t="n">
         <v>40.28668355491568</v>
       </c>
-      <c r="E5" s="39" t="n">
+      <c r="H5" s="39" t="n">
+        <v>17.92194239067766</v>
+      </c>
+      <c r="I5" s="39" t="n">
+        <v>18.70061788946713</v>
+      </c>
+      <c r="J5" s="39" t="n">
         <v>19.65691544253829</v>
       </c>
-      <c r="F5" s="39" t="n">
-        <v>1.308726980434709</v>
-      </c>
-      <c r="G5" s="26" t="n">
-        <v>40.61124847791206</v>
-      </c>
-      <c r="H5" s="39" t="n">
-        <v>18.70061788946713</v>
-      </c>
-      <c r="I5" s="39" t="n">
-        <v>19.65691544253829</v>
-      </c>
-      <c r="J5" s="39" t="n">
+      <c r="K5" s="39" t="n">
         <v>18.34818846210358</v>
       </c>
-      <c r="K5" s="39" t="n">
+      <c r="L5" s="39" t="n">
         <v>18.2803381153805</v>
-      </c>
-      <c r="L5" s="39" t="n">
-        <v>16.30968964991566</v>
       </c>
     </row>
     <row r="6">
@@ -6091,37 +6377,37 @@
         </is>
       </c>
       <c r="B6" s="39" t="n">
+        <v>1.400268169759111</v>
+      </c>
+      <c r="C6" s="39" t="n">
+        <v>0.7008617568434516</v>
+      </c>
+      <c r="D6" s="26" t="n">
+        <v>8.772780739390125</v>
+      </c>
+      <c r="E6" s="39" t="n">
         <v>0.6994064129156596</v>
       </c>
-      <c r="C6" s="39" t="n">
+      <c r="F6" s="39" t="n">
         <v>0.5360750721945751</v>
       </c>
-      <c r="D6" s="26" t="n">
+      <c r="G6" s="26" t="n">
         <v>8.712144740764185</v>
       </c>
-      <c r="E6" s="39" t="n">
+      <c r="H6" s="39" t="n">
+        <v>1.400268169759111</v>
+      </c>
+      <c r="I6" s="39" t="n">
+        <v>0.6994064129156596</v>
+      </c>
+      <c r="J6" s="39" t="n">
         <v>0.1633313407210846</v>
       </c>
-      <c r="F6" s="39" t="n">
-        <v>0.1957559636015183</v>
-      </c>
-      <c r="G6" s="26" t="n">
-        <v>8.665765484051152</v>
-      </c>
-      <c r="H6" s="39" t="n">
-        <v>0.6994064129156596</v>
-      </c>
-      <c r="I6" s="39" t="n">
-        <v>0.1633313407210846</v>
-      </c>
-      <c r="J6" s="37" t="n">
+      <c r="K6" s="37" t="n">
         <v>-0.03242462288043368</v>
       </c>
-      <c r="K6" s="37" t="n">
+      <c r="L6" s="37" t="n">
         <v>-0.0361254471118011</v>
-      </c>
-      <c r="L6" s="37" t="n">
-        <v>-1.631124094698189</v>
       </c>
     </row>
     <row r="7">
@@ -6131,37 +6417,37 @@
         </is>
       </c>
       <c r="B7" s="39" t="n">
+        <v>3.427905015900667</v>
+      </c>
+      <c r="C7" s="39" t="n">
+        <v>0.6638080360317873</v>
+      </c>
+      <c r="D7" s="26" t="n">
+        <v>7.462318551064556</v>
+      </c>
+      <c r="E7" s="39" t="n">
         <v>2.76409697986888</v>
       </c>
-      <c r="C7" s="39" t="n">
+      <c r="F7" s="39" t="n">
         <v>2.351529326862223</v>
       </c>
-      <c r="D7" s="26" t="n">
+      <c r="G7" s="26" t="n">
         <v>7.414424832044875</v>
       </c>
-      <c r="E7" s="39" t="n">
+      <c r="H7" s="39" t="n">
+        <v>3.427905015900667</v>
+      </c>
+      <c r="I7" s="39" t="n">
+        <v>2.76409697986888</v>
+      </c>
+      <c r="J7" s="39" t="n">
         <v>0.4125676530066569</v>
       </c>
-      <c r="F7" s="39" t="n">
-        <v>0.4979300617169113</v>
-      </c>
-      <c r="G7" s="26" t="n">
-        <v>7.24476210014947</v>
-      </c>
-      <c r="H7" s="39" t="n">
-        <v>2.76409697986888</v>
-      </c>
-      <c r="I7" s="39" t="n">
-        <v>0.4125676530066569</v>
-      </c>
-      <c r="J7" s="37" t="n">
+      <c r="K7" s="37" t="n">
         <v>-0.08536240871025447</v>
       </c>
-      <c r="K7" s="37" t="n">
+      <c r="L7" s="37" t="n">
         <v>-3.238432914175438</v>
-      </c>
-      <c r="L7" s="37" t="n">
-        <v>-2.610173450399955</v>
       </c>
     </row>
     <row r="8">
@@ -6171,37 +6457,37 @@
         </is>
       </c>
       <c r="B8" s="39" t="n">
+        <v>4.545796782882716</v>
+      </c>
+      <c r="C8" s="39" t="n">
+        <v>0.1972298212562515</v>
+      </c>
+      <c r="D8" s="26" t="n">
+        <v>15.89489459642429</v>
+      </c>
+      <c r="E8" s="39" t="n">
         <v>4.348566961626465</v>
       </c>
-      <c r="C8" s="39" t="n">
+      <c r="F8" s="39" t="n">
         <v>2.119449546778962</v>
       </c>
-      <c r="D8" s="26" t="n">
+      <c r="G8" s="26" t="n">
         <v>15.86490824291597</v>
       </c>
-      <c r="E8" s="39" t="n">
+      <c r="H8" s="39" t="n">
+        <v>4.545796782882716</v>
+      </c>
+      <c r="I8" s="39" t="n">
+        <v>4.348566961626465</v>
+      </c>
+      <c r="J8" s="39" t="n">
         <v>2.229117414847503</v>
       </c>
-      <c r="F8" s="39" t="n">
-        <v>0.550833485901902</v>
-      </c>
-      <c r="G8" s="26" t="n">
-        <v>15.54267216853362</v>
-      </c>
-      <c r="H8" s="39" t="n">
-        <v>4.348566961626465</v>
-      </c>
-      <c r="I8" s="39" t="n">
-        <v>2.229117414847503</v>
-      </c>
-      <c r="J8" s="39" t="n">
+      <c r="K8" s="39" t="n">
         <v>1.678283928945601</v>
       </c>
-      <c r="K8" s="37" t="n">
+      <c r="L8" s="37" t="n">
         <v>-1.540562000528767</v>
-      </c>
-      <c r="L8" s="37" t="n">
-        <v>-0.7697759192838771</v>
       </c>
     </row>
     <row r="9">
@@ -6211,37 +6497,37 @@
         </is>
       </c>
       <c r="B9" s="39" t="n">
+        <v>17.38551047702965</v>
+      </c>
+      <c r="C9" s="37" t="n">
+        <v>-0.3030672477159762</v>
+      </c>
+      <c r="D9" s="26" t="n">
+        <v>11.57984704129328</v>
+      </c>
+      <c r="E9" s="39" t="n">
         <v>17.68857772474563</v>
       </c>
-      <c r="C9" s="37" t="n">
-        <v>-1.792883531785524</v>
-      </c>
-      <c r="D9" s="26" t="n">
+      <c r="F9" s="37" t="n">
+        <v>-1.792883531785527</v>
+      </c>
+      <c r="G9" s="26" t="n">
         <v>11.60974402225383</v>
       </c>
-      <c r="E9" s="39" t="n">
+      <c r="H9" s="39" t="n">
+        <v>17.38551047702965</v>
+      </c>
+      <c r="I9" s="39" t="n">
+        <v>17.68857772474563</v>
+      </c>
+      <c r="J9" s="39" t="n">
         <v>19.48146125653116</v>
       </c>
-      <c r="F9" s="39" t="n">
-        <v>1.736349227460167</v>
-      </c>
-      <c r="G9" s="26" t="n">
-        <v>11.78660841528292</v>
-      </c>
-      <c r="H9" s="39" t="n">
-        <v>17.68857772474563</v>
-      </c>
-      <c r="I9" s="39" t="n">
-        <v>19.48146125653116</v>
-      </c>
-      <c r="J9" s="39" t="n">
+      <c r="K9" s="39" t="n">
         <v>17.74511202907099</v>
       </c>
-      <c r="K9" s="39" t="n">
+      <c r="L9" s="39" t="n">
         <v>16.49521729558234</v>
-      </c>
-      <c r="L9" s="39" t="n">
-        <v>15.822730185473</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
EGAT retirement pages update 2026-04-22T04:15:08Z
</commit_message>
<xml_diff>
--- a/EGAT Retirement.xlsx
+++ b/EGAT Retirement.xlsx
@@ -683,7 +683,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I16"/>
+  <dimension ref="A1:I17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1358,6 +1358,47 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-04-20</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>11:15:07</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>2026-04-20</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>EGAT1</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>ตราสารหนี้ (EGAT-1)</t>
+        </is>
+      </c>
+      <c r="F17" t="n">
+        <v>15.75653850665382</v>
+      </c>
+      <c r="G17" t="n">
+        <v>0.6081410899828832</v>
+      </c>
+      <c r="H17" t="n">
+        <v>0.3185044303538165</v>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>https://app.powerbi.com/view?r=eyJrIjoiMzZjYWU3YmQtNWQ1Ny00NjdjLWI1MmEtYjExY2ZiYWIxMzNiIiwidCI6IjVmZWJjNjlmLThlOWMtNDcwOC1iNzBlLWQ4YzYyYmUxODA1YiIsImMiOjEwfQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1369,7 +1410,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I16"/>
+  <dimension ref="A1:I17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -2044,6 +2085,47 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-04-20</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>11:15:07</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>2026-04-20</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>EGAT2</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>ตราสารทุน (EGAT-2)</t>
+        </is>
+      </c>
+      <c r="F17" t="n">
+        <v>40.00968825655211</v>
+      </c>
+      <c r="G17" t="n">
+        <v>2.326718155033669</v>
+      </c>
+      <c r="H17" t="n">
+        <v>17.88447939984901</v>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>https://app.powerbi.com/view?r=eyJrIjoiMzZjYWU3YmQtNWQ1Ny00NjdjLWI1MmEtYjExY2ZiYWIxMzNiIiwidCI6IjVmZWJjNjlmLThlOWMtNDcwOC1iNzBlLWQ4YzYyYmUxODA1YiIsImMiOjEwfQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2055,7 +2137,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I16"/>
+  <dimension ref="A1:I17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -2730,6 +2812,47 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-04-20</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>11:15:07</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>2026-04-20</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>EGAT3</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>อสังหาริมทรัพย์และโครงสร้างพื้นฐาน (EGAT-3)</t>
+        </is>
+      </c>
+      <c r="F17" t="n">
+        <v>8.763734028464144</v>
+      </c>
+      <c r="G17" t="n">
+        <v>4.149563803250089</v>
+      </c>
+      <c r="H17" t="n">
+        <v>1.295701676967398</v>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>https://app.powerbi.com/view?r=eyJrIjoiMzZjYWU3YmQtNWQ1Ny00NjdjLWI1MmEtYjExY2ZiYWIxMzNiIiwidCI6IjVmZWJjNjlmLThlOWMtNDcwOC1iNzBlLWQ4YzYyYmUxODA1YiIsImMiOjEwfQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2741,7 +2864,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I16"/>
+  <dimension ref="A1:I17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -3416,6 +3539,47 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-04-20</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>11:15:07</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>2026-04-20</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>EGAT4</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>ตราสารทุนต่างประเทศ (EGAT-4)</t>
+        </is>
+      </c>
+      <c r="F17" t="n">
+        <v>7.562013929915418</v>
+      </c>
+      <c r="G17" t="n">
+        <v>11.5291803014923</v>
+      </c>
+      <c r="H17" t="n">
+        <v>4.809685236585581</v>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>https://app.powerbi.com/view?r=eyJrIjoiMzZjYWU3YmQtNWQ1Ny00NjdjLWI1MmEtYjExY2ZiYWIxMzNiIiwidCI6IjVmZWJjNjlmLThlOWMtNDcwOC1iNzBlLWQ4YzYyYmUxODA1YiIsImMiOjEwfQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3427,7 +3591,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I16"/>
+  <dimension ref="A1:I17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -4102,6 +4266,47 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-04-20</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>11:15:07</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>2026-04-20</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>EGAT5</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>ตราสารทุนต่างประเทศแบบอิงดัชนี (EGAT-5)</t>
+        </is>
+      </c>
+      <c r="F17" t="n">
+        <v>16.11235108660363</v>
+      </c>
+      <c r="G17" t="n">
+        <v>10.91728212305738</v>
+      </c>
+      <c r="H17" t="n">
+        <v>5.976077549672043</v>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>https://app.powerbi.com/view?r=eyJrIjoiMzZjYWU3YmQtNWQ1Ny00NjdjLWI1MmEtYjExY2ZiYWIxMzNiIiwidCI6IjVmZWJjNjlmLThlOWMtNDcwOC1iNzBlLWQ4YzYyYmUxODA1YiIsImMiOjEwfQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4113,7 +4318,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I16"/>
+  <dimension ref="A1:I17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -4783,6 +4988,47 @@
         <v>17.38551047702965</v>
       </c>
       <c r="I16" t="inlineStr">
+        <is>
+          <t>https://app.powerbi.com/view?r=eyJrIjoiMzZjYWU3YmQtNWQ1Ny00NjdjLWI1MmEtYjExY2ZiYWIxMzNiIiwidCI6IjVmZWJjNjlmLThlOWMtNDcwOC1iNzBlLWQ4YzYyYmUxODA1YiIsImMiOjEwfQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-04-20</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>11:15:07</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>2026-04-20</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>EGAT6</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>การลงทุนตามหลักศาสนาอิสลาม (EGAT-6)</t>
+        </is>
+      </c>
+      <c r="F17" t="n">
+        <v>11.59759457528724</v>
+      </c>
+      <c r="G17" t="n">
+        <v>2.242616429456246</v>
+      </c>
+      <c r="H17" t="n">
+        <v>17.56541815026234</v>
+      </c>
+      <c r="I17" t="inlineStr">
         <is>
           <t>https://app.powerbi.com/view?r=eyJrIjoiMzZjYWU3YmQtNWQ1Ny00NjdjLWI1MmEtYjExY2ZiYWIxMzNiIiwidCI6IjVmZWJjNjlmLThlOWMtNDcwOC1iNzBlLWQ4YzYyYmUxODA1YiIsImMiOjEwfQ%3D%3D</t>
         </is>
@@ -5756,7 +6002,7 @@
         <v>17.92194239067766</v>
       </c>
       <c r="H19" s="36" t="n">
-        <v>-0.7786754987894717</v>
+        <v>-0.7786754987894682</v>
       </c>
       <c r="I19" s="19" t="n">
         <v>40.0224030990135</v>
@@ -5765,7 +6011,7 @@
         <v>1.400268169759111</v>
       </c>
       <c r="K19" s="35" t="n">
-        <v>0.7008617568434516</v>
+        <v>0.7008617568434514</v>
       </c>
       <c r="L19" s="19" t="n">
         <v>8.772780739390125</v>
@@ -5774,7 +6020,7 @@
         <v>3.427905015900667</v>
       </c>
       <c r="N19" s="35" t="n">
-        <v>0.6638080360317873</v>
+        <v>0.6638080360317868</v>
       </c>
       <c r="O19" s="19" t="n">
         <v>7.462318551064556</v>
@@ -5792,7 +6038,7 @@
         <v>17.38551047702965</v>
       </c>
       <c r="T19" s="36" t="n">
-        <v>-0.3030672477159762</v>
+        <v>-0.3030672477159797</v>
       </c>
       <c r="U19" s="19" t="n">
         <v>11.57984704129328</v>
@@ -5858,26 +6104,66 @@
           <t>20/4/69</t>
         </is>
       </c>
-      <c r="B22" s="33" t="n"/>
-      <c r="C22" s="33" t="n"/>
-      <c r="D22" s="33" t="n"/>
-      <c r="E22" s="33" t="n"/>
-      <c r="F22" s="12" t="n"/>
-      <c r="G22" s="33" t="n"/>
-      <c r="H22" s="33" t="n"/>
-      <c r="I22" s="12" t="n"/>
-      <c r="J22" s="33" t="n"/>
-      <c r="K22" s="33" t="n"/>
-      <c r="L22" s="12" t="n"/>
-      <c r="M22" s="33" t="n"/>
-      <c r="N22" s="33" t="n"/>
-      <c r="O22" s="12" t="n"/>
-      <c r="P22" s="33" t="n"/>
-      <c r="Q22" s="33" t="n"/>
-      <c r="R22" s="12" t="n"/>
-      <c r="S22" s="33" t="n"/>
-      <c r="T22" s="33" t="n"/>
-      <c r="U22" s="12" t="n"/>
+      <c r="B22" s="35" t="n">
+        <v>7.974977740615031</v>
+      </c>
+      <c r="C22" s="35" t="n">
+        <v>0.463566454544825</v>
+      </c>
+      <c r="D22" s="35" t="n">
+        <v>0.3185044303538165</v>
+      </c>
+      <c r="E22" s="36" t="n">
+        <v>-0.0685404498176112</v>
+      </c>
+      <c r="F22" s="19" t="n">
+        <v>15.75653850665382</v>
+      </c>
+      <c r="G22" s="35" t="n">
+        <v>17.88447939984901</v>
+      </c>
+      <c r="H22" s="36" t="n">
+        <v>-0.03746299082865434</v>
+      </c>
+      <c r="I22" s="19" t="n">
+        <v>40.00968825655211</v>
+      </c>
+      <c r="J22" s="35" t="n">
+        <v>1.295701676967398</v>
+      </c>
+      <c r="K22" s="36" t="n">
+        <v>-0.1045664927917132</v>
+      </c>
+      <c r="L22" s="19" t="n">
+        <v>8.763734028464144</v>
+      </c>
+      <c r="M22" s="35" t="n">
+        <v>4.809685236585581</v>
+      </c>
+      <c r="N22" s="35" t="n">
+        <v>1.381780220684914</v>
+      </c>
+      <c r="O22" s="19" t="n">
+        <v>7.562013929915418</v>
+      </c>
+      <c r="P22" s="35" t="n">
+        <v>5.976077549672043</v>
+      </c>
+      <c r="Q22" s="35" t="n">
+        <v>1.430280766789327</v>
+      </c>
+      <c r="R22" s="19" t="n">
+        <v>16.11235108660363</v>
+      </c>
+      <c r="S22" s="35" t="n">
+        <v>17.56541815026234</v>
+      </c>
+      <c r="T22" s="35" t="n">
+        <v>0.1799076732326839</v>
+      </c>
+      <c r="U22" s="19" t="n">
+        <v>11.59759457528724</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="10" t="inlineStr">
@@ -6196,14 +6482,14 @@
       </c>
       <c r="B1" s="4" t="inlineStr">
         <is>
-          <t>17 เม.ย. 69 (ศุกร์)</t>
+          <t>20 เม.ย. 69 (จันทร์)</t>
         </is>
       </c>
       <c r="C1" s="20" t="n"/>
       <c r="D1" s="20" t="n"/>
       <c r="E1" s="21" t="inlineStr">
         <is>
-          <t>16 เม.ย. 69 (พฤหัส)</t>
+          <t>17 เม.ย. 69 (ศุกร์)</t>
         </is>
       </c>
       <c r="F1" s="20" t="n"/>
@@ -6266,27 +6552,27 @@
       <c r="G3" s="20" t="n"/>
       <c r="H3" s="22" t="inlineStr">
         <is>
+          <t>20/4/69</t>
+        </is>
+      </c>
+      <c r="I3" s="22" t="inlineStr">
+        <is>
           <t>17/4/69</t>
         </is>
       </c>
-      <c r="I3" s="22" t="inlineStr">
+      <c r="J3" s="22" t="inlineStr">
         <is>
           <t>16/4/69</t>
         </is>
       </c>
-      <c r="J3" s="22" t="inlineStr">
+      <c r="K3" s="22" t="inlineStr">
         <is>
           <t>10/4/69</t>
         </is>
       </c>
-      <c r="K3" s="22" t="inlineStr">
+      <c r="L3" s="22" t="inlineStr">
         <is>
           <t>9/4/69</t>
-        </is>
-      </c>
-      <c r="L3" s="22" t="inlineStr">
-        <is>
-          <t>8/4/69</t>
         </is>
       </c>
     </row>
@@ -6297,37 +6583,37 @@
         </is>
       </c>
       <c r="B4" s="39" t="n">
+        <v>0.3185044303538165</v>
+      </c>
+      <c r="C4" s="37" t="n">
+        <v>-0.0685404498176112</v>
+      </c>
+      <c r="D4" s="26" t="n">
+        <v>15.75653850665382</v>
+      </c>
+      <c r="E4" s="39" t="n">
         <v>0.3870448801714277</v>
       </c>
-      <c r="C4" s="39" t="n">
+      <c r="F4" s="39" t="n">
         <v>0.002405161073282258</v>
       </c>
-      <c r="D4" s="26" t="n">
+      <c r="G4" s="26" t="n">
         <v>15.76730382101877</v>
       </c>
-      <c r="E4" s="39" t="n">
+      <c r="H4" s="39" t="n">
+        <v>0.3185044303538165</v>
+      </c>
+      <c r="I4" s="39" t="n">
+        <v>0.3870448801714277</v>
+      </c>
+      <c r="J4" s="39" t="n">
         <v>0.3846397190981454</v>
       </c>
-      <c r="F4" s="39" t="n">
-        <v>0.07872048604031795</v>
-      </c>
-      <c r="G4" s="26" t="n">
-        <v>15.76692605409251</v>
-      </c>
-      <c r="H4" s="39" t="n">
-        <v>0.3870448801714277</v>
-      </c>
-      <c r="I4" s="39" t="n">
-        <v>0.3846397190981454</v>
-      </c>
-      <c r="J4" s="39" t="n">
+      <c r="K4" s="39" t="n">
         <v>0.3059192330578275</v>
       </c>
-      <c r="K4" s="39" t="n">
+      <c r="L4" s="39" t="n">
         <v>0.3081397169595324</v>
-      </c>
-      <c r="L4" s="39" t="n">
-        <v>0.3247471759871168</v>
       </c>
     </row>
     <row r="5">
@@ -6337,37 +6623,37 @@
         </is>
       </c>
       <c r="B5" s="39" t="n">
+        <v>17.88447939984901</v>
+      </c>
+      <c r="C5" s="37" t="n">
+        <v>-0.03746299082865434</v>
+      </c>
+      <c r="D5" s="26" t="n">
+        <v>40.00968825655211</v>
+      </c>
+      <c r="E5" s="39" t="n">
         <v>17.92194239067766</v>
       </c>
-      <c r="C5" s="37" t="n">
-        <v>-0.7786754987894717</v>
-      </c>
-      <c r="D5" s="26" t="n">
+      <c r="F5" s="37" t="n">
+        <v>-0.7786754987894682</v>
+      </c>
+      <c r="G5" s="26" t="n">
         <v>40.0224030990135</v>
       </c>
-      <c r="E5" s="39" t="n">
+      <c r="H5" s="39" t="n">
+        <v>17.88447939984901</v>
+      </c>
+      <c r="I5" s="39" t="n">
+        <v>17.92194239067766</v>
+      </c>
+      <c r="J5" s="39" t="n">
         <v>18.70061788946713</v>
       </c>
-      <c r="F5" s="37" t="n">
-        <v>-0.9562975530711597</v>
-      </c>
-      <c r="G5" s="26" t="n">
-        <v>40.28668355491568</v>
-      </c>
-      <c r="H5" s="39" t="n">
-        <v>17.92194239067766</v>
-      </c>
-      <c r="I5" s="39" t="n">
-        <v>18.70061788946713</v>
-      </c>
-      <c r="J5" s="39" t="n">
+      <c r="K5" s="39" t="n">
         <v>19.65691544253829</v>
       </c>
-      <c r="K5" s="39" t="n">
+      <c r="L5" s="39" t="n">
         <v>18.34818846210358</v>
-      </c>
-      <c r="L5" s="39" t="n">
-        <v>18.2803381153805</v>
       </c>
     </row>
     <row r="6">
@@ -6377,37 +6663,37 @@
         </is>
       </c>
       <c r="B6" s="39" t="n">
+        <v>1.295701676967398</v>
+      </c>
+      <c r="C6" s="37" t="n">
+        <v>-0.1045664927917132</v>
+      </c>
+      <c r="D6" s="26" t="n">
+        <v>8.763734028464144</v>
+      </c>
+      <c r="E6" s="39" t="n">
         <v>1.400268169759111</v>
       </c>
-      <c r="C6" s="39" t="n">
-        <v>0.7008617568434516</v>
-      </c>
-      <c r="D6" s="26" t="n">
+      <c r="F6" s="39" t="n">
+        <v>0.7008617568434514</v>
+      </c>
+      <c r="G6" s="26" t="n">
         <v>8.772780739390125</v>
       </c>
-      <c r="E6" s="39" t="n">
+      <c r="H6" s="39" t="n">
+        <v>1.295701676967398</v>
+      </c>
+      <c r="I6" s="39" t="n">
+        <v>1.400268169759111</v>
+      </c>
+      <c r="J6" s="39" t="n">
         <v>0.6994064129156596</v>
       </c>
-      <c r="F6" s="39" t="n">
-        <v>0.5360750721945751</v>
-      </c>
-      <c r="G6" s="26" t="n">
-        <v>8.712144740764185</v>
-      </c>
-      <c r="H6" s="39" t="n">
-        <v>1.400268169759111</v>
-      </c>
-      <c r="I6" s="39" t="n">
-        <v>0.6994064129156596</v>
-      </c>
-      <c r="J6" s="39" t="n">
+      <c r="K6" s="39" t="n">
         <v>0.1633313407210846</v>
       </c>
-      <c r="K6" s="37" t="n">
+      <c r="L6" s="37" t="n">
         <v>-0.03242462288043368</v>
-      </c>
-      <c r="L6" s="37" t="n">
-        <v>-0.0361254471118011</v>
       </c>
     </row>
     <row r="7">
@@ -6417,37 +6703,37 @@
         </is>
       </c>
       <c r="B7" s="39" t="n">
+        <v>4.809685236585581</v>
+      </c>
+      <c r="C7" s="39" t="n">
+        <v>1.381780220684914</v>
+      </c>
+      <c r="D7" s="26" t="n">
+        <v>7.562013929915418</v>
+      </c>
+      <c r="E7" s="39" t="n">
         <v>3.427905015900667</v>
       </c>
-      <c r="C7" s="39" t="n">
-        <v>0.6638080360317873</v>
-      </c>
-      <c r="D7" s="26" t="n">
+      <c r="F7" s="39" t="n">
+        <v>0.6638080360317868</v>
+      </c>
+      <c r="G7" s="26" t="n">
         <v>7.462318551064556</v>
       </c>
-      <c r="E7" s="39" t="n">
+      <c r="H7" s="39" t="n">
+        <v>4.809685236585581</v>
+      </c>
+      <c r="I7" s="39" t="n">
+        <v>3.427905015900667</v>
+      </c>
+      <c r="J7" s="39" t="n">
         <v>2.76409697986888</v>
       </c>
-      <c r="F7" s="39" t="n">
-        <v>2.351529326862223</v>
-      </c>
-      <c r="G7" s="26" t="n">
-        <v>7.414424832044875</v>
-      </c>
-      <c r="H7" s="39" t="n">
-        <v>3.427905015900667</v>
-      </c>
-      <c r="I7" s="39" t="n">
-        <v>2.76409697986888</v>
-      </c>
-      <c r="J7" s="39" t="n">
+      <c r="K7" s="39" t="n">
         <v>0.4125676530066569</v>
       </c>
-      <c r="K7" s="37" t="n">
+      <c r="L7" s="37" t="n">
         <v>-0.08536240871025447</v>
-      </c>
-      <c r="L7" s="37" t="n">
-        <v>-3.238432914175438</v>
       </c>
     </row>
     <row r="8">
@@ -6457,37 +6743,37 @@
         </is>
       </c>
       <c r="B8" s="39" t="n">
+        <v>5.976077549672043</v>
+      </c>
+      <c r="C8" s="39" t="n">
+        <v>1.430280766789327</v>
+      </c>
+      <c r="D8" s="26" t="n">
+        <v>16.11235108660363</v>
+      </c>
+      <c r="E8" s="39" t="n">
         <v>4.545796782882716</v>
       </c>
-      <c r="C8" s="39" t="n">
+      <c r="F8" s="39" t="n">
         <v>0.1972298212562515</v>
       </c>
-      <c r="D8" s="26" t="n">
+      <c r="G8" s="26" t="n">
         <v>15.89489459642429</v>
       </c>
-      <c r="E8" s="39" t="n">
+      <c r="H8" s="39" t="n">
+        <v>5.976077549672043</v>
+      </c>
+      <c r="I8" s="39" t="n">
+        <v>4.545796782882716</v>
+      </c>
+      <c r="J8" s="39" t="n">
         <v>4.348566961626465</v>
       </c>
-      <c r="F8" s="39" t="n">
-        <v>2.119449546778962</v>
-      </c>
-      <c r="G8" s="26" t="n">
-        <v>15.86490824291597</v>
-      </c>
-      <c r="H8" s="39" t="n">
-        <v>4.545796782882716</v>
-      </c>
-      <c r="I8" s="39" t="n">
-        <v>4.348566961626465</v>
-      </c>
-      <c r="J8" s="39" t="n">
+      <c r="K8" s="39" t="n">
         <v>2.229117414847503</v>
       </c>
-      <c r="K8" s="39" t="n">
+      <c r="L8" s="39" t="n">
         <v>1.678283928945601</v>
-      </c>
-      <c r="L8" s="37" t="n">
-        <v>-1.540562000528767</v>
       </c>
     </row>
     <row r="9">
@@ -6497,37 +6783,37 @@
         </is>
       </c>
       <c r="B9" s="39" t="n">
+        <v>17.56541815026234</v>
+      </c>
+      <c r="C9" s="39" t="n">
+        <v>0.1799076732326839</v>
+      </c>
+      <c r="D9" s="26" t="n">
+        <v>11.59759457528724</v>
+      </c>
+      <c r="E9" s="39" t="n">
         <v>17.38551047702965</v>
       </c>
-      <c r="C9" s="37" t="n">
-        <v>-0.3030672477159762</v>
-      </c>
-      <c r="D9" s="26" t="n">
+      <c r="F9" s="37" t="n">
+        <v>-0.3030672477159797</v>
+      </c>
+      <c r="G9" s="26" t="n">
         <v>11.57984704129328</v>
       </c>
-      <c r="E9" s="39" t="n">
+      <c r="H9" s="39" t="n">
+        <v>17.56541815026234</v>
+      </c>
+      <c r="I9" s="39" t="n">
+        <v>17.38551047702965</v>
+      </c>
+      <c r="J9" s="39" t="n">
         <v>17.68857772474563</v>
       </c>
-      <c r="F9" s="37" t="n">
-        <v>-1.792883531785527</v>
-      </c>
-      <c r="G9" s="26" t="n">
-        <v>11.60974402225383</v>
-      </c>
-      <c r="H9" s="39" t="n">
-        <v>17.38551047702965</v>
-      </c>
-      <c r="I9" s="39" t="n">
-        <v>17.68857772474563</v>
-      </c>
-      <c r="J9" s="39" t="n">
+      <c r="K9" s="39" t="n">
         <v>19.48146125653116</v>
       </c>
-      <c r="K9" s="39" t="n">
+      <c r="L9" s="39" t="n">
         <v>17.74511202907099</v>
-      </c>
-      <c r="L9" s="39" t="n">
-        <v>16.49521729558234</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
EGAT retirement pages update 2026-04-23T04:15:07Z
</commit_message>
<xml_diff>
--- a/EGAT Retirement.xlsx
+++ b/EGAT Retirement.xlsx
@@ -683,7 +683,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I17"/>
+  <dimension ref="A1:I18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1399,6 +1399,47 @@
         </is>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-04-21</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>11:15:06</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>2026-04-21</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>EGAT1</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>ตราสารหนี้ (EGAT-1)</t>
+        </is>
+      </c>
+      <c r="F18" t="n">
+        <v>15.76333906599318</v>
+      </c>
+      <c r="G18" t="n">
+        <v>0.6515638019710668</v>
+      </c>
+      <c r="H18" t="n">
+        <v>0.3618021344736988</v>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>https://app.powerbi.com/view?r=eyJrIjoiMzZjYWU3YmQtNWQ1Ny00NjdjLWI1MmEtYjExY2ZiYWIxMzNiIiwidCI6IjVmZWJjNjlmLThlOWMtNDcwOC1iNzBlLWQ4YzYyYmUxODA1YiIsImMiOjEwfQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1410,7 +1451,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I17"/>
+  <dimension ref="A1:I18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -2126,6 +2167,47 @@
         </is>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-04-21</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>11:15:06</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>2026-04-21</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>EGAT2</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>ตราสารทุน (EGAT-2)</t>
+        </is>
+      </c>
+      <c r="F18" t="n">
+        <v>40.19627537813753</v>
+      </c>
+      <c r="G18" t="n">
+        <v>2.803923767819305</v>
+      </c>
+      <c r="H18" t="n">
+        <v>18.43423938672446</v>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>https://app.powerbi.com/view?r=eyJrIjoiMzZjYWU3YmQtNWQ1Ny00NjdjLWI1MmEtYjExY2ZiYWIxMzNiIiwidCI6IjVmZWJjNjlmLThlOWMtNDcwOC1iNzBlLWQ4YzYyYmUxODA1YiIsImMiOjEwfQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2137,7 +2219,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I17"/>
+  <dimension ref="A1:I18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -2853,6 +2935,47 @@
         </is>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-04-21</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>11:15:06</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>2026-04-21</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>EGAT3</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>อสังหาริมทรัพย์และโครงสร้างพื้นฐาน (EGAT-3)</t>
+        </is>
+      </c>
+      <c r="F18" t="n">
+        <v>8.835116823464528</v>
+      </c>
+      <c r="G18" t="n">
+        <v>4.997887923790478</v>
+      </c>
+      <c r="H18" t="n">
+        <v>2.120780380148246</v>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>https://app.powerbi.com/view?r=eyJrIjoiMzZjYWU3YmQtNWQ1Ny00NjdjLWI1MmEtYjExY2ZiYWIxMzNiIiwidCI6IjVmZWJjNjlmLThlOWMtNDcwOC1iNzBlLWQ4YzYyYmUxODA1YiIsImMiOjEwfQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2864,7 +2987,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I17"/>
+  <dimension ref="A1:I18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -3580,6 +3703,47 @@
         </is>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-04-21</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>11:15:06</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>2026-04-21</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>EGAT4</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>ตราสารทุนต่างประเทศ (EGAT-4)</t>
+        </is>
+      </c>
+      <c r="F18" t="n">
+        <v>7.538702486380125</v>
+      </c>
+      <c r="G18" t="n">
+        <v>11.18536895530444</v>
+      </c>
+      <c r="H18" t="n">
+        <v>4.486588098443733</v>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>https://app.powerbi.com/view?r=eyJrIjoiMzZjYWU3YmQtNWQ1Ny00NjdjLWI1MmEtYjExY2ZiYWIxMzNiIiwidCI6IjVmZWJjNjlmLThlOWMtNDcwOC1iNzBlLWQ4YzYyYmUxODA1YiIsImMiOjEwfQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3591,7 +3755,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I17"/>
+  <dimension ref="A1:I18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -4307,6 +4471,47 @@
         </is>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-04-21</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>11:15:06</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>2026-04-21</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>EGAT5</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>ตราสารทุนต่างประเทศแบบอิงดัชนี (EGAT-5)</t>
+        </is>
+      </c>
+      <c r="F18" t="n">
+        <v>16.0564065155152</v>
+      </c>
+      <c r="G18" t="n">
+        <v>10.53216019135934</v>
+      </c>
+      <c r="H18" t="n">
+        <v>5.608112243287855</v>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>https://app.powerbi.com/view?r=eyJrIjoiMzZjYWU3YmQtNWQ1Ny00NjdjLWI1MmEtYjExY2ZiYWIxMzNiIiwidCI6IjVmZWJjNjlmLThlOWMtNDcwOC1iNzBlLWQ4YzYyYmUxODA1YiIsImMiOjEwfQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4318,7 +4523,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I17"/>
+  <dimension ref="A1:I18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -5029,6 +5234,47 @@
         <v>17.56541815026234</v>
       </c>
       <c r="I17" t="inlineStr">
+        <is>
+          <t>https://app.powerbi.com/view?r=eyJrIjoiMzZjYWU3YmQtNWQ1Ny00NjdjLWI1MmEtYjExY2ZiYWIxMzNiIiwidCI6IjVmZWJjNjlmLThlOWMtNDcwOC1iNzBlLWQ4YzYyYmUxODA1YiIsImMiOjEwfQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-04-21</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>11:15:06</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>2026-04-21</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>EGAT6</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>การลงทุนตามหลักศาสนาอิสลาม (EGAT-6)</t>
+        </is>
+      </c>
+      <c r="F18" t="n">
+        <v>11.58222352728334</v>
+      </c>
+      <c r="G18" t="n">
+        <v>2.107107625886773</v>
+      </c>
+      <c r="H18" t="n">
+        <v>17.40960103885576</v>
+      </c>
+      <c r="I18" t="inlineStr">
         <is>
           <t>https://app.powerbi.com/view?r=eyJrIjoiMzZjYWU3YmQtNWQ1Ny00NjdjLWI1MmEtYjExY2ZiYWIxMzNiIiwidCI6IjVmZWJjNjlmLThlOWMtNDcwOC1iNzBlLWQ4YzYyYmUxODA1YiIsImMiOjEwfQ%3D%3D</t>
         </is>
@@ -6105,10 +6351,10 @@
         </is>
       </c>
       <c r="B22" s="35" t="n">
-        <v>7.974977740615031</v>
+        <v>7.974977740615032</v>
       </c>
       <c r="C22" s="35" t="n">
-        <v>0.463566454544825</v>
+        <v>0.4635664545448259</v>
       </c>
       <c r="D22" s="35" t="n">
         <v>0.3185044303538165</v>
@@ -6123,7 +6369,7 @@
         <v>17.88447939984901</v>
       </c>
       <c r="H22" s="36" t="n">
-        <v>-0.03746299082865434</v>
+        <v>-0.03746299082865079</v>
       </c>
       <c r="I22" s="19" t="n">
         <v>40.00968825655211</v>
@@ -6159,7 +6405,7 @@
         <v>17.56541815026234</v>
       </c>
       <c r="T22" s="35" t="n">
-        <v>0.1799076732326839</v>
+        <v>0.1799076732326874</v>
       </c>
       <c r="U22" s="19" t="n">
         <v>11.59759457528724</v>
@@ -6171,26 +6417,66 @@
           <t>21/4/69</t>
         </is>
       </c>
-      <c r="B23" s="33" t="n"/>
-      <c r="C23" s="33" t="n"/>
-      <c r="D23" s="33" t="n"/>
-      <c r="E23" s="33" t="n"/>
-      <c r="F23" s="12" t="n"/>
-      <c r="G23" s="33" t="n"/>
-      <c r="H23" s="33" t="n"/>
-      <c r="I23" s="12" t="n"/>
-      <c r="J23" s="33" t="n"/>
-      <c r="K23" s="33" t="n"/>
-      <c r="L23" s="12" t="n"/>
-      <c r="M23" s="33" t="n"/>
-      <c r="N23" s="33" t="n"/>
-      <c r="O23" s="12" t="n"/>
-      <c r="P23" s="33" t="n"/>
-      <c r="Q23" s="33" t="n"/>
-      <c r="R23" s="12" t="n"/>
-      <c r="S23" s="33" t="n"/>
-      <c r="T23" s="33" t="n"/>
-      <c r="U23" s="12" t="n"/>
+      <c r="B23" s="35" t="n">
+        <v>8.070187213655625</v>
+      </c>
+      <c r="C23" s="35" t="n">
+        <v>0.09520947304059391</v>
+      </c>
+      <c r="D23" s="35" t="n">
+        <v>0.3618021344736988</v>
+      </c>
+      <c r="E23" s="35" t="n">
+        <v>0.04329770411988232</v>
+      </c>
+      <c r="F23" s="19" t="n">
+        <v>15.76333906599318</v>
+      </c>
+      <c r="G23" s="35" t="n">
+        <v>18.43423938672446</v>
+      </c>
+      <c r="H23" s="35" t="n">
+        <v>0.5497599868754506</v>
+      </c>
+      <c r="I23" s="19" t="n">
+        <v>40.19627537813753</v>
+      </c>
+      <c r="J23" s="35" t="n">
+        <v>2.120780380148246</v>
+      </c>
+      <c r="K23" s="35" t="n">
+        <v>0.8250787031808482</v>
+      </c>
+      <c r="L23" s="19" t="n">
+        <v>8.835116823464528</v>
+      </c>
+      <c r="M23" s="35" t="n">
+        <v>4.486588098443733</v>
+      </c>
+      <c r="N23" s="36" t="n">
+        <v>-0.3230971381418479</v>
+      </c>
+      <c r="O23" s="19" t="n">
+        <v>7.538702486380125</v>
+      </c>
+      <c r="P23" s="35" t="n">
+        <v>5.608112243287855</v>
+      </c>
+      <c r="Q23" s="36" t="n">
+        <v>-0.3679653063841881</v>
+      </c>
+      <c r="R23" s="19" t="n">
+        <v>16.0564065155152</v>
+      </c>
+      <c r="S23" s="35" t="n">
+        <v>17.40960103885576</v>
+      </c>
+      <c r="T23" s="36" t="n">
+        <v>-0.1558171114065772</v>
+      </c>
+      <c r="U23" s="19" t="n">
+        <v>11.58222352728334</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="10" t="inlineStr">
@@ -6482,14 +6768,14 @@
       </c>
       <c r="B1" s="4" t="inlineStr">
         <is>
-          <t>20 เม.ย. 69 (จันทร์)</t>
+          <t>21 เม.ย. 69 (อังคาร)</t>
         </is>
       </c>
       <c r="C1" s="20" t="n"/>
       <c r="D1" s="20" t="n"/>
       <c r="E1" s="21" t="inlineStr">
         <is>
-          <t>17 เม.ย. 69 (ศุกร์)</t>
+          <t>20 เม.ย. 69 (จันทร์)</t>
         </is>
       </c>
       <c r="F1" s="20" t="n"/>
@@ -6552,27 +6838,27 @@
       <c r="G3" s="20" t="n"/>
       <c r="H3" s="22" t="inlineStr">
         <is>
+          <t>21/4/69</t>
+        </is>
+      </c>
+      <c r="I3" s="22" t="inlineStr">
+        <is>
           <t>20/4/69</t>
         </is>
       </c>
-      <c r="I3" s="22" t="inlineStr">
+      <c r="J3" s="22" t="inlineStr">
         <is>
           <t>17/4/69</t>
         </is>
       </c>
-      <c r="J3" s="22" t="inlineStr">
+      <c r="K3" s="22" t="inlineStr">
         <is>
           <t>16/4/69</t>
         </is>
       </c>
-      <c r="K3" s="22" t="inlineStr">
+      <c r="L3" s="22" t="inlineStr">
         <is>
           <t>10/4/69</t>
-        </is>
-      </c>
-      <c r="L3" s="22" t="inlineStr">
-        <is>
-          <t>9/4/69</t>
         </is>
       </c>
     </row>
@@ -6583,37 +6869,37 @@
         </is>
       </c>
       <c r="B4" s="39" t="n">
+        <v>0.3618021344736988</v>
+      </c>
+      <c r="C4" s="39" t="n">
+        <v>0.04329770411988232</v>
+      </c>
+      <c r="D4" s="26" t="n">
+        <v>15.76333906599318</v>
+      </c>
+      <c r="E4" s="39" t="n">
         <v>0.3185044303538165</v>
       </c>
-      <c r="C4" s="37" t="n">
+      <c r="F4" s="37" t="n">
         <v>-0.0685404498176112</v>
       </c>
-      <c r="D4" s="26" t="n">
+      <c r="G4" s="26" t="n">
         <v>15.75653850665382</v>
       </c>
-      <c r="E4" s="39" t="n">
+      <c r="H4" s="39" t="n">
+        <v>0.3618021344736988</v>
+      </c>
+      <c r="I4" s="39" t="n">
+        <v>0.3185044303538165</v>
+      </c>
+      <c r="J4" s="39" t="n">
         <v>0.3870448801714277</v>
       </c>
-      <c r="F4" s="39" t="n">
-        <v>0.002405161073282258</v>
-      </c>
-      <c r="G4" s="26" t="n">
-        <v>15.76730382101877</v>
-      </c>
-      <c r="H4" s="39" t="n">
-        <v>0.3185044303538165</v>
-      </c>
-      <c r="I4" s="39" t="n">
-        <v>0.3870448801714277</v>
-      </c>
-      <c r="J4" s="39" t="n">
+      <c r="K4" s="39" t="n">
         <v>0.3846397190981454</v>
       </c>
-      <c r="K4" s="39" t="n">
+      <c r="L4" s="39" t="n">
         <v>0.3059192330578275</v>
-      </c>
-      <c r="L4" s="39" t="n">
-        <v>0.3081397169595324</v>
       </c>
     </row>
     <row r="5">
@@ -6623,37 +6909,37 @@
         </is>
       </c>
       <c r="B5" s="39" t="n">
+        <v>18.43423938672446</v>
+      </c>
+      <c r="C5" s="39" t="n">
+        <v>0.5497599868754506</v>
+      </c>
+      <c r="D5" s="26" t="n">
+        <v>40.19627537813753</v>
+      </c>
+      <c r="E5" s="39" t="n">
         <v>17.88447939984901</v>
       </c>
-      <c r="C5" s="37" t="n">
-        <v>-0.03746299082865434</v>
-      </c>
-      <c r="D5" s="26" t="n">
+      <c r="F5" s="37" t="n">
+        <v>-0.03746299082865079</v>
+      </c>
+      <c r="G5" s="26" t="n">
         <v>40.00968825655211</v>
       </c>
-      <c r="E5" s="39" t="n">
+      <c r="H5" s="39" t="n">
+        <v>18.43423938672446</v>
+      </c>
+      <c r="I5" s="39" t="n">
+        <v>17.88447939984901</v>
+      </c>
+      <c r="J5" s="39" t="n">
         <v>17.92194239067766</v>
       </c>
-      <c r="F5" s="37" t="n">
-        <v>-0.7786754987894682</v>
-      </c>
-      <c r="G5" s="26" t="n">
-        <v>40.0224030990135</v>
-      </c>
-      <c r="H5" s="39" t="n">
-        <v>17.88447939984901</v>
-      </c>
-      <c r="I5" s="39" t="n">
-        <v>17.92194239067766</v>
-      </c>
-      <c r="J5" s="39" t="n">
+      <c r="K5" s="39" t="n">
         <v>18.70061788946713</v>
       </c>
-      <c r="K5" s="39" t="n">
+      <c r="L5" s="39" t="n">
         <v>19.65691544253829</v>
-      </c>
-      <c r="L5" s="39" t="n">
-        <v>18.34818846210358</v>
       </c>
     </row>
     <row r="6">
@@ -6663,37 +6949,37 @@
         </is>
       </c>
       <c r="B6" s="39" t="n">
+        <v>2.120780380148246</v>
+      </c>
+      <c r="C6" s="39" t="n">
+        <v>0.8250787031808482</v>
+      </c>
+      <c r="D6" s="26" t="n">
+        <v>8.835116823464528</v>
+      </c>
+      <c r="E6" s="39" t="n">
         <v>1.295701676967398</v>
       </c>
-      <c r="C6" s="37" t="n">
+      <c r="F6" s="37" t="n">
         <v>-0.1045664927917132</v>
       </c>
-      <c r="D6" s="26" t="n">
+      <c r="G6" s="26" t="n">
         <v>8.763734028464144</v>
       </c>
-      <c r="E6" s="39" t="n">
+      <c r="H6" s="39" t="n">
+        <v>2.120780380148246</v>
+      </c>
+      <c r="I6" s="39" t="n">
+        <v>1.295701676967398</v>
+      </c>
+      <c r="J6" s="39" t="n">
         <v>1.400268169759111</v>
       </c>
-      <c r="F6" s="39" t="n">
-        <v>0.7008617568434514</v>
-      </c>
-      <c r="G6" s="26" t="n">
-        <v>8.772780739390125</v>
-      </c>
-      <c r="H6" s="39" t="n">
-        <v>1.295701676967398</v>
-      </c>
-      <c r="I6" s="39" t="n">
-        <v>1.400268169759111</v>
-      </c>
-      <c r="J6" s="39" t="n">
+      <c r="K6" s="39" t="n">
         <v>0.6994064129156596</v>
       </c>
-      <c r="K6" s="39" t="n">
+      <c r="L6" s="39" t="n">
         <v>0.1633313407210846</v>
-      </c>
-      <c r="L6" s="37" t="n">
-        <v>-0.03242462288043368</v>
       </c>
     </row>
     <row r="7">
@@ -6703,37 +6989,37 @@
         </is>
       </c>
       <c r="B7" s="39" t="n">
+        <v>4.486588098443733</v>
+      </c>
+      <c r="C7" s="37" t="n">
+        <v>-0.3230971381418479</v>
+      </c>
+      <c r="D7" s="26" t="n">
+        <v>7.538702486380125</v>
+      </c>
+      <c r="E7" s="39" t="n">
         <v>4.809685236585581</v>
       </c>
-      <c r="C7" s="39" t="n">
+      <c r="F7" s="39" t="n">
         <v>1.381780220684914</v>
       </c>
-      <c r="D7" s="26" t="n">
+      <c r="G7" s="26" t="n">
         <v>7.562013929915418</v>
       </c>
-      <c r="E7" s="39" t="n">
+      <c r="H7" s="39" t="n">
+        <v>4.486588098443733</v>
+      </c>
+      <c r="I7" s="39" t="n">
+        <v>4.809685236585581</v>
+      </c>
+      <c r="J7" s="39" t="n">
         <v>3.427905015900667</v>
       </c>
-      <c r="F7" s="39" t="n">
-        <v>0.6638080360317868</v>
-      </c>
-      <c r="G7" s="26" t="n">
-        <v>7.462318551064556</v>
-      </c>
-      <c r="H7" s="39" t="n">
-        <v>4.809685236585581</v>
-      </c>
-      <c r="I7" s="39" t="n">
-        <v>3.427905015900667</v>
-      </c>
-      <c r="J7" s="39" t="n">
+      <c r="K7" s="39" t="n">
         <v>2.76409697986888</v>
       </c>
-      <c r="K7" s="39" t="n">
+      <c r="L7" s="39" t="n">
         <v>0.4125676530066569</v>
-      </c>
-      <c r="L7" s="37" t="n">
-        <v>-0.08536240871025447</v>
       </c>
     </row>
     <row r="8">
@@ -6743,37 +7029,37 @@
         </is>
       </c>
       <c r="B8" s="39" t="n">
+        <v>5.608112243287855</v>
+      </c>
+      <c r="C8" s="37" t="n">
+        <v>-0.3679653063841881</v>
+      </c>
+      <c r="D8" s="26" t="n">
+        <v>16.0564065155152</v>
+      </c>
+      <c r="E8" s="39" t="n">
         <v>5.976077549672043</v>
       </c>
-      <c r="C8" s="39" t="n">
+      <c r="F8" s="39" t="n">
         <v>1.430280766789327</v>
       </c>
-      <c r="D8" s="26" t="n">
+      <c r="G8" s="26" t="n">
         <v>16.11235108660363</v>
       </c>
-      <c r="E8" s="39" t="n">
+      <c r="H8" s="39" t="n">
+        <v>5.608112243287855</v>
+      </c>
+      <c r="I8" s="39" t="n">
+        <v>5.976077549672043</v>
+      </c>
+      <c r="J8" s="39" t="n">
         <v>4.545796782882716</v>
       </c>
-      <c r="F8" s="39" t="n">
-        <v>0.1972298212562515</v>
-      </c>
-      <c r="G8" s="26" t="n">
-        <v>15.89489459642429</v>
-      </c>
-      <c r="H8" s="39" t="n">
-        <v>5.976077549672043</v>
-      </c>
-      <c r="I8" s="39" t="n">
-        <v>4.545796782882716</v>
-      </c>
-      <c r="J8" s="39" t="n">
+      <c r="K8" s="39" t="n">
         <v>4.348566961626465</v>
       </c>
-      <c r="K8" s="39" t="n">
+      <c r="L8" s="39" t="n">
         <v>2.229117414847503</v>
-      </c>
-      <c r="L8" s="39" t="n">
-        <v>1.678283928945601</v>
       </c>
     </row>
     <row r="9">
@@ -6783,37 +7069,37 @@
         </is>
       </c>
       <c r="B9" s="39" t="n">
+        <v>17.40960103885576</v>
+      </c>
+      <c r="C9" s="37" t="n">
+        <v>-0.1558171114065772</v>
+      </c>
+      <c r="D9" s="26" t="n">
+        <v>11.58222352728334</v>
+      </c>
+      <c r="E9" s="39" t="n">
         <v>17.56541815026234</v>
       </c>
-      <c r="C9" s="39" t="n">
-        <v>0.1799076732326839</v>
-      </c>
-      <c r="D9" s="26" t="n">
+      <c r="F9" s="39" t="n">
+        <v>0.1799076732326874</v>
+      </c>
+      <c r="G9" s="26" t="n">
         <v>11.59759457528724</v>
       </c>
-      <c r="E9" s="39" t="n">
+      <c r="H9" s="39" t="n">
+        <v>17.40960103885576</v>
+      </c>
+      <c r="I9" s="39" t="n">
+        <v>17.56541815026234</v>
+      </c>
+      <c r="J9" s="39" t="n">
         <v>17.38551047702965</v>
       </c>
-      <c r="F9" s="37" t="n">
-        <v>-0.3030672477159797</v>
-      </c>
-      <c r="G9" s="26" t="n">
-        <v>11.57984704129328</v>
-      </c>
-      <c r="H9" s="39" t="n">
-        <v>17.56541815026234</v>
-      </c>
-      <c r="I9" s="39" t="n">
-        <v>17.38551047702965</v>
-      </c>
-      <c r="J9" s="39" t="n">
+      <c r="K9" s="39" t="n">
         <v>17.68857772474563</v>
       </c>
-      <c r="K9" s="39" t="n">
+      <c r="L9" s="39" t="n">
         <v>19.48146125653116</v>
-      </c>
-      <c r="L9" s="39" t="n">
-        <v>17.74511202907099</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
EGAT retirement pages update 2026-04-24T04:15:06Z
</commit_message>
<xml_diff>
--- a/EGAT Retirement.xlsx
+++ b/EGAT Retirement.xlsx
@@ -683,7 +683,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I18"/>
+  <dimension ref="A1:I19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1440,6 +1440,47 @@
         </is>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>11:15:05</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>EGAT1</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>ตราสารหนี้ (EGAT-1)</t>
+        </is>
+      </c>
+      <c r="F19" t="n">
+        <v>15.75867722946711</v>
+      </c>
+      <c r="G19" t="n">
+        <v>0.6217971938575317</v>
+      </c>
+      <c r="H19" t="n">
+        <v>0.3321212202299417</v>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>https://app.powerbi.com/view?r=eyJrIjoiMzZjYWU3YmQtNWQ1Ny00NjdjLWI1MmEtYjExY2ZiYWIxMzNiIiwidCI6IjVmZWJjNjlmLThlOWMtNDcwOC1iNzBlLWQ4YzYyYmUxODA1YiIsImMiOjEwfQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1451,7 +1492,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I18"/>
+  <dimension ref="A1:I19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -2208,6 +2249,47 @@
         </is>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>11:15:05</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>EGAT2</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>ตราสารทุน (EGAT-2)</t>
+        </is>
+      </c>
+      <c r="F19" t="n">
+        <v>40.13137454284129</v>
+      </c>
+      <c r="G19" t="n">
+        <v>2.63793673390893</v>
+      </c>
+      <c r="H19" t="n">
+        <v>18.24301567279665</v>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>https://app.powerbi.com/view?r=eyJrIjoiMzZjYWU3YmQtNWQ1Ny00NjdjLWI1MmEtYjExY2ZiYWIxMzNiIiwidCI6IjVmZWJjNjlmLThlOWMtNDcwOC1iNzBlLWQ4YzYyYmUxODA1YiIsImMiOjEwfQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2219,7 +2301,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I18"/>
+  <dimension ref="A1:I19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -2976,6 +3058,47 @@
         </is>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>11:15:05</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>EGAT3</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>อสังหาริมทรัพย์และโครงสร้างพื้นฐาน (EGAT-3)</t>
+        </is>
+      </c>
+      <c r="F19" t="n">
+        <v>8.834228099454517</v>
+      </c>
+      <c r="G19" t="n">
+        <v>4.987326190894037</v>
+      </c>
+      <c r="H19" t="n">
+        <v>2.110508055372207</v>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>https://app.powerbi.com/view?r=eyJrIjoiMzZjYWU3YmQtNWQ1Ny00NjdjLWI1MmEtYjExY2ZiYWIxMzNiIiwidCI6IjVmZWJjNjlmLThlOWMtNDcwOC1iNzBlLWQ4YzYyYmUxODA1YiIsImMiOjEwfQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2987,7 +3110,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I18"/>
+  <dimension ref="A1:I19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -3744,6 +3867,47 @@
         </is>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>11:15:05</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>EGAT4</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>ตราสารทุนต่างประเทศ (EGAT-4)</t>
+        </is>
+      </c>
+      <c r="F19" t="n">
+        <v>7.478054519319542</v>
+      </c>
+      <c r="G19" t="n">
+        <v>10.29089585383867</v>
+      </c>
+      <c r="H19" t="n">
+        <v>3.646005894183024</v>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>https://app.powerbi.com/view?r=eyJrIjoiMzZjYWU3YmQtNWQ1Ny00NjdjLWI1MmEtYjExY2ZiYWIxMzNiIiwidCI6IjVmZWJjNjlmLThlOWMtNDcwOC1iNzBlLWQ4YzYyYmUxODA1YiIsImMiOjEwfQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3755,7 +3919,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I18"/>
+  <dimension ref="A1:I19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -4512,6 +4676,47 @@
         </is>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>11:15:05</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>EGAT5</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>ตราสารทุนต่างประเทศแบบอิงดัชนี (EGAT-5)</t>
+        </is>
+      </c>
+      <c r="F19" t="n">
+        <v>15.89876204778846</v>
+      </c>
+      <c r="G19" t="n">
+        <v>9.44693707227502</v>
+      </c>
+      <c r="H19" t="n">
+        <v>4.571234245329148</v>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>https://app.powerbi.com/view?r=eyJrIjoiMzZjYWU3YmQtNWQ1Ny00NjdjLWI1MmEtYjExY2ZiYWIxMzNiIiwidCI6IjVmZWJjNjlmLThlOWMtNDcwOC1iNzBlLWQ4YzYyYmUxODA1YiIsImMiOjEwfQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4523,7 +4728,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I18"/>
+  <dimension ref="A1:I19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -5275,6 +5480,47 @@
         <v>17.40960103885576</v>
       </c>
       <c r="I18" t="inlineStr">
+        <is>
+          <t>https://app.powerbi.com/view?r=eyJrIjoiMzZjYWU3YmQtNWQ1Ny00NjdjLWI1MmEtYjExY2ZiYWIxMzNiIiwidCI6IjVmZWJjNjlmLThlOWMtNDcwOC1iNzBlLWQ4YzYyYmUxODA1YiIsImMiOjEwfQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>11:15:05</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>EGAT6</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>การลงทุนตามหลักศาสนาอิสลาม (EGAT-6)</t>
+        </is>
+      </c>
+      <c r="F19" t="n">
+        <v>11.58407269044301</v>
+      </c>
+      <c r="G19" t="n">
+        <v>2.123409564915812</v>
+      </c>
+      <c r="H19" t="n">
+        <v>17.42834610178099</v>
+      </c>
+      <c r="I19" t="inlineStr">
         <is>
           <t>https://app.powerbi.com/view?r=eyJrIjoiMzZjYWU3YmQtNWQ1Ny00NjdjLWI1MmEtYjExY2ZiYWIxMzNiIiwidCI6IjVmZWJjNjlmLThlOWMtNDcwOC1iNzBlLWQ4YzYyYmUxODA1YiIsImMiOjEwfQ%3D%3D</t>
         </is>
@@ -6484,26 +6730,66 @@
           <t>22/4/69</t>
         </is>
       </c>
-      <c r="B24" s="33" t="n"/>
-      <c r="C24" s="33" t="n"/>
-      <c r="D24" s="33" t="n"/>
-      <c r="E24" s="33" t="n"/>
-      <c r="F24" s="12" t="n"/>
-      <c r="G24" s="33" t="n"/>
-      <c r="H24" s="33" t="n"/>
-      <c r="I24" s="12" t="n"/>
-      <c r="J24" s="33" t="n"/>
-      <c r="K24" s="33" t="n"/>
-      <c r="L24" s="12" t="n"/>
-      <c r="M24" s="33" t="n"/>
-      <c r="N24" s="33" t="n"/>
-      <c r="O24" s="12" t="n"/>
-      <c r="P24" s="33" t="n"/>
-      <c r="Q24" s="33" t="n"/>
-      <c r="R24" s="12" t="n"/>
-      <c r="S24" s="33" t="n"/>
-      <c r="T24" s="33" t="n"/>
-      <c r="U24" s="12" t="n"/>
+      <c r="B24" s="35" t="n">
+        <v>7.72187186494866</v>
+      </c>
+      <c r="C24" s="36" t="n">
+        <v>-0.3483153487069659</v>
+      </c>
+      <c r="D24" s="35" t="n">
+        <v>0.3321212202299417</v>
+      </c>
+      <c r="E24" s="36" t="n">
+        <v>-0.02968091424375707</v>
+      </c>
+      <c r="F24" s="19" t="n">
+        <v>15.75867722946711</v>
+      </c>
+      <c r="G24" s="35" t="n">
+        <v>18.24301567279665</v>
+      </c>
+      <c r="H24" s="36" t="n">
+        <v>-0.1912237139278119</v>
+      </c>
+      <c r="I24" s="19" t="n">
+        <v>40.13137454284129</v>
+      </c>
+      <c r="J24" s="35" t="n">
+        <v>2.110508055372207</v>
+      </c>
+      <c r="K24" s="36" t="n">
+        <v>-0.01027232477603945</v>
+      </c>
+      <c r="L24" s="19" t="n">
+        <v>8.834228099454517</v>
+      </c>
+      <c r="M24" s="35" t="n">
+        <v>3.646005894183024</v>
+      </c>
+      <c r="N24" s="36" t="n">
+        <v>-0.8405822042607092</v>
+      </c>
+      <c r="O24" s="19" t="n">
+        <v>7.478054519319542</v>
+      </c>
+      <c r="P24" s="35" t="n">
+        <v>4.571234245329148</v>
+      </c>
+      <c r="Q24" s="36" t="n">
+        <v>-1.036877997958707</v>
+      </c>
+      <c r="R24" s="19" t="n">
+        <v>15.89876204778846</v>
+      </c>
+      <c r="S24" s="35" t="n">
+        <v>17.42834610178099</v>
+      </c>
+      <c r="T24" s="35" t="n">
+        <v>0.01874506292522682</v>
+      </c>
+      <c r="U24" s="19" t="n">
+        <v>11.58407269044301</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="10" t="inlineStr">
@@ -6768,14 +7054,14 @@
       </c>
       <c r="B1" s="4" t="inlineStr">
         <is>
-          <t>21 เม.ย. 69 (อังคาร)</t>
+          <t>22 เม.ย. 69 (พุธ)</t>
         </is>
       </c>
       <c r="C1" s="20" t="n"/>
       <c r="D1" s="20" t="n"/>
       <c r="E1" s="21" t="inlineStr">
         <is>
-          <t>20 เม.ย. 69 (จันทร์)</t>
+          <t>21 เม.ย. 69 (อังคาร)</t>
         </is>
       </c>
       <c r="F1" s="20" t="n"/>
@@ -6838,27 +7124,27 @@
       <c r="G3" s="20" t="n"/>
       <c r="H3" s="22" t="inlineStr">
         <is>
+          <t>22/4/69</t>
+        </is>
+      </c>
+      <c r="I3" s="22" t="inlineStr">
+        <is>
           <t>21/4/69</t>
         </is>
       </c>
-      <c r="I3" s="22" t="inlineStr">
+      <c r="J3" s="22" t="inlineStr">
         <is>
           <t>20/4/69</t>
         </is>
       </c>
-      <c r="J3" s="22" t="inlineStr">
+      <c r="K3" s="22" t="inlineStr">
         <is>
           <t>17/4/69</t>
         </is>
       </c>
-      <c r="K3" s="22" t="inlineStr">
+      <c r="L3" s="22" t="inlineStr">
         <is>
           <t>16/4/69</t>
-        </is>
-      </c>
-      <c r="L3" s="22" t="inlineStr">
-        <is>
-          <t>10/4/69</t>
         </is>
       </c>
     </row>
@@ -6869,37 +7155,37 @@
         </is>
       </c>
       <c r="B4" s="39" t="n">
+        <v>0.3321212202299417</v>
+      </c>
+      <c r="C4" s="37" t="n">
+        <v>-0.02968091424375707</v>
+      </c>
+      <c r="D4" s="26" t="n">
+        <v>15.75867722946711</v>
+      </c>
+      <c r="E4" s="39" t="n">
         <v>0.3618021344736988</v>
       </c>
-      <c r="C4" s="39" t="n">
+      <c r="F4" s="39" t="n">
         <v>0.04329770411988232</v>
       </c>
-      <c r="D4" s="26" t="n">
+      <c r="G4" s="26" t="n">
         <v>15.76333906599318</v>
       </c>
-      <c r="E4" s="39" t="n">
+      <c r="H4" s="39" t="n">
+        <v>0.3321212202299417</v>
+      </c>
+      <c r="I4" s="39" t="n">
+        <v>0.3618021344736988</v>
+      </c>
+      <c r="J4" s="39" t="n">
         <v>0.3185044303538165</v>
       </c>
-      <c r="F4" s="37" t="n">
-        <v>-0.0685404498176112</v>
-      </c>
-      <c r="G4" s="26" t="n">
-        <v>15.75653850665382</v>
-      </c>
-      <c r="H4" s="39" t="n">
-        <v>0.3618021344736988</v>
-      </c>
-      <c r="I4" s="39" t="n">
-        <v>0.3185044303538165</v>
-      </c>
-      <c r="J4" s="39" t="n">
+      <c r="K4" s="39" t="n">
         <v>0.3870448801714277</v>
       </c>
-      <c r="K4" s="39" t="n">
+      <c r="L4" s="39" t="n">
         <v>0.3846397190981454</v>
-      </c>
-      <c r="L4" s="39" t="n">
-        <v>0.3059192330578275</v>
       </c>
     </row>
     <row r="5">
@@ -6909,37 +7195,37 @@
         </is>
       </c>
       <c r="B5" s="39" t="n">
+        <v>18.24301567279665</v>
+      </c>
+      <c r="C5" s="37" t="n">
+        <v>-0.1912237139278119</v>
+      </c>
+      <c r="D5" s="26" t="n">
+        <v>40.13137454284129</v>
+      </c>
+      <c r="E5" s="39" t="n">
         <v>18.43423938672446</v>
       </c>
-      <c r="C5" s="39" t="n">
+      <c r="F5" s="39" t="n">
         <v>0.5497599868754506</v>
       </c>
-      <c r="D5" s="26" t="n">
+      <c r="G5" s="26" t="n">
         <v>40.19627537813753</v>
       </c>
-      <c r="E5" s="39" t="n">
+      <c r="H5" s="39" t="n">
+        <v>18.24301567279665</v>
+      </c>
+      <c r="I5" s="39" t="n">
+        <v>18.43423938672446</v>
+      </c>
+      <c r="J5" s="39" t="n">
         <v>17.88447939984901</v>
       </c>
-      <c r="F5" s="37" t="n">
-        <v>-0.03746299082865079</v>
-      </c>
-      <c r="G5" s="26" t="n">
-        <v>40.00968825655211</v>
-      </c>
-      <c r="H5" s="39" t="n">
-        <v>18.43423938672446</v>
-      </c>
-      <c r="I5" s="39" t="n">
-        <v>17.88447939984901</v>
-      </c>
-      <c r="J5" s="39" t="n">
+      <c r="K5" s="39" t="n">
         <v>17.92194239067766</v>
       </c>
-      <c r="K5" s="39" t="n">
+      <c r="L5" s="39" t="n">
         <v>18.70061788946713</v>
-      </c>
-      <c r="L5" s="39" t="n">
-        <v>19.65691544253829</v>
       </c>
     </row>
     <row r="6">
@@ -6949,37 +7235,37 @@
         </is>
       </c>
       <c r="B6" s="39" t="n">
+        <v>2.110508055372207</v>
+      </c>
+      <c r="C6" s="37" t="n">
+        <v>-0.01027232477603945</v>
+      </c>
+      <c r="D6" s="26" t="n">
+        <v>8.834228099454517</v>
+      </c>
+      <c r="E6" s="39" t="n">
         <v>2.120780380148246</v>
       </c>
-      <c r="C6" s="39" t="n">
+      <c r="F6" s="39" t="n">
         <v>0.8250787031808482</v>
       </c>
-      <c r="D6" s="26" t="n">
+      <c r="G6" s="26" t="n">
         <v>8.835116823464528</v>
       </c>
-      <c r="E6" s="39" t="n">
+      <c r="H6" s="39" t="n">
+        <v>2.110508055372207</v>
+      </c>
+      <c r="I6" s="39" t="n">
+        <v>2.120780380148246</v>
+      </c>
+      <c r="J6" s="39" t="n">
         <v>1.295701676967398</v>
       </c>
-      <c r="F6" s="37" t="n">
-        <v>-0.1045664927917132</v>
-      </c>
-      <c r="G6" s="26" t="n">
-        <v>8.763734028464144</v>
-      </c>
-      <c r="H6" s="39" t="n">
-        <v>2.120780380148246</v>
-      </c>
-      <c r="I6" s="39" t="n">
-        <v>1.295701676967398</v>
-      </c>
-      <c r="J6" s="39" t="n">
+      <c r="K6" s="39" t="n">
         <v>1.400268169759111</v>
       </c>
-      <c r="K6" s="39" t="n">
+      <c r="L6" s="39" t="n">
         <v>0.6994064129156596</v>
-      </c>
-      <c r="L6" s="39" t="n">
-        <v>0.1633313407210846</v>
       </c>
     </row>
     <row r="7">
@@ -6989,37 +7275,37 @@
         </is>
       </c>
       <c r="B7" s="39" t="n">
+        <v>3.646005894183024</v>
+      </c>
+      <c r="C7" s="37" t="n">
+        <v>-0.8405822042607092</v>
+      </c>
+      <c r="D7" s="26" t="n">
+        <v>7.478054519319542</v>
+      </c>
+      <c r="E7" s="39" t="n">
         <v>4.486588098443733</v>
       </c>
-      <c r="C7" s="37" t="n">
+      <c r="F7" s="37" t="n">
         <v>-0.3230971381418479</v>
       </c>
-      <c r="D7" s="26" t="n">
+      <c r="G7" s="26" t="n">
         <v>7.538702486380125</v>
       </c>
-      <c r="E7" s="39" t="n">
+      <c r="H7" s="39" t="n">
+        <v>3.646005894183024</v>
+      </c>
+      <c r="I7" s="39" t="n">
+        <v>4.486588098443733</v>
+      </c>
+      <c r="J7" s="39" t="n">
         <v>4.809685236585581</v>
       </c>
-      <c r="F7" s="39" t="n">
-        <v>1.381780220684914</v>
-      </c>
-      <c r="G7" s="26" t="n">
-        <v>7.562013929915418</v>
-      </c>
-      <c r="H7" s="39" t="n">
-        <v>4.486588098443733</v>
-      </c>
-      <c r="I7" s="39" t="n">
-        <v>4.809685236585581</v>
-      </c>
-      <c r="J7" s="39" t="n">
+      <c r="K7" s="39" t="n">
         <v>3.427905015900667</v>
       </c>
-      <c r="K7" s="39" t="n">
+      <c r="L7" s="39" t="n">
         <v>2.76409697986888</v>
-      </c>
-      <c r="L7" s="39" t="n">
-        <v>0.4125676530066569</v>
       </c>
     </row>
     <row r="8">
@@ -7029,37 +7315,37 @@
         </is>
       </c>
       <c r="B8" s="39" t="n">
+        <v>4.571234245329148</v>
+      </c>
+      <c r="C8" s="37" t="n">
+        <v>-1.036877997958707</v>
+      </c>
+      <c r="D8" s="26" t="n">
+        <v>15.89876204778846</v>
+      </c>
+      <c r="E8" s="39" t="n">
         <v>5.608112243287855</v>
       </c>
-      <c r="C8" s="37" t="n">
+      <c r="F8" s="37" t="n">
         <v>-0.3679653063841881</v>
       </c>
-      <c r="D8" s="26" t="n">
+      <c r="G8" s="26" t="n">
         <v>16.0564065155152</v>
       </c>
-      <c r="E8" s="39" t="n">
+      <c r="H8" s="39" t="n">
+        <v>4.571234245329148</v>
+      </c>
+      <c r="I8" s="39" t="n">
+        <v>5.608112243287855</v>
+      </c>
+      <c r="J8" s="39" t="n">
         <v>5.976077549672043</v>
       </c>
-      <c r="F8" s="39" t="n">
-        <v>1.430280766789327</v>
-      </c>
-      <c r="G8" s="26" t="n">
-        <v>16.11235108660363</v>
-      </c>
-      <c r="H8" s="39" t="n">
-        <v>5.608112243287855</v>
-      </c>
-      <c r="I8" s="39" t="n">
-        <v>5.976077549672043</v>
-      </c>
-      <c r="J8" s="39" t="n">
+      <c r="K8" s="39" t="n">
         <v>4.545796782882716</v>
       </c>
-      <c r="K8" s="39" t="n">
+      <c r="L8" s="39" t="n">
         <v>4.348566961626465</v>
-      </c>
-      <c r="L8" s="39" t="n">
-        <v>2.229117414847503</v>
       </c>
     </row>
     <row r="9">
@@ -7069,37 +7355,37 @@
         </is>
       </c>
       <c r="B9" s="39" t="n">
+        <v>17.42834610178099</v>
+      </c>
+      <c r="C9" s="39" t="n">
+        <v>0.01874506292522682</v>
+      </c>
+      <c r="D9" s="26" t="n">
+        <v>11.58407269044301</v>
+      </c>
+      <c r="E9" s="39" t="n">
         <v>17.40960103885576</v>
       </c>
-      <c r="C9" s="37" t="n">
+      <c r="F9" s="37" t="n">
         <v>-0.1558171114065772</v>
       </c>
-      <c r="D9" s="26" t="n">
+      <c r="G9" s="26" t="n">
         <v>11.58222352728334</v>
       </c>
-      <c r="E9" s="39" t="n">
+      <c r="H9" s="39" t="n">
+        <v>17.42834610178099</v>
+      </c>
+      <c r="I9" s="39" t="n">
+        <v>17.40960103885576</v>
+      </c>
+      <c r="J9" s="39" t="n">
         <v>17.56541815026234</v>
       </c>
-      <c r="F9" s="39" t="n">
-        <v>0.1799076732326874</v>
-      </c>
-      <c r="G9" s="26" t="n">
-        <v>11.59759457528724</v>
-      </c>
-      <c r="H9" s="39" t="n">
-        <v>17.40960103885576</v>
-      </c>
-      <c r="I9" s="39" t="n">
-        <v>17.56541815026234</v>
-      </c>
-      <c r="J9" s="39" t="n">
+      <c r="K9" s="39" t="n">
         <v>17.38551047702965</v>
       </c>
-      <c r="K9" s="39" t="n">
+      <c r="L9" s="39" t="n">
         <v>17.68857772474563</v>
-      </c>
-      <c r="L9" s="39" t="n">
-        <v>19.48146125653116</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
EGAT retirement pages update 2026-04-27T04:15:07Z
</commit_message>
<xml_diff>
--- a/EGAT Retirement.xlsx
+++ b/EGAT Retirement.xlsx
@@ -683,7 +683,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I19"/>
+  <dimension ref="A1:I20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1481,6 +1481,47 @@
         </is>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-04-23</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>11:15:07</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>2026-04-23</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>EGAT1</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>ตราสารหนี้ (EGAT-1)</t>
+        </is>
+      </c>
+      <c r="F20" t="n">
+        <v>15.75181093537439</v>
+      </c>
+      <c r="G20" t="n">
+        <v>0.5779547544439323</v>
+      </c>
+      <c r="H20" t="n">
+        <v>0.2884049970207636</v>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>https://app.powerbi.com/view?r=eyJrIjoiMzZjYWU3YmQtNWQ1Ny00NjdjLWI1MmEtYjExY2ZiYWIxMzNiIiwidCI6IjVmZWJjNjlmLThlOWMtNDcwOC1iNzBlLWQ4YzYyYmUxODA1YiIsImMiOjEwfQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1492,7 +1533,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I19"/>
+  <dimension ref="A1:I20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -2290,6 +2331,47 @@
         </is>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-04-23</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>11:15:07</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>2026-04-23</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>EGAT2</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>ตราสารทุน (EGAT-2)</t>
+        </is>
+      </c>
+      <c r="F20" t="n">
+        <v>39.67425959738566</v>
+      </c>
+      <c r="G20" t="n">
+        <v>1.468843091185223</v>
+      </c>
+      <c r="H20" t="n">
+        <v>16.89617295246872</v>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>https://app.powerbi.com/view?r=eyJrIjoiMzZjYWU3YmQtNWQ1Ny00NjdjLWI1MmEtYjExY2ZiYWIxMzNiIiwidCI6IjVmZWJjNjlmLThlOWMtNDcwOC1iNzBlLWQ4YzYyYmUxODA1YiIsImMiOjEwfQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2301,7 +2383,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I19"/>
+  <dimension ref="A1:I20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -3099,6 +3181,47 @@
         </is>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-04-23</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>11:15:07</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>2026-04-23</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>EGAT3</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>อสังหาริมทรัพย์และโครงสร้างพื้นฐาน (EGAT-3)</t>
+        </is>
+      </c>
+      <c r="F20" t="n">
+        <v>8.785765996543011</v>
+      </c>
+      <c r="G20" t="n">
+        <v>4.411395102293203</v>
+      </c>
+      <c r="H20" t="n">
+        <v>1.550358385925565</v>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>https://app.powerbi.com/view?r=eyJrIjoiMzZjYWU3YmQtNWQ1Ny00NjdjLWI1MmEtYjExY2ZiYWIxMzNiIiwidCI6IjVmZWJjNjlmLThlOWMtNDcwOC1iNzBlLWQ4YzYyYmUxODA1YiIsImMiOjEwfQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3110,7 +3233,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I19"/>
+  <dimension ref="A1:I20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -3908,6 +4031,47 @@
         </is>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-04-23</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>11:15:07</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>2026-04-23</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>EGAT4</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>ตราสารทุนต่างประเทศ (EGAT-4)</t>
+        </is>
+      </c>
+      <c r="F20" t="n">
+        <v>7.625160270532558</v>
+      </c>
+      <c r="G20" t="n">
+        <v>12.4605009355641</v>
+      </c>
+      <c r="H20" t="n">
+        <v>5.684894955221842</v>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>https://app.powerbi.com/view?r=eyJrIjoiMzZjYWU3YmQtNWQ1Ny00NjdjLWI1MmEtYjExY2ZiYWIxMzNiIiwidCI6IjVmZWJjNjlmLThlOWMtNDcwOC1iNzBlLWQ4YzYyYmUxODA1YiIsImMiOjEwfQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3919,7 +4083,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I19"/>
+  <dimension ref="A1:I20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -4717,6 +4881,47 @@
         </is>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-04-23</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>11:15:07</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>2026-04-23</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>EGAT5</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>ตราสารทุนต่างประเทศแบบอิงดัชนี (EGAT-5)</t>
+        </is>
+      </c>
+      <c r="F20" t="n">
+        <v>16.11731394089035</v>
+      </c>
+      <c r="G20" t="n">
+        <v>10.95144636799572</v>
+      </c>
+      <c r="H20" t="n">
+        <v>6.008719826887177</v>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>https://app.powerbi.com/view?r=eyJrIjoiMzZjYWU3YmQtNWQ1Ny00NjdjLWI1MmEtYjExY2ZiYWIxMzNiIiwidCI6IjVmZWJjNjlmLThlOWMtNDcwOC1iNzBlLWQ4YzYyYmUxODA1YiIsImMiOjEwfQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4728,7 +4933,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I19"/>
+  <dimension ref="A1:I20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -5521,6 +5726,47 @@
         <v>17.42834610178099</v>
       </c>
       <c r="I19" t="inlineStr">
+        <is>
+          <t>https://app.powerbi.com/view?r=eyJrIjoiMzZjYWU3YmQtNWQ1Ny00NjdjLWI1MmEtYjExY2ZiYWIxMzNiIiwidCI6IjVmZWJjNjlmLThlOWMtNDcwOC1iNzBlLWQ4YzYyYmUxODA1YiIsImMiOjEwfQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-04-23</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>11:15:07</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>2026-04-23</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>EGAT6</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>การลงทุนตามหลักศาสนาอิสลาม (EGAT-6)</t>
+        </is>
+      </c>
+      <c r="F20" t="n">
+        <v>11.4991072702717</v>
+      </c>
+      <c r="G20" t="n">
+        <v>1.37436744174535</v>
+      </c>
+      <c r="H20" t="n">
+        <v>16.56704722761286</v>
+      </c>
+      <c r="I20" t="inlineStr">
         <is>
           <t>https://app.powerbi.com/view?r=eyJrIjoiMzZjYWU3YmQtNWQ1Ny00NjdjLWI1MmEtYjExY2ZiYWIxMzNiIiwidCI6IjVmZWJjNjlmLThlOWMtNDcwOC1iNzBlLWQ4YzYyYmUxODA1YiIsImMiOjEwfQ%3D%3D</t>
         </is>
@@ -6758,7 +7004,7 @@
         <v>2.110508055372207</v>
       </c>
       <c r="K24" s="36" t="n">
-        <v>-0.01027232477603945</v>
+        <v>-0.01027232477603901</v>
       </c>
       <c r="L24" s="19" t="n">
         <v>8.834228099454517</v>
@@ -6767,7 +7013,7 @@
         <v>3.646005894183024</v>
       </c>
       <c r="N24" s="36" t="n">
-        <v>-0.8405822042607092</v>
+        <v>-0.8405822042607096</v>
       </c>
       <c r="O24" s="19" t="n">
         <v>7.478054519319542</v>
@@ -6797,26 +7043,66 @@
           <t>23/4/69</t>
         </is>
       </c>
-      <c r="B25" s="33" t="n"/>
-      <c r="C25" s="33" t="n"/>
-      <c r="D25" s="33" t="n"/>
-      <c r="E25" s="33" t="n"/>
-      <c r="F25" s="12" t="n"/>
-      <c r="G25" s="33" t="n"/>
-      <c r="H25" s="33" t="n"/>
-      <c r="I25" s="12" t="n"/>
-      <c r="J25" s="33" t="n"/>
-      <c r="K25" s="33" t="n"/>
-      <c r="L25" s="12" t="n"/>
-      <c r="M25" s="33" t="n"/>
-      <c r="N25" s="33" t="n"/>
-      <c r="O25" s="12" t="n"/>
-      <c r="P25" s="33" t="n"/>
-      <c r="Q25" s="33" t="n"/>
-      <c r="R25" s="12" t="n"/>
-      <c r="S25" s="33" t="n"/>
-      <c r="T25" s="33" t="n"/>
-      <c r="U25" s="12" t="n"/>
+      <c r="B25" s="35" t="n">
+        <v>7.832599724189489</v>
+      </c>
+      <c r="C25" s="35" t="n">
+        <v>0.1107278592408294</v>
+      </c>
+      <c r="D25" s="35" t="n">
+        <v>0.2884049970207636</v>
+      </c>
+      <c r="E25" s="36" t="n">
+        <v>-0.04371622320917812</v>
+      </c>
+      <c r="F25" s="19" t="n">
+        <v>15.75181093537439</v>
+      </c>
+      <c r="G25" s="35" t="n">
+        <v>16.89617295246872</v>
+      </c>
+      <c r="H25" s="36" t="n">
+        <v>-1.346842720327924</v>
+      </c>
+      <c r="I25" s="19" t="n">
+        <v>39.67425959738566</v>
+      </c>
+      <c r="J25" s="35" t="n">
+        <v>1.550358385925565</v>
+      </c>
+      <c r="K25" s="36" t="n">
+        <v>-0.5601496694466417</v>
+      </c>
+      <c r="L25" s="19" t="n">
+        <v>8.785765996543011</v>
+      </c>
+      <c r="M25" s="35" t="n">
+        <v>5.684894955221842</v>
+      </c>
+      <c r="N25" s="35" t="n">
+        <v>2.038889061038818</v>
+      </c>
+      <c r="O25" s="19" t="n">
+        <v>7.625160270532558</v>
+      </c>
+      <c r="P25" s="35" t="n">
+        <v>6.008719826887177</v>
+      </c>
+      <c r="Q25" s="35" t="n">
+        <v>1.437485581558029</v>
+      </c>
+      <c r="R25" s="19" t="n">
+        <v>16.11731394089035</v>
+      </c>
+      <c r="S25" s="35" t="n">
+        <v>16.56704722761286</v>
+      </c>
+      <c r="T25" s="36" t="n">
+        <v>-0.8612988741681242</v>
+      </c>
+      <c r="U25" s="19" t="n">
+        <v>11.4991072702717</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="10" t="inlineStr">
@@ -7054,14 +7340,14 @@
       </c>
       <c r="B1" s="4" t="inlineStr">
         <is>
-          <t>22 เม.ย. 69 (พุธ)</t>
+          <t>23 เม.ย. 69 (พฤหัส)</t>
         </is>
       </c>
       <c r="C1" s="20" t="n"/>
       <c r="D1" s="20" t="n"/>
       <c r="E1" s="21" t="inlineStr">
         <is>
-          <t>21 เม.ย. 69 (อังคาร)</t>
+          <t>22 เม.ย. 69 (พุธ)</t>
         </is>
       </c>
       <c r="F1" s="20" t="n"/>
@@ -7124,27 +7410,27 @@
       <c r="G3" s="20" t="n"/>
       <c r="H3" s="22" t="inlineStr">
         <is>
+          <t>23/4/69</t>
+        </is>
+      </c>
+      <c r="I3" s="22" t="inlineStr">
+        <is>
           <t>22/4/69</t>
         </is>
       </c>
-      <c r="I3" s="22" t="inlineStr">
+      <c r="J3" s="22" t="inlineStr">
         <is>
           <t>21/4/69</t>
         </is>
       </c>
-      <c r="J3" s="22" t="inlineStr">
+      <c r="K3" s="22" t="inlineStr">
         <is>
           <t>20/4/69</t>
         </is>
       </c>
-      <c r="K3" s="22" t="inlineStr">
+      <c r="L3" s="22" t="inlineStr">
         <is>
           <t>17/4/69</t>
-        </is>
-      </c>
-      <c r="L3" s="22" t="inlineStr">
-        <is>
-          <t>16/4/69</t>
         </is>
       </c>
     </row>
@@ -7155,37 +7441,37 @@
         </is>
       </c>
       <c r="B4" s="39" t="n">
+        <v>0.2884049970207636</v>
+      </c>
+      <c r="C4" s="37" t="n">
+        <v>-0.04371622320917812</v>
+      </c>
+      <c r="D4" s="26" t="n">
+        <v>15.75181093537439</v>
+      </c>
+      <c r="E4" s="39" t="n">
         <v>0.3321212202299417</v>
       </c>
-      <c r="C4" s="37" t="n">
+      <c r="F4" s="37" t="n">
         <v>-0.02968091424375707</v>
       </c>
-      <c r="D4" s="26" t="n">
+      <c r="G4" s="26" t="n">
         <v>15.75867722946711</v>
       </c>
-      <c r="E4" s="39" t="n">
+      <c r="H4" s="39" t="n">
+        <v>0.2884049970207636</v>
+      </c>
+      <c r="I4" s="39" t="n">
+        <v>0.3321212202299417</v>
+      </c>
+      <c r="J4" s="39" t="n">
         <v>0.3618021344736988</v>
       </c>
-      <c r="F4" s="39" t="n">
-        <v>0.04329770411988232</v>
-      </c>
-      <c r="G4" s="26" t="n">
-        <v>15.76333906599318</v>
-      </c>
-      <c r="H4" s="39" t="n">
-        <v>0.3321212202299417</v>
-      </c>
-      <c r="I4" s="39" t="n">
-        <v>0.3618021344736988</v>
-      </c>
-      <c r="J4" s="39" t="n">
+      <c r="K4" s="39" t="n">
         <v>0.3185044303538165</v>
       </c>
-      <c r="K4" s="39" t="n">
+      <c r="L4" s="39" t="n">
         <v>0.3870448801714277</v>
-      </c>
-      <c r="L4" s="39" t="n">
-        <v>0.3846397190981454</v>
       </c>
     </row>
     <row r="5">
@@ -7195,37 +7481,37 @@
         </is>
       </c>
       <c r="B5" s="39" t="n">
+        <v>16.89617295246872</v>
+      </c>
+      <c r="C5" s="37" t="n">
+        <v>-1.346842720327924</v>
+      </c>
+      <c r="D5" s="26" t="n">
+        <v>39.67425959738566</v>
+      </c>
+      <c r="E5" s="39" t="n">
         <v>18.24301567279665</v>
       </c>
-      <c r="C5" s="37" t="n">
+      <c r="F5" s="37" t="n">
         <v>-0.1912237139278119</v>
       </c>
-      <c r="D5" s="26" t="n">
+      <c r="G5" s="26" t="n">
         <v>40.13137454284129</v>
       </c>
-      <c r="E5" s="39" t="n">
+      <c r="H5" s="39" t="n">
+        <v>16.89617295246872</v>
+      </c>
+      <c r="I5" s="39" t="n">
+        <v>18.24301567279665</v>
+      </c>
+      <c r="J5" s="39" t="n">
         <v>18.43423938672446</v>
       </c>
-      <c r="F5" s="39" t="n">
-        <v>0.5497599868754506</v>
-      </c>
-      <c r="G5" s="26" t="n">
-        <v>40.19627537813753</v>
-      </c>
-      <c r="H5" s="39" t="n">
-        <v>18.24301567279665</v>
-      </c>
-      <c r="I5" s="39" t="n">
-        <v>18.43423938672446</v>
-      </c>
-      <c r="J5" s="39" t="n">
+      <c r="K5" s="39" t="n">
         <v>17.88447939984901</v>
       </c>
-      <c r="K5" s="39" t="n">
+      <c r="L5" s="39" t="n">
         <v>17.92194239067766</v>
-      </c>
-      <c r="L5" s="39" t="n">
-        <v>18.70061788946713</v>
       </c>
     </row>
     <row r="6">
@@ -7235,37 +7521,37 @@
         </is>
       </c>
       <c r="B6" s="39" t="n">
+        <v>1.550358385925565</v>
+      </c>
+      <c r="C6" s="37" t="n">
+        <v>-0.5601496694466417</v>
+      </c>
+      <c r="D6" s="26" t="n">
+        <v>8.785765996543011</v>
+      </c>
+      <c r="E6" s="39" t="n">
         <v>2.110508055372207</v>
       </c>
-      <c r="C6" s="37" t="n">
-        <v>-0.01027232477603945</v>
-      </c>
-      <c r="D6" s="26" t="n">
+      <c r="F6" s="37" t="n">
+        <v>-0.01027232477603901</v>
+      </c>
+      <c r="G6" s="26" t="n">
         <v>8.834228099454517</v>
       </c>
-      <c r="E6" s="39" t="n">
+      <c r="H6" s="39" t="n">
+        <v>1.550358385925565</v>
+      </c>
+      <c r="I6" s="39" t="n">
+        <v>2.110508055372207</v>
+      </c>
+      <c r="J6" s="39" t="n">
         <v>2.120780380148246</v>
       </c>
-      <c r="F6" s="39" t="n">
-        <v>0.8250787031808482</v>
-      </c>
-      <c r="G6" s="26" t="n">
-        <v>8.835116823464528</v>
-      </c>
-      <c r="H6" s="39" t="n">
-        <v>2.110508055372207</v>
-      </c>
-      <c r="I6" s="39" t="n">
-        <v>2.120780380148246</v>
-      </c>
-      <c r="J6" s="39" t="n">
+      <c r="K6" s="39" t="n">
         <v>1.295701676967398</v>
       </c>
-      <c r="K6" s="39" t="n">
+      <c r="L6" s="39" t="n">
         <v>1.400268169759111</v>
-      </c>
-      <c r="L6" s="39" t="n">
-        <v>0.6994064129156596</v>
       </c>
     </row>
     <row r="7">
@@ -7275,37 +7561,37 @@
         </is>
       </c>
       <c r="B7" s="39" t="n">
+        <v>5.684894955221842</v>
+      </c>
+      <c r="C7" s="39" t="n">
+        <v>2.038889061038818</v>
+      </c>
+      <c r="D7" s="26" t="n">
+        <v>7.625160270532558</v>
+      </c>
+      <c r="E7" s="39" t="n">
         <v>3.646005894183024</v>
       </c>
-      <c r="C7" s="37" t="n">
-        <v>-0.8405822042607092</v>
-      </c>
-      <c r="D7" s="26" t="n">
+      <c r="F7" s="37" t="n">
+        <v>-0.8405822042607096</v>
+      </c>
+      <c r="G7" s="26" t="n">
         <v>7.478054519319542</v>
       </c>
-      <c r="E7" s="39" t="n">
+      <c r="H7" s="39" t="n">
+        <v>5.684894955221842</v>
+      </c>
+      <c r="I7" s="39" t="n">
+        <v>3.646005894183024</v>
+      </c>
+      <c r="J7" s="39" t="n">
         <v>4.486588098443733</v>
       </c>
-      <c r="F7" s="37" t="n">
-        <v>-0.3230971381418479</v>
-      </c>
-      <c r="G7" s="26" t="n">
-        <v>7.538702486380125</v>
-      </c>
-      <c r="H7" s="39" t="n">
-        <v>3.646005894183024</v>
-      </c>
-      <c r="I7" s="39" t="n">
-        <v>4.486588098443733</v>
-      </c>
-      <c r="J7" s="39" t="n">
+      <c r="K7" s="39" t="n">
         <v>4.809685236585581</v>
       </c>
-      <c r="K7" s="39" t="n">
+      <c r="L7" s="39" t="n">
         <v>3.427905015900667</v>
-      </c>
-      <c r="L7" s="39" t="n">
-        <v>2.76409697986888</v>
       </c>
     </row>
     <row r="8">
@@ -7315,37 +7601,37 @@
         </is>
       </c>
       <c r="B8" s="39" t="n">
+        <v>6.008719826887177</v>
+      </c>
+      <c r="C8" s="39" t="n">
+        <v>1.437485581558029</v>
+      </c>
+      <c r="D8" s="26" t="n">
+        <v>16.11731394089035</v>
+      </c>
+      <c r="E8" s="39" t="n">
         <v>4.571234245329148</v>
       </c>
-      <c r="C8" s="37" t="n">
+      <c r="F8" s="37" t="n">
         <v>-1.036877997958707</v>
       </c>
-      <c r="D8" s="26" t="n">
+      <c r="G8" s="26" t="n">
         <v>15.89876204778846</v>
       </c>
-      <c r="E8" s="39" t="n">
+      <c r="H8" s="39" t="n">
+        <v>6.008719826887177</v>
+      </c>
+      <c r="I8" s="39" t="n">
+        <v>4.571234245329148</v>
+      </c>
+      <c r="J8" s="39" t="n">
         <v>5.608112243287855</v>
       </c>
-      <c r="F8" s="37" t="n">
-        <v>-0.3679653063841881</v>
-      </c>
-      <c r="G8" s="26" t="n">
-        <v>16.0564065155152</v>
-      </c>
-      <c r="H8" s="39" t="n">
-        <v>4.571234245329148</v>
-      </c>
-      <c r="I8" s="39" t="n">
-        <v>5.608112243287855</v>
-      </c>
-      <c r="J8" s="39" t="n">
+      <c r="K8" s="39" t="n">
         <v>5.976077549672043</v>
       </c>
-      <c r="K8" s="39" t="n">
+      <c r="L8" s="39" t="n">
         <v>4.545796782882716</v>
-      </c>
-      <c r="L8" s="39" t="n">
-        <v>4.348566961626465</v>
       </c>
     </row>
     <row r="9">
@@ -7355,37 +7641,37 @@
         </is>
       </c>
       <c r="B9" s="39" t="n">
+        <v>16.56704722761286</v>
+      </c>
+      <c r="C9" s="37" t="n">
+        <v>-0.8612988741681242</v>
+      </c>
+      <c r="D9" s="26" t="n">
+        <v>11.4991072702717</v>
+      </c>
+      <c r="E9" s="39" t="n">
         <v>17.42834610178099</v>
       </c>
-      <c r="C9" s="39" t="n">
+      <c r="F9" s="39" t="n">
         <v>0.01874506292522682</v>
       </c>
-      <c r="D9" s="26" t="n">
+      <c r="G9" s="26" t="n">
         <v>11.58407269044301</v>
       </c>
-      <c r="E9" s="39" t="n">
+      <c r="H9" s="39" t="n">
+        <v>16.56704722761286</v>
+      </c>
+      <c r="I9" s="39" t="n">
+        <v>17.42834610178099</v>
+      </c>
+      <c r="J9" s="39" t="n">
         <v>17.40960103885576</v>
       </c>
-      <c r="F9" s="37" t="n">
-        <v>-0.1558171114065772</v>
-      </c>
-      <c r="G9" s="26" t="n">
-        <v>11.58222352728334</v>
-      </c>
-      <c r="H9" s="39" t="n">
-        <v>17.42834610178099</v>
-      </c>
-      <c r="I9" s="39" t="n">
-        <v>17.40960103885576</v>
-      </c>
-      <c r="J9" s="39" t="n">
+      <c r="K9" s="39" t="n">
         <v>17.56541815026234</v>
       </c>
-      <c r="K9" s="39" t="n">
+      <c r="L9" s="39" t="n">
         <v>17.38551047702965</v>
-      </c>
-      <c r="L9" s="39" t="n">
-        <v>17.68857772474563</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
EGAT retirement pages update 2026-04-28T04:15:08Z
</commit_message>
<xml_diff>
--- a/EGAT Retirement.xlsx
+++ b/EGAT Retirement.xlsx
@@ -683,7 +683,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I20"/>
+  <dimension ref="A1:I21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1522,6 +1522,47 @@
         </is>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>11:15:07</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>EGAT1</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>ตราสารหนี้ (EGAT-1)</t>
+        </is>
+      </c>
+      <c r="F21" t="n">
+        <v>15.75701985540809</v>
+      </c>
+      <c r="G21" t="n">
+        <v>0.6112145825118986</v>
+      </c>
+      <c r="H21" t="n">
+        <v>0.3215690747309763</v>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>https://app.powerbi.com/view?r=eyJrIjoiMzZjYWU3YmQtNWQ1Ny00NjdjLWI1MmEtYjExY2ZiYWIxMzNiIiwidCI6IjVmZWJjNjlmLThlOWMtNDcwOC1iNzBlLWQ4YzYyYmUxODA1YiIsImMiOjEwfQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1533,7 +1574,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I20"/>
+  <dimension ref="A1:I21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -2372,6 +2413,47 @@
         </is>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>11:15:07</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>EGAT2</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>ตราสารทุน (EGAT-2)</t>
+        </is>
+      </c>
+      <c r="F21" t="n">
+        <v>39.52436402199133</v>
+      </c>
+      <c r="G21" t="n">
+        <v>1.085477887294894</v>
+      </c>
+      <c r="H21" t="n">
+        <v>16.45452087669159</v>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>https://app.powerbi.com/view?r=eyJrIjoiMzZjYWU3YmQtNWQ1Ny00NjdjLWI1MmEtYjExY2ZiYWIxMzNiIiwidCI6IjVmZWJjNjlmLThlOWMtNDcwOC1iNzBlLWQ4YzYyYmUxODA1YiIsImMiOjEwfQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2383,7 +2465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I20"/>
+  <dimension ref="A1:I21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -3222,6 +3304,47 @@
         </is>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>11:15:07</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>EGAT3</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>อสังหาริมทรัพย์และโครงสร้างพื้นฐาน (EGAT-3)</t>
+        </is>
+      </c>
+      <c r="F21" t="n">
+        <v>8.773807101034656</v>
+      </c>
+      <c r="G21" t="n">
+        <v>4.26927374777486</v>
+      </c>
+      <c r="H21" t="n">
+        <v>1.412131380420178</v>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>https://app.powerbi.com/view?r=eyJrIjoiMzZjYWU3YmQtNWQ1Ny00NjdjLWI1MmEtYjExY2ZiYWIxMzNiIiwidCI6IjVmZWJjNjlmLThlOWMtNDcwOC1iNzBlLWQ4YzYyYmUxODA1YiIsImMiOjEwfQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3233,7 +3356,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I20"/>
+  <dimension ref="A1:I21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -4072,6 +4195,47 @@
         </is>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>11:15:07</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>EGAT4</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>ตราสารทุนต่างประเทศ (EGAT-4)</t>
+        </is>
+      </c>
+      <c r="F21" t="n">
+        <v>7.573289366524095</v>
+      </c>
+      <c r="G21" t="n">
+        <v>11.69547729779012</v>
+      </c>
+      <c r="H21" t="n">
+        <v>4.965963044695054</v>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>https://app.powerbi.com/view?r=eyJrIjoiMzZjYWU3YmQtNWQ1Ny00NjdjLWI1MmEtYjExY2ZiYWIxMzNiIiwidCI6IjVmZWJjNjlmLThlOWMtNDcwOC1iNzBlLWQ4YzYyYmUxODA1YiIsImMiOjEwfQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4083,7 +4247,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I20"/>
+  <dimension ref="A1:I21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -4922,6 +5086,47 @@
         </is>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>11:15:07</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>EGAT5</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>ตราสารทุนต่างประเทศแบบอิงดัชนี (EGAT-5)</t>
+        </is>
+      </c>
+      <c r="F21" t="n">
+        <v>16.02176201763107</v>
+      </c>
+      <c r="G21" t="n">
+        <v>10.2936677748789</v>
+      </c>
+      <c r="H21" t="n">
+        <v>5.380244319190153</v>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>https://app.powerbi.com/view?r=eyJrIjoiMzZjYWU3YmQtNWQ1Ny00NjdjLWI1MmEtYjExY2ZiYWIxMzNiIiwidCI6IjVmZWJjNjlmLThlOWMtNDcwOC1iNzBlLWQ4YzYyYmUxODA1YiIsImMiOjEwfQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4933,7 +5138,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I20"/>
+  <dimension ref="A1:I21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -5767,6 +5972,47 @@
         <v>16.56704722761286</v>
       </c>
       <c r="I20" t="inlineStr">
+        <is>
+          <t>https://app.powerbi.com/view?r=eyJrIjoiMzZjYWU3YmQtNWQ1Ny00NjdjLWI1MmEtYjExY2ZiYWIxMzNiIiwidCI6IjVmZWJjNjlmLThlOWMtNDcwOC1iNzBlLWQ4YzYyYmUxODA1YiIsImMiOjEwfQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>11:15:07</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>EGAT6</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>การลงทุนตามหลักศาสนาอิสลาม (EGAT-6)</t>
+        </is>
+      </c>
+      <c r="F21" t="n">
+        <v>11.49463721306256</v>
+      </c>
+      <c r="G21" t="n">
+        <v>1.33496010243157</v>
+      </c>
+      <c r="H21" t="n">
+        <v>16.52173402567803</v>
+      </c>
+      <c r="I21" t="inlineStr">
         <is>
           <t>https://app.powerbi.com/view?r=eyJrIjoiMzZjYWU3YmQtNWQ1Ny00NjdjLWI1MmEtYjExY2ZiYWIxMzNiIiwidCI6IjVmZWJjNjlmLThlOWMtNDcwOC1iNzBlLWQ4YzYyYmUxODA1YiIsImMiOjEwfQ%3D%3D</t>
         </is>
@@ -7044,10 +7290,10 @@
         </is>
       </c>
       <c r="B25" s="35" t="n">
-        <v>7.832599724189489</v>
+        <v>7.832599724189488</v>
       </c>
       <c r="C25" s="35" t="n">
-        <v>0.1107278592408294</v>
+        <v>0.1107278592408285</v>
       </c>
       <c r="D25" s="35" t="n">
         <v>0.2884049970207636</v>
@@ -7062,7 +7308,7 @@
         <v>16.89617295246872</v>
       </c>
       <c r="H25" s="36" t="n">
-        <v>-1.346842720327924</v>
+        <v>-1.346842720327928</v>
       </c>
       <c r="I25" s="19" t="n">
         <v>39.67425959738566</v>
@@ -7071,7 +7317,7 @@
         <v>1.550358385925565</v>
       </c>
       <c r="K25" s="36" t="n">
-        <v>-0.5601496694466417</v>
+        <v>-0.5601496694466421</v>
       </c>
       <c r="L25" s="19" t="n">
         <v>8.785765996543011</v>
@@ -7098,7 +7344,7 @@
         <v>16.56704722761286</v>
       </c>
       <c r="T25" s="36" t="n">
-        <v>-0.8612988741681242</v>
+        <v>-0.8612988741681278</v>
       </c>
       <c r="U25" s="19" t="n">
         <v>11.4991072702717</v>
@@ -7110,26 +7356,66 @@
           <t>24/4/69</t>
         </is>
       </c>
-      <c r="B26" s="33" t="n"/>
-      <c r="C26" s="33" t="n"/>
-      <c r="D26" s="33" t="n"/>
-      <c r="E26" s="33" t="n"/>
-      <c r="F26" s="12" t="n"/>
-      <c r="G26" s="33" t="n"/>
-      <c r="H26" s="33" t="n"/>
-      <c r="I26" s="12" t="n"/>
-      <c r="J26" s="33" t="n"/>
-      <c r="K26" s="33" t="n"/>
-      <c r="L26" s="12" t="n"/>
-      <c r="M26" s="33" t="n"/>
-      <c r="N26" s="33" t="n"/>
-      <c r="O26" s="12" t="n"/>
-      <c r="P26" s="33" t="n"/>
-      <c r="Q26" s="33" t="n"/>
-      <c r="R26" s="12" t="n"/>
-      <c r="S26" s="33" t="n"/>
-      <c r="T26" s="33" t="n"/>
-      <c r="U26" s="12" t="n"/>
+      <c r="B26" s="35" t="n">
+        <v>7.509360453567663</v>
+      </c>
+      <c r="C26" s="36" t="n">
+        <v>-0.3232392706218246</v>
+      </c>
+      <c r="D26" s="35" t="n">
+        <v>0.3215690747309763</v>
+      </c>
+      <c r="E26" s="35" t="n">
+        <v>0.03316407771021268</v>
+      </c>
+      <c r="F26" s="19" t="n">
+        <v>15.75701985540809</v>
+      </c>
+      <c r="G26" s="35" t="n">
+        <v>16.45452087669159</v>
+      </c>
+      <c r="H26" s="36" t="n">
+        <v>-0.4416520757771281</v>
+      </c>
+      <c r="I26" s="19" t="n">
+        <v>39.52436402199133</v>
+      </c>
+      <c r="J26" s="35" t="n">
+        <v>1.412131380420178</v>
+      </c>
+      <c r="K26" s="36" t="n">
+        <v>-0.1382270055053865</v>
+      </c>
+      <c r="L26" s="19" t="n">
+        <v>8.773807101034656</v>
+      </c>
+      <c r="M26" s="35" t="n">
+        <v>4.965963044695054</v>
+      </c>
+      <c r="N26" s="36" t="n">
+        <v>-0.7189319105267877</v>
+      </c>
+      <c r="O26" s="19" t="n">
+        <v>7.573289366524095</v>
+      </c>
+      <c r="P26" s="35" t="n">
+        <v>5.380244319190153</v>
+      </c>
+      <c r="Q26" s="36" t="n">
+        <v>-0.6284755076970239</v>
+      </c>
+      <c r="R26" s="19" t="n">
+        <v>16.02176201763107</v>
+      </c>
+      <c r="S26" s="35" t="n">
+        <v>16.52173402567803</v>
+      </c>
+      <c r="T26" s="36" t="n">
+        <v>-0.04531320193483523</v>
+      </c>
+      <c r="U26" s="19" t="n">
+        <v>11.49463721306256</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="13" t="inlineStr">
@@ -7340,14 +7626,14 @@
       </c>
       <c r="B1" s="4" t="inlineStr">
         <is>
-          <t>23 เม.ย. 69 (พฤหัส)</t>
+          <t>24 เม.ย. 69 (ศุกร์)</t>
         </is>
       </c>
       <c r="C1" s="20" t="n"/>
       <c r="D1" s="20" t="n"/>
       <c r="E1" s="21" t="inlineStr">
         <is>
-          <t>22 เม.ย. 69 (พุธ)</t>
+          <t>23 เม.ย. 69 (พฤหัส)</t>
         </is>
       </c>
       <c r="F1" s="20" t="n"/>
@@ -7410,27 +7696,27 @@
       <c r="G3" s="20" t="n"/>
       <c r="H3" s="22" t="inlineStr">
         <is>
+          <t>24/4/69</t>
+        </is>
+      </c>
+      <c r="I3" s="22" t="inlineStr">
+        <is>
           <t>23/4/69</t>
         </is>
       </c>
-      <c r="I3" s="22" t="inlineStr">
+      <c r="J3" s="22" t="inlineStr">
         <is>
           <t>22/4/69</t>
         </is>
       </c>
-      <c r="J3" s="22" t="inlineStr">
+      <c r="K3" s="22" t="inlineStr">
         <is>
           <t>21/4/69</t>
         </is>
       </c>
-      <c r="K3" s="22" t="inlineStr">
+      <c r="L3" s="22" t="inlineStr">
         <is>
           <t>20/4/69</t>
-        </is>
-      </c>
-      <c r="L3" s="22" t="inlineStr">
-        <is>
-          <t>17/4/69</t>
         </is>
       </c>
     </row>
@@ -7441,37 +7727,37 @@
         </is>
       </c>
       <c r="B4" s="39" t="n">
+        <v>0.3215690747309763</v>
+      </c>
+      <c r="C4" s="39" t="n">
+        <v>0.03316407771021268</v>
+      </c>
+      <c r="D4" s="26" t="n">
+        <v>15.75701985540809</v>
+      </c>
+      <c r="E4" s="39" t="n">
         <v>0.2884049970207636</v>
       </c>
-      <c r="C4" s="37" t="n">
+      <c r="F4" s="37" t="n">
         <v>-0.04371622320917812</v>
       </c>
-      <c r="D4" s="26" t="n">
+      <c r="G4" s="26" t="n">
         <v>15.75181093537439</v>
       </c>
-      <c r="E4" s="39" t="n">
+      <c r="H4" s="39" t="n">
+        <v>0.3215690747309763</v>
+      </c>
+      <c r="I4" s="39" t="n">
+        <v>0.2884049970207636</v>
+      </c>
+      <c r="J4" s="39" t="n">
         <v>0.3321212202299417</v>
       </c>
-      <c r="F4" s="37" t="n">
-        <v>-0.02968091424375707</v>
-      </c>
-      <c r="G4" s="26" t="n">
-        <v>15.75867722946711</v>
-      </c>
-      <c r="H4" s="39" t="n">
-        <v>0.2884049970207636</v>
-      </c>
-      <c r="I4" s="39" t="n">
-        <v>0.3321212202299417</v>
-      </c>
-      <c r="J4" s="39" t="n">
+      <c r="K4" s="39" t="n">
         <v>0.3618021344736988</v>
       </c>
-      <c r="K4" s="39" t="n">
+      <c r="L4" s="39" t="n">
         <v>0.3185044303538165</v>
-      </c>
-      <c r="L4" s="39" t="n">
-        <v>0.3870448801714277</v>
       </c>
     </row>
     <row r="5">
@@ -7481,37 +7767,37 @@
         </is>
       </c>
       <c r="B5" s="39" t="n">
+        <v>16.45452087669159</v>
+      </c>
+      <c r="C5" s="37" t="n">
+        <v>-0.4416520757771281</v>
+      </c>
+      <c r="D5" s="26" t="n">
+        <v>39.52436402199133</v>
+      </c>
+      <c r="E5" s="39" t="n">
         <v>16.89617295246872</v>
       </c>
-      <c r="C5" s="37" t="n">
-        <v>-1.346842720327924</v>
-      </c>
-      <c r="D5" s="26" t="n">
+      <c r="F5" s="37" t="n">
+        <v>-1.346842720327928</v>
+      </c>
+      <c r="G5" s="26" t="n">
         <v>39.67425959738566</v>
       </c>
-      <c r="E5" s="39" t="n">
+      <c r="H5" s="39" t="n">
+        <v>16.45452087669159</v>
+      </c>
+      <c r="I5" s="39" t="n">
+        <v>16.89617295246872</v>
+      </c>
+      <c r="J5" s="39" t="n">
         <v>18.24301567279665</v>
       </c>
-      <c r="F5" s="37" t="n">
-        <v>-0.1912237139278119</v>
-      </c>
-      <c r="G5" s="26" t="n">
-        <v>40.13137454284129</v>
-      </c>
-      <c r="H5" s="39" t="n">
-        <v>16.89617295246872</v>
-      </c>
-      <c r="I5" s="39" t="n">
-        <v>18.24301567279665</v>
-      </c>
-      <c r="J5" s="39" t="n">
+      <c r="K5" s="39" t="n">
         <v>18.43423938672446</v>
       </c>
-      <c r="K5" s="39" t="n">
+      <c r="L5" s="39" t="n">
         <v>17.88447939984901</v>
-      </c>
-      <c r="L5" s="39" t="n">
-        <v>17.92194239067766</v>
       </c>
     </row>
     <row r="6">
@@ -7521,37 +7807,37 @@
         </is>
       </c>
       <c r="B6" s="39" t="n">
+        <v>1.412131380420178</v>
+      </c>
+      <c r="C6" s="37" t="n">
+        <v>-0.1382270055053865</v>
+      </c>
+      <c r="D6" s="26" t="n">
+        <v>8.773807101034656</v>
+      </c>
+      <c r="E6" s="39" t="n">
         <v>1.550358385925565</v>
       </c>
-      <c r="C6" s="37" t="n">
-        <v>-0.5601496694466417</v>
-      </c>
-      <c r="D6" s="26" t="n">
+      <c r="F6" s="37" t="n">
+        <v>-0.5601496694466421</v>
+      </c>
+      <c r="G6" s="26" t="n">
         <v>8.785765996543011</v>
       </c>
-      <c r="E6" s="39" t="n">
+      <c r="H6" s="39" t="n">
+        <v>1.412131380420178</v>
+      </c>
+      <c r="I6" s="39" t="n">
+        <v>1.550358385925565</v>
+      </c>
+      <c r="J6" s="39" t="n">
         <v>2.110508055372207</v>
       </c>
-      <c r="F6" s="37" t="n">
-        <v>-0.01027232477603901</v>
-      </c>
-      <c r="G6" s="26" t="n">
-        <v>8.834228099454517</v>
-      </c>
-      <c r="H6" s="39" t="n">
-        <v>1.550358385925565</v>
-      </c>
-      <c r="I6" s="39" t="n">
-        <v>2.110508055372207</v>
-      </c>
-      <c r="J6" s="39" t="n">
+      <c r="K6" s="39" t="n">
         <v>2.120780380148246</v>
       </c>
-      <c r="K6" s="39" t="n">
+      <c r="L6" s="39" t="n">
         <v>1.295701676967398</v>
-      </c>
-      <c r="L6" s="39" t="n">
-        <v>1.400268169759111</v>
       </c>
     </row>
     <row r="7">
@@ -7561,37 +7847,37 @@
         </is>
       </c>
       <c r="B7" s="39" t="n">
+        <v>4.965963044695054</v>
+      </c>
+      <c r="C7" s="37" t="n">
+        <v>-0.7189319105267877</v>
+      </c>
+      <c r="D7" s="26" t="n">
+        <v>7.573289366524095</v>
+      </c>
+      <c r="E7" s="39" t="n">
         <v>5.684894955221842</v>
       </c>
-      <c r="C7" s="39" t="n">
+      <c r="F7" s="39" t="n">
         <v>2.038889061038818</v>
       </c>
-      <c r="D7" s="26" t="n">
+      <c r="G7" s="26" t="n">
         <v>7.625160270532558</v>
       </c>
-      <c r="E7" s="39" t="n">
+      <c r="H7" s="39" t="n">
+        <v>4.965963044695054</v>
+      </c>
+      <c r="I7" s="39" t="n">
+        <v>5.684894955221842</v>
+      </c>
+      <c r="J7" s="39" t="n">
         <v>3.646005894183024</v>
       </c>
-      <c r="F7" s="37" t="n">
-        <v>-0.8405822042607096</v>
-      </c>
-      <c r="G7" s="26" t="n">
-        <v>7.478054519319542</v>
-      </c>
-      <c r="H7" s="39" t="n">
-        <v>5.684894955221842</v>
-      </c>
-      <c r="I7" s="39" t="n">
-        <v>3.646005894183024</v>
-      </c>
-      <c r="J7" s="39" t="n">
+      <c r="K7" s="39" t="n">
         <v>4.486588098443733</v>
       </c>
-      <c r="K7" s="39" t="n">
+      <c r="L7" s="39" t="n">
         <v>4.809685236585581</v>
-      </c>
-      <c r="L7" s="39" t="n">
-        <v>3.427905015900667</v>
       </c>
     </row>
     <row r="8">
@@ -7601,37 +7887,37 @@
         </is>
       </c>
       <c r="B8" s="39" t="n">
+        <v>5.380244319190153</v>
+      </c>
+      <c r="C8" s="37" t="n">
+        <v>-0.6284755076970239</v>
+      </c>
+      <c r="D8" s="26" t="n">
+        <v>16.02176201763107</v>
+      </c>
+      <c r="E8" s="39" t="n">
         <v>6.008719826887177</v>
       </c>
-      <c r="C8" s="39" t="n">
+      <c r="F8" s="39" t="n">
         <v>1.437485581558029</v>
       </c>
-      <c r="D8" s="26" t="n">
+      <c r="G8" s="26" t="n">
         <v>16.11731394089035</v>
       </c>
-      <c r="E8" s="39" t="n">
+      <c r="H8" s="39" t="n">
+        <v>5.380244319190153</v>
+      </c>
+      <c r="I8" s="39" t="n">
+        <v>6.008719826887177</v>
+      </c>
+      <c r="J8" s="39" t="n">
         <v>4.571234245329148</v>
       </c>
-      <c r="F8" s="37" t="n">
-        <v>-1.036877997958707</v>
-      </c>
-      <c r="G8" s="26" t="n">
-        <v>15.89876204778846</v>
-      </c>
-      <c r="H8" s="39" t="n">
-        <v>6.008719826887177</v>
-      </c>
-      <c r="I8" s="39" t="n">
-        <v>4.571234245329148</v>
-      </c>
-      <c r="J8" s="39" t="n">
+      <c r="K8" s="39" t="n">
         <v>5.608112243287855</v>
       </c>
-      <c r="K8" s="39" t="n">
+      <c r="L8" s="39" t="n">
         <v>5.976077549672043</v>
-      </c>
-      <c r="L8" s="39" t="n">
-        <v>4.545796782882716</v>
       </c>
     </row>
     <row r="9">
@@ -7641,37 +7927,37 @@
         </is>
       </c>
       <c r="B9" s="39" t="n">
+        <v>16.52173402567803</v>
+      </c>
+      <c r="C9" s="37" t="n">
+        <v>-0.04531320193483523</v>
+      </c>
+      <c r="D9" s="26" t="n">
+        <v>11.49463721306256</v>
+      </c>
+      <c r="E9" s="39" t="n">
         <v>16.56704722761286</v>
       </c>
-      <c r="C9" s="37" t="n">
-        <v>-0.8612988741681242</v>
-      </c>
-      <c r="D9" s="26" t="n">
+      <c r="F9" s="37" t="n">
+        <v>-0.8612988741681278</v>
+      </c>
+      <c r="G9" s="26" t="n">
         <v>11.4991072702717</v>
       </c>
-      <c r="E9" s="39" t="n">
+      <c r="H9" s="39" t="n">
+        <v>16.52173402567803</v>
+      </c>
+      <c r="I9" s="39" t="n">
+        <v>16.56704722761286</v>
+      </c>
+      <c r="J9" s="39" t="n">
         <v>17.42834610178099</v>
       </c>
-      <c r="F9" s="39" t="n">
-        <v>0.01874506292522682</v>
-      </c>
-      <c r="G9" s="26" t="n">
-        <v>11.58407269044301</v>
-      </c>
-      <c r="H9" s="39" t="n">
-        <v>16.56704722761286</v>
-      </c>
-      <c r="I9" s="39" t="n">
-        <v>17.42834610178099</v>
-      </c>
-      <c r="J9" s="39" t="n">
+      <c r="K9" s="39" t="n">
         <v>17.40960103885576</v>
       </c>
-      <c r="K9" s="39" t="n">
+      <c r="L9" s="39" t="n">
         <v>17.56541815026234</v>
-      </c>
-      <c r="L9" s="39" t="n">
-        <v>17.38551047702965</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
EGAT retirement pages update 2026-04-29T04:15:08Z
</commit_message>
<xml_diff>
--- a/EGAT Retirement.xlsx
+++ b/EGAT Retirement.xlsx
@@ -683,7 +683,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I21"/>
+  <dimension ref="A1:I22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1563,6 +1563,47 @@
         </is>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>11:15:07</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>EGAT1</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>ตราสารหนี้ (EGAT-1)</t>
+        </is>
+      </c>
+      <c r="F22" t="n">
+        <v>15.75961586953918</v>
+      </c>
+      <c r="G22" t="n">
+        <v>0.6277905681486562</v>
+      </c>
+      <c r="H22" t="n">
+        <v>0.3380973404411236</v>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>https://app.powerbi.com/view?r=eyJrIjoiMzZjYWU3YmQtNWQ1Ny00NjdjLWI1MmEtYjExY2ZiYWIxMzNiIiwidCI6IjVmZWJjNjlmLThlOWMtNDcwOC1iNzBlLWQ4YzYyYmUxODA1YiIsImMiOjEwfQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1574,7 +1615,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I21"/>
+  <dimension ref="A1:I22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -2454,6 +2495,47 @@
         </is>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>11:15:07</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>EGAT2</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>ตราสารทุน (EGAT-2)</t>
+        </is>
+      </c>
+      <c r="F22" t="n">
+        <v>40.02823802524581</v>
+      </c>
+      <c r="G22" t="n">
+        <v>2.374160088117239</v>
+      </c>
+      <c r="H22" t="n">
+        <v>17.93913440769168</v>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>https://app.powerbi.com/view?r=eyJrIjoiMzZjYWU3YmQtNWQ1Ny00NjdjLWI1MmEtYjExY2ZiYWIxMzNiIiwidCI6IjVmZWJjNjlmLThlOWMtNDcwOC1iNzBlLWQ4YzYyYmUxODA1YiIsImMiOjEwfQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2465,7 +2547,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I21"/>
+  <dimension ref="A1:I22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -3345,6 +3427,47 @@
         </is>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>11:15:07</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>EGAT3</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>อสังหาริมทรัพย์และโครงสร้างพื้นฐาน (EGAT-3)</t>
+        </is>
+      </c>
+      <c r="F22" t="n">
+        <v>8.763384622383818</v>
+      </c>
+      <c r="G22" t="n">
+        <v>4.145411407623056</v>
+      </c>
+      <c r="H22" t="n">
+        <v>1.291663063522286</v>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>https://app.powerbi.com/view?r=eyJrIjoiMzZjYWU3YmQtNWQ1Ny00NjdjLWI1MmEtYjExY2ZiYWIxMzNiIiwidCI6IjVmZWJjNjlmLThlOWMtNDcwOC1iNzBlLWQ4YzYyYmUxODA1YiIsImMiOjEwfQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3356,7 +3479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I21"/>
+  <dimension ref="A1:I22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -4236,6 +4359,47 @@
         </is>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>11:15:07</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>EGAT4</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>ตราสารทุนต่างประเทศ (EGAT-4)</t>
+        </is>
+      </c>
+      <c r="F22" t="n">
+        <v>7.669062142032713</v>
+      </c>
+      <c r="G22" t="n">
+        <v>13.10799243551277</v>
+      </c>
+      <c r="H22" t="n">
+        <v>6.293375893748721</v>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>https://app.powerbi.com/view?r=eyJrIjoiMzZjYWU3YmQtNWQ1Ny00NjdjLWI1MmEtYjExY2ZiYWIxMzNiIiwidCI6IjVmZWJjNjlmLThlOWMtNDcwOC1iNzBlLWQ4YzYyYmUxODA1YiIsImMiOjEwfQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4247,7 +4411,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I21"/>
+  <dimension ref="A1:I22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -5127,6 +5291,47 @@
         </is>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>11:15:07</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>EGAT5</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>ตราสารทุนต่างประเทศแบบอิงดัชนี (EGAT-5)</t>
+        </is>
+      </c>
+      <c r="F22" t="n">
+        <v>16.12058896045554</v>
+      </c>
+      <c r="G22" t="n">
+        <v>10.9739915736655</v>
+      </c>
+      <c r="H22" t="n">
+        <v>6.030260676236354</v>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>https://app.powerbi.com/view?r=eyJrIjoiMzZjYWU3YmQtNWQ1Ny00NjdjLWI1MmEtYjExY2ZiYWIxMzNiIiwidCI6IjVmZWJjNjlmLThlOWMtNDcwOC1iNzBlLWQ4YzYyYmUxODA1YiIsImMiOjEwfQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -5138,7 +5343,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I21"/>
+  <dimension ref="A1:I22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -6013,6 +6218,47 @@
         <v>16.52173402567803</v>
       </c>
       <c r="I21" t="inlineStr">
+        <is>
+          <t>https://app.powerbi.com/view?r=eyJrIjoiMzZjYWU3YmQtNWQ1Ny00NjdjLWI1MmEtYjExY2ZiYWIxMzNiIiwidCI6IjVmZWJjNjlmLThlOWMtNDcwOC1iNzBlLWQ4YzYyYmUxODA1YiIsImMiOjEwfQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>11:15:07</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>EGAT6</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>การลงทุนตามหลักศาสนาอิสลาม (EGAT-6)</t>
+        </is>
+      </c>
+      <c r="F22" t="n">
+        <v>11.71493023240685</v>
+      </c>
+      <c r="G22" t="n">
+        <v>3.277029600782511</v>
+      </c>
+      <c r="H22" t="n">
+        <v>18.75485579646165</v>
+      </c>
+      <c r="I22" t="inlineStr">
         <is>
           <t>https://app.powerbi.com/view?r=eyJrIjoiMzZjYWU3YmQtNWQ1Ny00NjdjLWI1MmEtYjExY2ZiYWIxMzNiIiwidCI6IjVmZWJjNjlmLThlOWMtNDcwOC1iNzBlLWQ4YzYyYmUxODA1YiIsImMiOjEwfQ%3D%3D</t>
         </is>
@@ -7375,7 +7621,7 @@
         <v>16.45452087669159</v>
       </c>
       <c r="H26" s="36" t="n">
-        <v>-0.4416520757771281</v>
+        <v>-0.4416520757771316</v>
       </c>
       <c r="I26" s="19" t="n">
         <v>39.52436402199133</v>
@@ -7384,7 +7630,7 @@
         <v>1.412131380420178</v>
       </c>
       <c r="K26" s="36" t="n">
-        <v>-0.1382270055053865</v>
+        <v>-0.1382270055053869</v>
       </c>
       <c r="L26" s="19" t="n">
         <v>8.773807101034656</v>
@@ -7411,7 +7657,7 @@
         <v>16.52173402567803</v>
       </c>
       <c r="T26" s="36" t="n">
-        <v>-0.04531320193483523</v>
+        <v>-0.04531320193483168</v>
       </c>
       <c r="U26" s="19" t="n">
         <v>11.49463721306256</v>
@@ -7477,26 +7723,66 @@
           <t>27/4/69</t>
         </is>
       </c>
-      <c r="B29" s="33" t="n"/>
-      <c r="C29" s="33" t="n"/>
-      <c r="D29" s="33" t="n"/>
-      <c r="E29" s="33" t="n"/>
-      <c r="F29" s="12" t="n"/>
-      <c r="G29" s="33" t="n"/>
-      <c r="H29" s="33" t="n"/>
-      <c r="I29" s="12" t="n"/>
-      <c r="J29" s="33" t="n"/>
-      <c r="K29" s="33" t="n"/>
-      <c r="L29" s="12" t="n"/>
-      <c r="M29" s="33" t="n"/>
-      <c r="N29" s="33" t="n"/>
-      <c r="O29" s="12" t="n"/>
-      <c r="P29" s="33" t="n"/>
-      <c r="Q29" s="33" t="n"/>
-      <c r="R29" s="12" t="n"/>
-      <c r="S29" s="33" t="n"/>
-      <c r="T29" s="33" t="n"/>
-      <c r="U29" s="12" t="n"/>
+      <c r="B29" s="35" t="n">
+        <v>8.441231196350303</v>
+      </c>
+      <c r="C29" s="35" t="n">
+        <v>0.9318707427826398</v>
+      </c>
+      <c r="D29" s="35" t="n">
+        <v>0.3380973404411236</v>
+      </c>
+      <c r="E29" s="35" t="n">
+        <v>0.01652826571014732</v>
+      </c>
+      <c r="F29" s="19" t="n">
+        <v>15.75961586953918</v>
+      </c>
+      <c r="G29" s="35" t="n">
+        <v>17.93913440769168</v>
+      </c>
+      <c r="H29" s="35" t="n">
+        <v>1.484613531000093</v>
+      </c>
+      <c r="I29" s="19" t="n">
+        <v>40.02823802524581</v>
+      </c>
+      <c r="J29" s="35" t="n">
+        <v>1.291663063522286</v>
+      </c>
+      <c r="K29" s="36" t="n">
+        <v>-0.1204683168978922</v>
+      </c>
+      <c r="L29" s="19" t="n">
+        <v>8.763384622383818</v>
+      </c>
+      <c r="M29" s="35" t="n">
+        <v>6.293375893748721</v>
+      </c>
+      <c r="N29" s="35" t="n">
+        <v>1.327412849053666</v>
+      </c>
+      <c r="O29" s="19" t="n">
+        <v>7.669062142032713</v>
+      </c>
+      <c r="P29" s="35" t="n">
+        <v>6.030260676236354</v>
+      </c>
+      <c r="Q29" s="35" t="n">
+        <v>0.6500163570462014</v>
+      </c>
+      <c r="R29" s="19" t="n">
+        <v>16.12058896045554</v>
+      </c>
+      <c r="S29" s="35" t="n">
+        <v>18.75485579646165</v>
+      </c>
+      <c r="T29" s="35" t="n">
+        <v>2.233121770783626</v>
+      </c>
+      <c r="U29" s="19" t="n">
+        <v>11.71493023240685</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="10" t="inlineStr">
@@ -7626,14 +7912,14 @@
       </c>
       <c r="B1" s="4" t="inlineStr">
         <is>
-          <t>24 เม.ย. 69 (ศุกร์)</t>
+          <t>27 เม.ย. 69 (จันทร์)</t>
         </is>
       </c>
       <c r="C1" s="20" t="n"/>
       <c r="D1" s="20" t="n"/>
       <c r="E1" s="21" t="inlineStr">
         <is>
-          <t>23 เม.ย. 69 (พฤหัส)</t>
+          <t>24 เม.ย. 69 (ศุกร์)</t>
         </is>
       </c>
       <c r="F1" s="20" t="n"/>
@@ -7696,27 +7982,27 @@
       <c r="G3" s="20" t="n"/>
       <c r="H3" s="22" t="inlineStr">
         <is>
+          <t>27/4/69</t>
+        </is>
+      </c>
+      <c r="I3" s="22" t="inlineStr">
+        <is>
           <t>24/4/69</t>
         </is>
       </c>
-      <c r="I3" s="22" t="inlineStr">
+      <c r="J3" s="22" t="inlineStr">
         <is>
           <t>23/4/69</t>
         </is>
       </c>
-      <c r="J3" s="22" t="inlineStr">
+      <c r="K3" s="22" t="inlineStr">
         <is>
           <t>22/4/69</t>
         </is>
       </c>
-      <c r="K3" s="22" t="inlineStr">
+      <c r="L3" s="22" t="inlineStr">
         <is>
           <t>21/4/69</t>
-        </is>
-      </c>
-      <c r="L3" s="22" t="inlineStr">
-        <is>
-          <t>20/4/69</t>
         </is>
       </c>
     </row>
@@ -7727,37 +8013,37 @@
         </is>
       </c>
       <c r="B4" s="39" t="n">
+        <v>0.3380973404411236</v>
+      </c>
+      <c r="C4" s="39" t="n">
+        <v>0.01652826571014732</v>
+      </c>
+      <c r="D4" s="26" t="n">
+        <v>15.75961586953918</v>
+      </c>
+      <c r="E4" s="39" t="n">
         <v>0.3215690747309763</v>
       </c>
-      <c r="C4" s="39" t="n">
+      <c r="F4" s="39" t="n">
         <v>0.03316407771021268</v>
       </c>
-      <c r="D4" s="26" t="n">
+      <c r="G4" s="26" t="n">
         <v>15.75701985540809</v>
       </c>
-      <c r="E4" s="39" t="n">
+      <c r="H4" s="39" t="n">
+        <v>0.3380973404411236</v>
+      </c>
+      <c r="I4" s="39" t="n">
+        <v>0.3215690747309763</v>
+      </c>
+      <c r="J4" s="39" t="n">
         <v>0.2884049970207636</v>
       </c>
-      <c r="F4" s="37" t="n">
-        <v>-0.04371622320917812</v>
-      </c>
-      <c r="G4" s="26" t="n">
-        <v>15.75181093537439</v>
-      </c>
-      <c r="H4" s="39" t="n">
-        <v>0.3215690747309763</v>
-      </c>
-      <c r="I4" s="39" t="n">
-        <v>0.2884049970207636</v>
-      </c>
-      <c r="J4" s="39" t="n">
+      <c r="K4" s="39" t="n">
         <v>0.3321212202299417</v>
       </c>
-      <c r="K4" s="39" t="n">
+      <c r="L4" s="39" t="n">
         <v>0.3618021344736988</v>
-      </c>
-      <c r="L4" s="39" t="n">
-        <v>0.3185044303538165</v>
       </c>
     </row>
     <row r="5">
@@ -7767,37 +8053,37 @@
         </is>
       </c>
       <c r="B5" s="39" t="n">
+        <v>17.93913440769168</v>
+      </c>
+      <c r="C5" s="39" t="n">
+        <v>1.484613531000093</v>
+      </c>
+      <c r="D5" s="26" t="n">
+        <v>40.02823802524581</v>
+      </c>
+      <c r="E5" s="39" t="n">
         <v>16.45452087669159</v>
       </c>
-      <c r="C5" s="37" t="n">
-        <v>-0.4416520757771281</v>
-      </c>
-      <c r="D5" s="26" t="n">
+      <c r="F5" s="37" t="n">
+        <v>-0.4416520757771316</v>
+      </c>
+      <c r="G5" s="26" t="n">
         <v>39.52436402199133</v>
       </c>
-      <c r="E5" s="39" t="n">
+      <c r="H5" s="39" t="n">
+        <v>17.93913440769168</v>
+      </c>
+      <c r="I5" s="39" t="n">
+        <v>16.45452087669159</v>
+      </c>
+      <c r="J5" s="39" t="n">
         <v>16.89617295246872</v>
       </c>
-      <c r="F5" s="37" t="n">
-        <v>-1.346842720327928</v>
-      </c>
-      <c r="G5" s="26" t="n">
-        <v>39.67425959738566</v>
-      </c>
-      <c r="H5" s="39" t="n">
-        <v>16.45452087669159</v>
-      </c>
-      <c r="I5" s="39" t="n">
-        <v>16.89617295246872</v>
-      </c>
-      <c r="J5" s="39" t="n">
+      <c r="K5" s="39" t="n">
         <v>18.24301567279665</v>
       </c>
-      <c r="K5" s="39" t="n">
+      <c r="L5" s="39" t="n">
         <v>18.43423938672446</v>
-      </c>
-      <c r="L5" s="39" t="n">
-        <v>17.88447939984901</v>
       </c>
     </row>
     <row r="6">
@@ -7807,37 +8093,37 @@
         </is>
       </c>
       <c r="B6" s="39" t="n">
+        <v>1.291663063522286</v>
+      </c>
+      <c r="C6" s="37" t="n">
+        <v>-0.1204683168978922</v>
+      </c>
+      <c r="D6" s="26" t="n">
+        <v>8.763384622383818</v>
+      </c>
+      <c r="E6" s="39" t="n">
         <v>1.412131380420178</v>
       </c>
-      <c r="C6" s="37" t="n">
-        <v>-0.1382270055053865</v>
-      </c>
-      <c r="D6" s="26" t="n">
+      <c r="F6" s="37" t="n">
+        <v>-0.1382270055053869</v>
+      </c>
+      <c r="G6" s="26" t="n">
         <v>8.773807101034656</v>
       </c>
-      <c r="E6" s="39" t="n">
+      <c r="H6" s="39" t="n">
+        <v>1.291663063522286</v>
+      </c>
+      <c r="I6" s="39" t="n">
+        <v>1.412131380420178</v>
+      </c>
+      <c r="J6" s="39" t="n">
         <v>1.550358385925565</v>
       </c>
-      <c r="F6" s="37" t="n">
-        <v>-0.5601496694466421</v>
-      </c>
-      <c r="G6" s="26" t="n">
-        <v>8.785765996543011</v>
-      </c>
-      <c r="H6" s="39" t="n">
-        <v>1.412131380420178</v>
-      </c>
-      <c r="I6" s="39" t="n">
-        <v>1.550358385925565</v>
-      </c>
-      <c r="J6" s="39" t="n">
+      <c r="K6" s="39" t="n">
         <v>2.110508055372207</v>
       </c>
-      <c r="K6" s="39" t="n">
+      <c r="L6" s="39" t="n">
         <v>2.120780380148246</v>
-      </c>
-      <c r="L6" s="39" t="n">
-        <v>1.295701676967398</v>
       </c>
     </row>
     <row r="7">
@@ -7847,37 +8133,37 @@
         </is>
       </c>
       <c r="B7" s="39" t="n">
+        <v>6.293375893748721</v>
+      </c>
+      <c r="C7" s="39" t="n">
+        <v>1.327412849053666</v>
+      </c>
+      <c r="D7" s="26" t="n">
+        <v>7.669062142032713</v>
+      </c>
+      <c r="E7" s="39" t="n">
         <v>4.965963044695054</v>
       </c>
-      <c r="C7" s="37" t="n">
+      <c r="F7" s="37" t="n">
         <v>-0.7189319105267877</v>
       </c>
-      <c r="D7" s="26" t="n">
+      <c r="G7" s="26" t="n">
         <v>7.573289366524095</v>
       </c>
-      <c r="E7" s="39" t="n">
+      <c r="H7" s="39" t="n">
+        <v>6.293375893748721</v>
+      </c>
+      <c r="I7" s="39" t="n">
+        <v>4.965963044695054</v>
+      </c>
+      <c r="J7" s="39" t="n">
         <v>5.684894955221842</v>
       </c>
-      <c r="F7" s="39" t="n">
-        <v>2.038889061038818</v>
-      </c>
-      <c r="G7" s="26" t="n">
-        <v>7.625160270532558</v>
-      </c>
-      <c r="H7" s="39" t="n">
-        <v>4.965963044695054</v>
-      </c>
-      <c r="I7" s="39" t="n">
-        <v>5.684894955221842</v>
-      </c>
-      <c r="J7" s="39" t="n">
+      <c r="K7" s="39" t="n">
         <v>3.646005894183024</v>
       </c>
-      <c r="K7" s="39" t="n">
+      <c r="L7" s="39" t="n">
         <v>4.486588098443733</v>
-      </c>
-      <c r="L7" s="39" t="n">
-        <v>4.809685236585581</v>
       </c>
     </row>
     <row r="8">
@@ -7887,37 +8173,37 @@
         </is>
       </c>
       <c r="B8" s="39" t="n">
+        <v>6.030260676236354</v>
+      </c>
+      <c r="C8" s="39" t="n">
+        <v>0.6500163570462014</v>
+      </c>
+      <c r="D8" s="26" t="n">
+        <v>16.12058896045554</v>
+      </c>
+      <c r="E8" s="39" t="n">
         <v>5.380244319190153</v>
       </c>
-      <c r="C8" s="37" t="n">
+      <c r="F8" s="37" t="n">
         <v>-0.6284755076970239</v>
       </c>
-      <c r="D8" s="26" t="n">
+      <c r="G8" s="26" t="n">
         <v>16.02176201763107</v>
       </c>
-      <c r="E8" s="39" t="n">
+      <c r="H8" s="39" t="n">
+        <v>6.030260676236354</v>
+      </c>
+      <c r="I8" s="39" t="n">
+        <v>5.380244319190153</v>
+      </c>
+      <c r="J8" s="39" t="n">
         <v>6.008719826887177</v>
       </c>
-      <c r="F8" s="39" t="n">
-        <v>1.437485581558029</v>
-      </c>
-      <c r="G8" s="26" t="n">
-        <v>16.11731394089035</v>
-      </c>
-      <c r="H8" s="39" t="n">
-        <v>5.380244319190153</v>
-      </c>
-      <c r="I8" s="39" t="n">
-        <v>6.008719826887177</v>
-      </c>
-      <c r="J8" s="39" t="n">
+      <c r="K8" s="39" t="n">
         <v>4.571234245329148</v>
       </c>
-      <c r="K8" s="39" t="n">
+      <c r="L8" s="39" t="n">
         <v>5.608112243287855</v>
-      </c>
-      <c r="L8" s="39" t="n">
-        <v>5.976077549672043</v>
       </c>
     </row>
     <row r="9">
@@ -7927,37 +8213,37 @@
         </is>
       </c>
       <c r="B9" s="39" t="n">
+        <v>18.75485579646165</v>
+      </c>
+      <c r="C9" s="39" t="n">
+        <v>2.233121770783626</v>
+      </c>
+      <c r="D9" s="26" t="n">
+        <v>11.71493023240685</v>
+      </c>
+      <c r="E9" s="39" t="n">
         <v>16.52173402567803</v>
       </c>
-      <c r="C9" s="37" t="n">
-        <v>-0.04531320193483523</v>
-      </c>
-      <c r="D9" s="26" t="n">
+      <c r="F9" s="37" t="n">
+        <v>-0.04531320193483168</v>
+      </c>
+      <c r="G9" s="26" t="n">
         <v>11.49463721306256</v>
       </c>
-      <c r="E9" s="39" t="n">
+      <c r="H9" s="39" t="n">
+        <v>18.75485579646165</v>
+      </c>
+      <c r="I9" s="39" t="n">
+        <v>16.52173402567803</v>
+      </c>
+      <c r="J9" s="39" t="n">
         <v>16.56704722761286</v>
       </c>
-      <c r="F9" s="37" t="n">
-        <v>-0.8612988741681278</v>
-      </c>
-      <c r="G9" s="26" t="n">
-        <v>11.4991072702717</v>
-      </c>
-      <c r="H9" s="39" t="n">
-        <v>16.52173402567803</v>
-      </c>
-      <c r="I9" s="39" t="n">
-        <v>16.56704722761286</v>
-      </c>
-      <c r="J9" s="39" t="n">
+      <c r="K9" s="39" t="n">
         <v>17.42834610178099</v>
       </c>
-      <c r="K9" s="39" t="n">
+      <c r="L9" s="39" t="n">
         <v>17.40960103885576</v>
-      </c>
-      <c r="L9" s="39" t="n">
-        <v>17.56541815026234</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
EGAT retirement pages update 2026-04-30T04:15:09Z
</commit_message>
<xml_diff>
--- a/EGAT Retirement.xlsx
+++ b/EGAT Retirement.xlsx
@@ -683,7 +683,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I22"/>
+  <dimension ref="A1:I23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1604,6 +1604,47 @@
         </is>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>11:15:08</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>EGAT1</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>ตราสารหนี้ (EGAT-1)</t>
+        </is>
+      </c>
+      <c r="F23" t="n">
+        <v>15.75867395748817</v>
+      </c>
+      <c r="G23" t="n">
+        <v>0.6217763017231981</v>
+      </c>
+      <c r="H23" t="n">
+        <v>0.3321003882411189</v>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>https://app.powerbi.com/view?r=eyJrIjoiMzZjYWU3YmQtNWQ1Ny00NjdjLWI1MmEtYjExY2ZiYWIxMzNiIiwidCI6IjVmZWJjNjlmLThlOWMtNDcwOC1iNzBlLWQ4YzYyYmUxODA1YiIsImMiOjEwfQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1615,7 +1656,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I22"/>
+  <dimension ref="A1:I23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -2536,6 +2577,47 @@
         </is>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>11:15:08</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>EGAT2</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>ตราสารทุน (EGAT-2)</t>
+        </is>
+      </c>
+      <c r="F23" t="n">
+        <v>39.98803622524575</v>
+      </c>
+      <c r="G23" t="n">
+        <v>2.271342034860901</v>
+      </c>
+      <c r="H23" t="n">
+        <v>17.82068389056803</v>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>https://app.powerbi.com/view?r=eyJrIjoiMzZjYWU3YmQtNWQ1Ny00NjdjLWI1MmEtYjExY2ZiYWIxMzNiIiwidCI6IjVmZWJjNjlmLThlOWMtNDcwOC1iNzBlLWQ4YzYyYmUxODA1YiIsImMiOjEwfQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2547,7 +2629,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I22"/>
+  <dimension ref="A1:I23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -3468,6 +3550,47 @@
         </is>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>11:15:08</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>EGAT3</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>อสังหาริมทรัพย์และโครงสร้างพื้นฐาน (EGAT-3)</t>
+        </is>
+      </c>
+      <c r="F23" t="n">
+        <v>8.807082536052755</v>
+      </c>
+      <c r="G23" t="n">
+        <v>4.664724138126997</v>
+      </c>
+      <c r="H23" t="n">
+        <v>1.796745807080891</v>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>https://app.powerbi.com/view?r=eyJrIjoiMzZjYWU3YmQtNWQ1Ny00NjdjLWI1MmEtYjExY2ZiYWIxMzNiIiwidCI6IjVmZWJjNjlmLThlOWMtNDcwOC1iNzBlLWQ4YzYyYmUxODA1YiIsImMiOjEwfQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3479,7 +3602,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I22"/>
+  <dimension ref="A1:I23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -4400,6 +4523,47 @@
         </is>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>11:15:08</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>EGAT4</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>ตราสารทุนต่างประเทศ (EGAT-4)</t>
+        </is>
+      </c>
+      <c r="F23" t="n">
+        <v>7.696982082335076</v>
+      </c>
+      <c r="G23" t="n">
+        <v>13.51977269469353</v>
+      </c>
+      <c r="H23" t="n">
+        <v>6.680346902005985</v>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>https://app.powerbi.com/view?r=eyJrIjoiMzZjYWU3YmQtNWQ1Ny00NjdjLWI1MmEtYjExY2ZiYWIxMzNiIiwidCI6IjVmZWJjNjlmLThlOWMtNDcwOC1iNzBlLWQ4YzYyYmUxODA1YiIsImMiOjEwfQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4411,7 +4575,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I22"/>
+  <dimension ref="A1:I23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -5332,6 +5496,47 @@
         </is>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>11:15:08</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>EGAT5</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>ตราสารทุนต่างประเทศแบบอิงดัชนี (EGAT-5)</t>
+        </is>
+      </c>
+      <c r="F23" t="n">
+        <v>16.1630645690105</v>
+      </c>
+      <c r="G23" t="n">
+        <v>11.26639328661947</v>
+      </c>
+      <c r="H23" t="n">
+        <v>6.309636315582523</v>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>https://app.powerbi.com/view?r=eyJrIjoiMzZjYWU3YmQtNWQ1Ny00NjdjLWI1MmEtYjExY2ZiYWIxMzNiIiwidCI6IjVmZWJjNjlmLThlOWMtNDcwOC1iNzBlLWQ4YzYyYmUxODA1YiIsImMiOjEwfQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -5343,7 +5548,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I22"/>
+  <dimension ref="A1:I23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -6259,6 +6464,47 @@
         <v>18.75485579646165</v>
       </c>
       <c r="I22" t="inlineStr">
+        <is>
+          <t>https://app.powerbi.com/view?r=eyJrIjoiMzZjYWU3YmQtNWQ1Ny00NjdjLWI1MmEtYjExY2ZiYWIxMzNiIiwidCI6IjVmZWJjNjlmLThlOWMtNDcwOC1iNzBlLWQ4YzYyYmUxODA1YiIsImMiOjEwfQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>11:15:08</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>EGAT6</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>การลงทุนตามหลักศาสนาอิสลาม (EGAT-6)</t>
+        </is>
+      </c>
+      <c r="F23" t="n">
+        <v>11.73018971108939</v>
+      </c>
+      <c r="G23" t="n">
+        <v>3.411554826313035</v>
+      </c>
+      <c r="H23" t="n">
+        <v>18.90954192386691</v>
+      </c>
+      <c r="I23" t="inlineStr">
         <is>
           <t>https://app.powerbi.com/view?r=eyJrIjoiMzZjYWU3YmQtNWQ1Ny00NjdjLWI1MmEtYjExY2ZiYWIxMzNiIiwidCI6IjVmZWJjNjlmLThlOWMtNDcwOC1iNzBlLWQ4YzYyYmUxODA1YiIsImMiOjEwfQ%3D%3D</t>
         </is>
@@ -7742,7 +7988,7 @@
         <v>17.93913440769168</v>
       </c>
       <c r="H29" s="35" t="n">
-        <v>1.484613531000093</v>
+        <v>1.48461353100009</v>
       </c>
       <c r="I29" s="19" t="n">
         <v>40.02823802524581</v>
@@ -7751,7 +7997,7 @@
         <v>1.291663063522286</v>
       </c>
       <c r="K29" s="36" t="n">
-        <v>-0.1204683168978922</v>
+        <v>-0.1204683168978919</v>
       </c>
       <c r="L29" s="19" t="n">
         <v>8.763384622383818</v>
@@ -7760,7 +8006,7 @@
         <v>6.293375893748721</v>
       </c>
       <c r="N29" s="35" t="n">
-        <v>1.327412849053666</v>
+        <v>1.327412849053667</v>
       </c>
       <c r="O29" s="19" t="n">
         <v>7.669062142032713</v>
@@ -7778,7 +8024,7 @@
         <v>18.75485579646165</v>
       </c>
       <c r="T29" s="35" t="n">
-        <v>2.233121770783626</v>
+        <v>2.233121770783622</v>
       </c>
       <c r="U29" s="19" t="n">
         <v>11.71493023240685</v>
@@ -7790,26 +8036,66 @@
           <t>28/4/69</t>
         </is>
       </c>
-      <c r="B30" s="33" t="n"/>
-      <c r="C30" s="33" t="n"/>
-      <c r="D30" s="33" t="n"/>
-      <c r="E30" s="33" t="n"/>
-      <c r="F30" s="12" t="n"/>
-      <c r="G30" s="33" t="n"/>
-      <c r="H30" s="33" t="n"/>
-      <c r="I30" s="12" t="n"/>
-      <c r="J30" s="33" t="n"/>
-      <c r="K30" s="33" t="n"/>
-      <c r="L30" s="12" t="n"/>
-      <c r="M30" s="33" t="n"/>
-      <c r="N30" s="33" t="n"/>
-      <c r="O30" s="12" t="n"/>
-      <c r="P30" s="33" t="n"/>
-      <c r="Q30" s="33" t="n"/>
-      <c r="R30" s="12" t="n"/>
-      <c r="S30" s="33" t="n"/>
-      <c r="T30" s="33" t="n"/>
-      <c r="U30" s="12" t="n"/>
+      <c r="B30" s="35" t="n">
+        <v>8.641509204557577</v>
+      </c>
+      <c r="C30" s="35" t="n">
+        <v>0.2002780082072739</v>
+      </c>
+      <c r="D30" s="35" t="n">
+        <v>0.3321003882411189</v>
+      </c>
+      <c r="E30" s="36" t="n">
+        <v>-0.005996952200004735</v>
+      </c>
+      <c r="F30" s="19" t="n">
+        <v>15.75867395748817</v>
+      </c>
+      <c r="G30" s="35" t="n">
+        <v>17.82068389056803</v>
+      </c>
+      <c r="H30" s="36" t="n">
+        <v>-0.1184505171236445</v>
+      </c>
+      <c r="I30" s="19" t="n">
+        <v>39.98803622524575</v>
+      </c>
+      <c r="J30" s="35" t="n">
+        <v>1.796745807080891</v>
+      </c>
+      <c r="K30" s="35" t="n">
+        <v>0.5050827435586045</v>
+      </c>
+      <c r="L30" s="19" t="n">
+        <v>8.807082536052755</v>
+      </c>
+      <c r="M30" s="35" t="n">
+        <v>6.680346902005985</v>
+      </c>
+      <c r="N30" s="35" t="n">
+        <v>0.3869710082572633</v>
+      </c>
+      <c r="O30" s="19" t="n">
+        <v>7.696982082335076</v>
+      </c>
+      <c r="P30" s="35" t="n">
+        <v>6.309636315582523</v>
+      </c>
+      <c r="Q30" s="35" t="n">
+        <v>0.2793756393461688</v>
+      </c>
+      <c r="R30" s="19" t="n">
+        <v>16.1630645690105</v>
+      </c>
+      <c r="S30" s="35" t="n">
+        <v>18.90954192386691</v>
+      </c>
+      <c r="T30" s="35" t="n">
+        <v>0.1546861274052596</v>
+      </c>
+      <c r="U30" s="19" t="n">
+        <v>11.73018971108939</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="10" t="inlineStr">
@@ -7912,14 +8198,14 @@
       </c>
       <c r="B1" s="4" t="inlineStr">
         <is>
-          <t>27 เม.ย. 69 (จันทร์)</t>
+          <t>28 เม.ย. 69 (อังคาร)</t>
         </is>
       </c>
       <c r="C1" s="20" t="n"/>
       <c r="D1" s="20" t="n"/>
       <c r="E1" s="21" t="inlineStr">
         <is>
-          <t>24 เม.ย. 69 (ศุกร์)</t>
+          <t>27 เม.ย. 69 (จันทร์)</t>
         </is>
       </c>
       <c r="F1" s="20" t="n"/>
@@ -7982,27 +8268,27 @@
       <c r="G3" s="20" t="n"/>
       <c r="H3" s="22" t="inlineStr">
         <is>
+          <t>28/4/69</t>
+        </is>
+      </c>
+      <c r="I3" s="22" t="inlineStr">
+        <is>
           <t>27/4/69</t>
         </is>
       </c>
-      <c r="I3" s="22" t="inlineStr">
+      <c r="J3" s="22" t="inlineStr">
         <is>
           <t>24/4/69</t>
         </is>
       </c>
-      <c r="J3" s="22" t="inlineStr">
+      <c r="K3" s="22" t="inlineStr">
         <is>
           <t>23/4/69</t>
         </is>
       </c>
-      <c r="K3" s="22" t="inlineStr">
+      <c r="L3" s="22" t="inlineStr">
         <is>
           <t>22/4/69</t>
-        </is>
-      </c>
-      <c r="L3" s="22" t="inlineStr">
-        <is>
-          <t>21/4/69</t>
         </is>
       </c>
     </row>
@@ -8013,37 +8299,37 @@
         </is>
       </c>
       <c r="B4" s="39" t="n">
+        <v>0.3321003882411189</v>
+      </c>
+      <c r="C4" s="37" t="n">
+        <v>-0.005996952200004735</v>
+      </c>
+      <c r="D4" s="26" t="n">
+        <v>15.75867395748817</v>
+      </c>
+      <c r="E4" s="39" t="n">
         <v>0.3380973404411236</v>
       </c>
-      <c r="C4" s="39" t="n">
+      <c r="F4" s="39" t="n">
         <v>0.01652826571014732</v>
       </c>
-      <c r="D4" s="26" t="n">
+      <c r="G4" s="26" t="n">
         <v>15.75961586953918</v>
       </c>
-      <c r="E4" s="39" t="n">
+      <c r="H4" s="39" t="n">
+        <v>0.3321003882411189</v>
+      </c>
+      <c r="I4" s="39" t="n">
+        <v>0.3380973404411236</v>
+      </c>
+      <c r="J4" s="39" t="n">
         <v>0.3215690747309763</v>
       </c>
-      <c r="F4" s="39" t="n">
-        <v>0.03316407771021268</v>
-      </c>
-      <c r="G4" s="26" t="n">
-        <v>15.75701985540809</v>
-      </c>
-      <c r="H4" s="39" t="n">
-        <v>0.3380973404411236</v>
-      </c>
-      <c r="I4" s="39" t="n">
-        <v>0.3215690747309763</v>
-      </c>
-      <c r="J4" s="39" t="n">
+      <c r="K4" s="39" t="n">
         <v>0.2884049970207636</v>
       </c>
-      <c r="K4" s="39" t="n">
+      <c r="L4" s="39" t="n">
         <v>0.3321212202299417</v>
-      </c>
-      <c r="L4" s="39" t="n">
-        <v>0.3618021344736988</v>
       </c>
     </row>
     <row r="5">
@@ -8053,37 +8339,37 @@
         </is>
       </c>
       <c r="B5" s="39" t="n">
+        <v>17.82068389056803</v>
+      </c>
+      <c r="C5" s="37" t="n">
+        <v>-0.1184505171236445</v>
+      </c>
+      <c r="D5" s="26" t="n">
+        <v>39.98803622524575</v>
+      </c>
+      <c r="E5" s="39" t="n">
         <v>17.93913440769168</v>
       </c>
-      <c r="C5" s="39" t="n">
-        <v>1.484613531000093</v>
-      </c>
-      <c r="D5" s="26" t="n">
+      <c r="F5" s="39" t="n">
+        <v>1.48461353100009</v>
+      </c>
+      <c r="G5" s="26" t="n">
         <v>40.02823802524581</v>
       </c>
-      <c r="E5" s="39" t="n">
+      <c r="H5" s="39" t="n">
+        <v>17.82068389056803</v>
+      </c>
+      <c r="I5" s="39" t="n">
+        <v>17.93913440769168</v>
+      </c>
+      <c r="J5" s="39" t="n">
         <v>16.45452087669159</v>
       </c>
-      <c r="F5" s="37" t="n">
-        <v>-0.4416520757771316</v>
-      </c>
-      <c r="G5" s="26" t="n">
-        <v>39.52436402199133</v>
-      </c>
-      <c r="H5" s="39" t="n">
-        <v>17.93913440769168</v>
-      </c>
-      <c r="I5" s="39" t="n">
-        <v>16.45452087669159</v>
-      </c>
-      <c r="J5" s="39" t="n">
+      <c r="K5" s="39" t="n">
         <v>16.89617295246872</v>
       </c>
-      <c r="K5" s="39" t="n">
+      <c r="L5" s="39" t="n">
         <v>18.24301567279665</v>
-      </c>
-      <c r="L5" s="39" t="n">
-        <v>18.43423938672446</v>
       </c>
     </row>
     <row r="6">
@@ -8093,37 +8379,37 @@
         </is>
       </c>
       <c r="B6" s="39" t="n">
+        <v>1.796745807080891</v>
+      </c>
+      <c r="C6" s="39" t="n">
+        <v>0.5050827435586045</v>
+      </c>
+      <c r="D6" s="26" t="n">
+        <v>8.807082536052755</v>
+      </c>
+      <c r="E6" s="39" t="n">
         <v>1.291663063522286</v>
       </c>
-      <c r="C6" s="37" t="n">
-        <v>-0.1204683168978922</v>
-      </c>
-      <c r="D6" s="26" t="n">
+      <c r="F6" s="37" t="n">
+        <v>-0.1204683168978919</v>
+      </c>
+      <c r="G6" s="26" t="n">
         <v>8.763384622383818</v>
       </c>
-      <c r="E6" s="39" t="n">
+      <c r="H6" s="39" t="n">
+        <v>1.796745807080891</v>
+      </c>
+      <c r="I6" s="39" t="n">
+        <v>1.291663063522286</v>
+      </c>
+      <c r="J6" s="39" t="n">
         <v>1.412131380420178</v>
       </c>
-      <c r="F6" s="37" t="n">
-        <v>-0.1382270055053869</v>
-      </c>
-      <c r="G6" s="26" t="n">
-        <v>8.773807101034656</v>
-      </c>
-      <c r="H6" s="39" t="n">
-        <v>1.291663063522286</v>
-      </c>
-      <c r="I6" s="39" t="n">
-        <v>1.412131380420178</v>
-      </c>
-      <c r="J6" s="39" t="n">
+      <c r="K6" s="39" t="n">
         <v>1.550358385925565</v>
       </c>
-      <c r="K6" s="39" t="n">
+      <c r="L6" s="39" t="n">
         <v>2.110508055372207</v>
-      </c>
-      <c r="L6" s="39" t="n">
-        <v>2.120780380148246</v>
       </c>
     </row>
     <row r="7">
@@ -8133,37 +8419,37 @@
         </is>
       </c>
       <c r="B7" s="39" t="n">
+        <v>6.680346902005985</v>
+      </c>
+      <c r="C7" s="39" t="n">
+        <v>0.3869710082572633</v>
+      </c>
+      <c r="D7" s="26" t="n">
+        <v>7.696982082335076</v>
+      </c>
+      <c r="E7" s="39" t="n">
         <v>6.293375893748721</v>
       </c>
-      <c r="C7" s="39" t="n">
-        <v>1.327412849053666</v>
-      </c>
-      <c r="D7" s="26" t="n">
+      <c r="F7" s="39" t="n">
+        <v>1.327412849053667</v>
+      </c>
+      <c r="G7" s="26" t="n">
         <v>7.669062142032713</v>
       </c>
-      <c r="E7" s="39" t="n">
+      <c r="H7" s="39" t="n">
+        <v>6.680346902005985</v>
+      </c>
+      <c r="I7" s="39" t="n">
+        <v>6.293375893748721</v>
+      </c>
+      <c r="J7" s="39" t="n">
         <v>4.965963044695054</v>
       </c>
-      <c r="F7" s="37" t="n">
-        <v>-0.7189319105267877</v>
-      </c>
-      <c r="G7" s="26" t="n">
-        <v>7.573289366524095</v>
-      </c>
-      <c r="H7" s="39" t="n">
-        <v>6.293375893748721</v>
-      </c>
-      <c r="I7" s="39" t="n">
-        <v>4.965963044695054</v>
-      </c>
-      <c r="J7" s="39" t="n">
+      <c r="K7" s="39" t="n">
         <v>5.684894955221842</v>
       </c>
-      <c r="K7" s="39" t="n">
+      <c r="L7" s="39" t="n">
         <v>3.646005894183024</v>
-      </c>
-      <c r="L7" s="39" t="n">
-        <v>4.486588098443733</v>
       </c>
     </row>
     <row r="8">
@@ -8173,37 +8459,37 @@
         </is>
       </c>
       <c r="B8" s="39" t="n">
+        <v>6.309636315582523</v>
+      </c>
+      <c r="C8" s="39" t="n">
+        <v>0.2793756393461688</v>
+      </c>
+      <c r="D8" s="26" t="n">
+        <v>16.1630645690105</v>
+      </c>
+      <c r="E8" s="39" t="n">
         <v>6.030260676236354</v>
       </c>
-      <c r="C8" s="39" t="n">
+      <c r="F8" s="39" t="n">
         <v>0.6500163570462014</v>
       </c>
-      <c r="D8" s="26" t="n">
+      <c r="G8" s="26" t="n">
         <v>16.12058896045554</v>
       </c>
-      <c r="E8" s="39" t="n">
+      <c r="H8" s="39" t="n">
+        <v>6.309636315582523</v>
+      </c>
+      <c r="I8" s="39" t="n">
+        <v>6.030260676236354</v>
+      </c>
+      <c r="J8" s="39" t="n">
         <v>5.380244319190153</v>
       </c>
-      <c r="F8" s="37" t="n">
-        <v>-0.6284755076970239</v>
-      </c>
-      <c r="G8" s="26" t="n">
-        <v>16.02176201763107</v>
-      </c>
-      <c r="H8" s="39" t="n">
-        <v>6.030260676236354</v>
-      </c>
-      <c r="I8" s="39" t="n">
-        <v>5.380244319190153</v>
-      </c>
-      <c r="J8" s="39" t="n">
+      <c r="K8" s="39" t="n">
         <v>6.008719826887177</v>
       </c>
-      <c r="K8" s="39" t="n">
+      <c r="L8" s="39" t="n">
         <v>4.571234245329148</v>
-      </c>
-      <c r="L8" s="39" t="n">
-        <v>5.608112243287855</v>
       </c>
     </row>
     <row r="9">
@@ -8213,37 +8499,37 @@
         </is>
       </c>
       <c r="B9" s="39" t="n">
+        <v>18.90954192386691</v>
+      </c>
+      <c r="C9" s="39" t="n">
+        <v>0.1546861274052596</v>
+      </c>
+      <c r="D9" s="26" t="n">
+        <v>11.73018971108939</v>
+      </c>
+      <c r="E9" s="39" t="n">
         <v>18.75485579646165</v>
       </c>
-      <c r="C9" s="39" t="n">
-        <v>2.233121770783626</v>
-      </c>
-      <c r="D9" s="26" t="n">
+      <c r="F9" s="39" t="n">
+        <v>2.233121770783622</v>
+      </c>
+      <c r="G9" s="26" t="n">
         <v>11.71493023240685</v>
       </c>
-      <c r="E9" s="39" t="n">
+      <c r="H9" s="39" t="n">
+        <v>18.90954192386691</v>
+      </c>
+      <c r="I9" s="39" t="n">
+        <v>18.75485579646165</v>
+      </c>
+      <c r="J9" s="39" t="n">
         <v>16.52173402567803</v>
       </c>
-      <c r="F9" s="37" t="n">
-        <v>-0.04531320193483168</v>
-      </c>
-      <c r="G9" s="26" t="n">
-        <v>11.49463721306256</v>
-      </c>
-      <c r="H9" s="39" t="n">
-        <v>18.75485579646165</v>
-      </c>
-      <c r="I9" s="39" t="n">
-        <v>16.52173402567803</v>
-      </c>
-      <c r="J9" s="39" t="n">
+      <c r="K9" s="39" t="n">
         <v>16.56704722761286</v>
       </c>
-      <c r="K9" s="39" t="n">
+      <c r="L9" s="39" t="n">
         <v>17.42834610178099</v>
-      </c>
-      <c r="L9" s="39" t="n">
-        <v>17.40960103885576</v>
       </c>
     </row>
   </sheetData>

</xml_diff>